<commit_message>
Phone: progress 2, log 2 in Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -3432,16 +3432,16 @@
         <v/>
       </c>
       <c r="S34" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-05</v>
       </c>
       <c r="T34" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U34" t="str">
         <v>2.5</v>
       </c>
       <c r="V34" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W34" t="str">
         <v>1</v>
@@ -3462,10 +3462,10 @@
         <v/>
       </c>
       <c r="AC34" t="str">
-        <v>1.18</v>
+        <v>0.99</v>
       </c>
       <c r="AD34" t="str">
-        <v>7.61</v>
+        <v>7.98</v>
       </c>
       <c r="AE34" t="str">
         <v>2026-09-04</v>
@@ -3842,10 +3842,10 @@
         <v/>
       </c>
       <c r="AC38" t="str">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="AD38" t="str">
-        <v>9.21</v>
+        <v>9.44</v>
       </c>
       <c r="AE38" t="str">
         <v>2026-09-04</v>
@@ -18457,7 +18457,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H212"/>
+  <dimension ref="A1:H214"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -23981,9 +23981,61 @@
         <v>0</v>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>1eb35f1d-82a9-4b9b-babe-edbdf2672381</v>
+      </c>
+      <c r="B213" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C213" t="str">
+        <v>2026-09-04T06:01:47.134Z</v>
+      </c>
+      <c r="D213" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E213" t="str">
+        <v>0</v>
+      </c>
+      <c r="F213" t="str">
+        <v>0.99</v>
+      </c>
+      <c r="G213" t="str">
+        <v>7.98</v>
+      </c>
+      <c r="H213" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>ebc6c3f3-1578-49db-a2ec-0c9cbb8b9efc</v>
+      </c>
+      <c r="B214" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C214" t="str">
+        <v>2026-09-04T06:02:11.503Z</v>
+      </c>
+      <c r="D214" t="str">
+        <v>again</v>
+      </c>
+      <c r="E214" t="str">
+        <v>0</v>
+      </c>
+      <c r="F214" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="G214" t="str">
+        <v>9.44</v>
+      </c>
+      <c r="H214" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H212"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H214"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add word "hjerner" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,42 +194,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH175"/>
+  <dimension ref="A1:AH176"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -17469,9 +17469,113 @@
         <v/>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>ea0c5d72-3c7a-408e-879d-bad2f1ef70ee</v>
+      </c>
+      <c r="B176" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C176" t="str">
+        <v>hjerner</v>
+      </c>
+      <c r="D176" t="str">
+        <v>hjerne</v>
+      </c>
+      <c r="E176" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F176" t="str">
+        <v>en</v>
+      </c>
+      <c r="G176" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H176" t="str">
+        <v>[ˈjæɐ̯nə]</v>
+      </c>
+      <c r="I176" t="str">
+        <v>https://static.ordnet.dk/mp3/11020/11020957_1.mp3</v>
+      </c>
+      <c r="J176" t="str">
+        <v>organ i kraniets øverste hulrum der udgør den højest udviklede del af centralnervesystemet, bl.a. med centre for sansning og højere åndsevner som tænkning, forestillingsevne, hukommelse og sprog</v>
+      </c>
+      <c r="K176" t="str">
+        <v>Brains</v>
+      </c>
+      <c r="L176" t="str">
+        <v>Mike Doustdar vil have sine ansatte til at være dedikerede - nærmest besatte - i jagten på fremtidens guld, og med tidens største mestre inden for computerhjerner vælger topchefen AI-værktøjskassen som sit våben over for Novos skarpladte konkurrenter.</v>
+      </c>
+      <c r="M176" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N176" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O176" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=hjerner</v>
+      </c>
+      <c r="P176" t="str">
+        <v/>
+      </c>
+      <c r="Q176" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R176" t="str">
+        <v/>
+      </c>
+      <c r="S176" t="str">
+        <v/>
+      </c>
+      <c r="T176" t="str">
+        <v/>
+      </c>
+      <c r="U176" t="str">
+        <v/>
+      </c>
+      <c r="V176" t="str">
+        <v/>
+      </c>
+      <c r="W176" t="str">
+        <v/>
+      </c>
+      <c r="X176" t="str">
+        <v/>
+      </c>
+      <c r="Y176" t="str">
+        <v/>
+      </c>
+      <c r="Z176" t="str">
+        <v/>
+      </c>
+      <c r="AA176" t="str">
+        <v/>
+      </c>
+      <c r="AB176" t="str">
+        <v/>
+      </c>
+      <c r="AC176" t="str">
+        <v/>
+      </c>
+      <c r="AD176" t="str">
+        <v/>
+      </c>
+      <c r="AE176" t="str">
+        <v/>
+      </c>
+      <c r="AF176" t="str">
+        <v/>
+      </c>
+      <c r="AG176" t="str">
+        <v/>
+      </c>
+      <c r="AH176" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH175"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH176"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "våben" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH176"/>
+  <dimension ref="A1:AH177"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -17573,9 +17573,113 @@
         <v/>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>dc657128-7ffc-48eb-945f-a3c131cc6572</v>
+      </c>
+      <c r="B177" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C177" t="str">
+        <v>våben</v>
+      </c>
+      <c r="D177" t="str">
+        <v>våben</v>
+      </c>
+      <c r="E177" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F177" t="str">
+        <v>et</v>
+      </c>
+      <c r="G177" t="str">
+        <v>betydning 1: våbnet eller -et, -, våbnene Se bøjning i skema</v>
+      </c>
+      <c r="H177" t="str">
+        <v>[ˈvɔˀbən]</v>
+      </c>
+      <c r="I177" t="str">
+        <v>https://static.ordnet.dk/mp3/12007/12007603_1.mp3</v>
+      </c>
+      <c r="J177" t="str">
+        <v>redskab som bruges til angreb eller forsvar fx kniv, pistol eller kanon</v>
+      </c>
+      <c r="K177" t="str">
+        <v>arms</v>
+      </c>
+      <c r="L177" t="str">
+        <v>Mike Doustdar vil have sine ansatte til at være dedikerede - nærmest besatte - i jagten på fremtidens guld, og med tidens største mestre inden for computerhjerner vælger topchefen AI-værktøjskassen som sit våben over for Novos skarpladte konkurrenter.</v>
+      </c>
+      <c r="M177" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N177" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O177" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=v%C3%A5ben</v>
+      </c>
+      <c r="P177" t="str">
+        <v/>
+      </c>
+      <c r="Q177" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R177" t="str">
+        <v/>
+      </c>
+      <c r="S177" t="str">
+        <v/>
+      </c>
+      <c r="T177" t="str">
+        <v/>
+      </c>
+      <c r="U177" t="str">
+        <v/>
+      </c>
+      <c r="V177" t="str">
+        <v/>
+      </c>
+      <c r="W177" t="str">
+        <v/>
+      </c>
+      <c r="X177" t="str">
+        <v/>
+      </c>
+      <c r="Y177" t="str">
+        <v/>
+      </c>
+      <c r="Z177" t="str">
+        <v/>
+      </c>
+      <c r="AA177" t="str">
+        <v/>
+      </c>
+      <c r="AB177" t="str">
+        <v/>
+      </c>
+      <c r="AC177" t="str">
+        <v/>
+      </c>
+      <c r="AD177" t="str">
+        <v/>
+      </c>
+      <c r="AE177" t="str">
+        <v/>
+      </c>
+      <c r="AF177" t="str">
+        <v/>
+      </c>
+      <c r="AG177" t="str">
+        <v/>
+      </c>
+      <c r="AH177" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH176"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH177"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "gentagelsen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH177"/>
+  <dimension ref="A1:AH178"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -17677,9 +17677,113 @@
         <v/>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>c51e08b7-fee2-4713-9bd1-2becd62bbaad</v>
+      </c>
+      <c r="B178" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C178" t="str">
+        <v>gentagelsen</v>
+      </c>
+      <c r="D178" t="str">
+        <v>gentagelse</v>
+      </c>
+      <c r="E178" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F178" t="str">
+        <v>en</v>
+      </c>
+      <c r="G178" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H178" t="str">
+        <v>[ˈgεnˌtæˀjəlsə]</v>
+      </c>
+      <c r="I178" t="str">
+        <v>https://static.ordnet.dk/mp3/11017/11017802_1.mp3</v>
+      </c>
+      <c r="J178" t="str">
+        <v>det at gentage noget</v>
+      </c>
+      <c r="K178" t="str">
+        <v>The repetition</v>
+      </c>
+      <c r="L178" t="str">
+        <v>Med nu Anthropic, Amazon og OpenAI på holdet samt gentagelsen af at være nummer ét på AI i medicinalindustrien ligner det en taktik set i fodboldklubber som Real Madrid og Paris Saint-Germain.</v>
+      </c>
+      <c r="M178" t="str">
+        <v>Turbulente tider i Novo Nordisk</v>
+      </c>
+      <c r="N178" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk</v>
+      </c>
+      <c r="O178" t="str">
+        <v>https://nyheder.tv2.dk/live/business/2025-08-20-turbulente-tider-i-novo-nordisk#:~:text=gentagelsen</v>
+      </c>
+      <c r="P178" t="str">
+        <v/>
+      </c>
+      <c r="Q178" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R178" t="str">
+        <v/>
+      </c>
+      <c r="S178" t="str">
+        <v/>
+      </c>
+      <c r="T178" t="str">
+        <v/>
+      </c>
+      <c r="U178" t="str">
+        <v/>
+      </c>
+      <c r="V178" t="str">
+        <v/>
+      </c>
+      <c r="W178" t="str">
+        <v/>
+      </c>
+      <c r="X178" t="str">
+        <v/>
+      </c>
+      <c r="Y178" t="str">
+        <v/>
+      </c>
+      <c r="Z178" t="str">
+        <v/>
+      </c>
+      <c r="AA178" t="str">
+        <v/>
+      </c>
+      <c r="AB178" t="str">
+        <v/>
+      </c>
+      <c r="AC178" t="str">
+        <v/>
+      </c>
+      <c r="AD178" t="str">
+        <v/>
+      </c>
+      <c r="AE178" t="str">
+        <v/>
+      </c>
+      <c r="AF178" t="str">
+        <v/>
+      </c>
+      <c r="AG178" t="str">
+        <v/>
+      </c>
+      <c r="AH178" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH177"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH178"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Samle" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH178"/>
+  <dimension ref="A1:AH179"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -17781,9 +17781,113 @@
         <v/>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>a99a873f-4642-46ce-8573-5496517f5d35</v>
+      </c>
+      <c r="B179" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="C179" t="str">
+        <v>Samle</v>
+      </c>
+      <c r="D179" t="str">
+        <v>samle</v>
+      </c>
+      <c r="E179" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F179" t="str">
+        <v/>
+      </c>
+      <c r="G179" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H179" t="str">
+        <v>[ˈsɑmlə]</v>
+      </c>
+      <c r="I179" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044641_1.mp3</v>
+      </c>
+      <c r="J179" t="str">
+        <v>bringe genstande sammen der forekommer spredt, ofte for at udnytte dem</v>
+      </c>
+      <c r="K179" t="str">
+        <v>Gather</v>
+      </c>
+      <c r="L179" t="str">
+        <v>Samle info</v>
+      </c>
+      <c r="M179" t="str">
+        <v>Sækkestol SNEKKERSTEN 60x90x60 grå | JYSK</v>
+      </c>
+      <c r="N179" t="str">
+        <v>https://jysk.dk/indretning/bornemobler/saekkestol-snekkersten-60x90x60-graa</v>
+      </c>
+      <c r="O179" t="str">
+        <v>https://jysk.dk/indretning/bornemobler/saekkestol-snekkersten-60x90x60-graa#:~:text=Samle</v>
+      </c>
+      <c r="P179" t="str">
+        <v/>
+      </c>
+      <c r="Q179" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R179" t="str">
+        <v/>
+      </c>
+      <c r="S179" t="str">
+        <v/>
+      </c>
+      <c r="T179" t="str">
+        <v/>
+      </c>
+      <c r="U179" t="str">
+        <v/>
+      </c>
+      <c r="V179" t="str">
+        <v/>
+      </c>
+      <c r="W179" t="str">
+        <v/>
+      </c>
+      <c r="X179" t="str">
+        <v/>
+      </c>
+      <c r="Y179" t="str">
+        <v/>
+      </c>
+      <c r="Z179" t="str">
+        <v/>
+      </c>
+      <c r="AA179" t="str">
+        <v/>
+      </c>
+      <c r="AB179" t="str">
+        <v/>
+      </c>
+      <c r="AC179" t="str">
+        <v/>
+      </c>
+      <c r="AD179" t="str">
+        <v/>
+      </c>
+      <c r="AE179" t="str">
+        <v/>
+      </c>
+      <c r="AF179" t="str">
+        <v/>
+      </c>
+      <c r="AG179" t="str">
+        <v/>
+      </c>
+      <c r="AH179" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH178"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH179"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "knækker" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH179"/>
+  <dimension ref="A1:AH180"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -17885,9 +17885,113 @@
         <v/>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>73bbaa2d-1112-42b0-a3b5-564bcc84d9ca</v>
+      </c>
+      <c r="B180" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C180" t="str">
+        <v>knækker</v>
+      </c>
+      <c r="D180" t="str">
+        <v>knække</v>
+      </c>
+      <c r="E180" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F180" t="str">
+        <v/>
+      </c>
+      <c r="G180" t="str">
+        <v>-r, -de (eller uofficiel form: knak), -t Se bøjning i skema</v>
+      </c>
+      <c r="H180" t="str">
+        <v>[ˈknεgə]</v>
+      </c>
+      <c r="I180" t="str">
+        <v>https://static.ordnet.dk/mp3/11026/11026736_1.mp3</v>
+      </c>
+      <c r="J180" t="str">
+        <v>pludselig briste eller gå i to eller flere stykker som følge af et stærkt tryk, ofte ledsaget af en kort, skarp lyd</v>
+      </c>
+      <c r="K180" t="str">
+        <v>breaks</v>
+      </c>
+      <c r="L180" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden</v>
+      </c>
+      <c r="M180" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N180" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O180" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=kn%C3%A6kker</v>
+      </c>
+      <c r="P180" t="str">
+        <v/>
+      </c>
+      <c r="Q180" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R180" t="str">
+        <v/>
+      </c>
+      <c r="S180" t="str">
+        <v/>
+      </c>
+      <c r="T180" t="str">
+        <v/>
+      </c>
+      <c r="U180" t="str">
+        <v/>
+      </c>
+      <c r="V180" t="str">
+        <v/>
+      </c>
+      <c r="W180" t="str">
+        <v/>
+      </c>
+      <c r="X180" t="str">
+        <v/>
+      </c>
+      <c r="Y180" t="str">
+        <v/>
+      </c>
+      <c r="Z180" t="str">
+        <v/>
+      </c>
+      <c r="AA180" t="str">
+        <v/>
+      </c>
+      <c r="AB180" t="str">
+        <v/>
+      </c>
+      <c r="AC180" t="str">
+        <v/>
+      </c>
+      <c r="AD180" t="str">
+        <v/>
+      </c>
+      <c r="AE180" t="str">
+        <v/>
+      </c>
+      <c r="AF180" t="str">
+        <v/>
+      </c>
+      <c r="AG180" t="str">
+        <v/>
+      </c>
+      <c r="AH180" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH179"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH180"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "rækkevidde" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH180"/>
+  <dimension ref="A1:AH181"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -17989,9 +17989,113 @@
         <v/>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>9077c686-192a-44ad-a7cb-49c032791680</v>
+      </c>
+      <c r="B181" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C181" t="str">
+        <v>rækkevidde</v>
+      </c>
+      <c r="D181" t="str">
+        <v>rækkevidde</v>
+      </c>
+      <c r="E181" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F181" t="str">
+        <v>en</v>
+      </c>
+      <c r="G181" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H181" t="str">
+        <v/>
+      </c>
+      <c r="I181" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044072_1.mp3</v>
+      </c>
+      <c r="J181" t="str">
+        <v>afstand eller område som noget eller nogen er i stand til at tilbagelægge, dække, nå hen over el.lign.</v>
+      </c>
+      <c r="K181" t="str">
+        <v>range</v>
+      </c>
+      <c r="L181" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden</v>
+      </c>
+      <c r="M181" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N181" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O181" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=r%C3%A6kkevidde</v>
+      </c>
+      <c r="P181" t="str">
+        <v/>
+      </c>
+      <c r="Q181" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R181" t="str">
+        <v/>
+      </c>
+      <c r="S181" t="str">
+        <v/>
+      </c>
+      <c r="T181" t="str">
+        <v/>
+      </c>
+      <c r="U181" t="str">
+        <v/>
+      </c>
+      <c r="V181" t="str">
+        <v/>
+      </c>
+      <c r="W181" t="str">
+        <v/>
+      </c>
+      <c r="X181" t="str">
+        <v/>
+      </c>
+      <c r="Y181" t="str">
+        <v/>
+      </c>
+      <c r="Z181" t="str">
+        <v/>
+      </c>
+      <c r="AA181" t="str">
+        <v/>
+      </c>
+      <c r="AB181" t="str">
+        <v/>
+      </c>
+      <c r="AC181" t="str">
+        <v/>
+      </c>
+      <c r="AD181" t="str">
+        <v/>
+      </c>
+      <c r="AE181" t="str">
+        <v/>
+      </c>
+      <c r="AF181" t="str">
+        <v/>
+      </c>
+      <c r="AG181" t="str">
+        <v/>
+      </c>
+      <c r="AH181" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH180"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH181"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "rammer" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH181"/>
+  <dimension ref="A1:AH182"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18093,9 +18093,113 @@
         <v/>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>05f2d3bb-4950-475f-a193-d442a4a05cb0</v>
+      </c>
+      <c r="B182" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C182" t="str">
+        <v>rammer</v>
+      </c>
+      <c r="D182" t="str">
+        <v>ramme</v>
+      </c>
+      <c r="E182" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F182" t="str">
+        <v>en</v>
+      </c>
+      <c r="G182" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H182" t="str">
+        <v>[ˈʁɑmə]</v>
+      </c>
+      <c r="I182" t="str">
+        <v>https://static.ordnet.dk/mp3/11042/11042091_1.mp3</v>
+      </c>
+      <c r="J182" t="str">
+        <v>(firkantet) indretning, ofte af trælister, til indfatning eller omkransning af en genstand, fx et maleri</v>
+      </c>
+      <c r="K182" t="str">
+        <v>hits</v>
+      </c>
+      <c r="L182" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden</v>
+      </c>
+      <c r="M182" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N182" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O182" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=rammer</v>
+      </c>
+      <c r="P182" t="str">
+        <v/>
+      </c>
+      <c r="Q182" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R182" t="str">
+        <v/>
+      </c>
+      <c r="S182" t="str">
+        <v/>
+      </c>
+      <c r="T182" t="str">
+        <v/>
+      </c>
+      <c r="U182" t="str">
+        <v/>
+      </c>
+      <c r="V182" t="str">
+        <v/>
+      </c>
+      <c r="W182" t="str">
+        <v/>
+      </c>
+      <c r="X182" t="str">
+        <v/>
+      </c>
+      <c r="Y182" t="str">
+        <v/>
+      </c>
+      <c r="Z182" t="str">
+        <v/>
+      </c>
+      <c r="AA182" t="str">
+        <v/>
+      </c>
+      <c r="AB182" t="str">
+        <v/>
+      </c>
+      <c r="AC182" t="str">
+        <v/>
+      </c>
+      <c r="AD182" t="str">
+        <v/>
+      </c>
+      <c r="AE182" t="str">
+        <v/>
+      </c>
+      <c r="AF182" t="str">
+        <v/>
+      </c>
+      <c r="AG182" t="str">
+        <v/>
+      </c>
+      <c r="AH182" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH181"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH182"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "knækker kode" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -196,40 +196,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH182"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18206,36 +18206,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB13"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19129,9 +19129,95 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>e9113aac-2b28-4234-aa73-6596306cdbea</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C13" t="str">
+        <v>knækker kode</v>
+      </c>
+      <c r="D13" t="str">
+        <v>knækker=breaks · kode=code</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Cracks code</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="H13" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="I13" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=kn%C3%A6kker%20kode</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
+        <v/>
+      </c>
+      <c r="Z13" t="str">
+        <v/>
+      </c>
+      <c r="AA13" t="str">
+        <v/>
+      </c>
+      <c r="AB13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "lastbil" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,42 +194,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH182"/>
+  <dimension ref="A1:AH183"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18197,9 +18197,113 @@
         <v/>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>5270a3bf-dd03-4fc5-bf0f-2b444872a0cd</v>
+      </c>
+      <c r="B183" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C183" t="str">
+        <v>lastbil</v>
+      </c>
+      <c r="D183" t="str">
+        <v>lastbil</v>
+      </c>
+      <c r="E183" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F183" t="str">
+        <v>en</v>
+      </c>
+      <c r="G183" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H183" t="str">
+        <v/>
+      </c>
+      <c r="I183" t="str">
+        <v>https://static.ordnet.dk/mp3/11029/11029849_1.mp3</v>
+      </c>
+      <c r="J183" t="str">
+        <v>stor bil som er beregnet til transport af gods, og som forrest har et førerhus og bagest et lad, et lastrum eller en sættevogn</v>
+      </c>
+      <c r="K183" t="str">
+        <v>lorry</v>
+      </c>
+      <c r="L183" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden</v>
+      </c>
+      <c r="M183" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N183" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O183" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=lastbil</v>
+      </c>
+      <c r="P183" t="str">
+        <v/>
+      </c>
+      <c r="Q183" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R183" t="str">
+        <v/>
+      </c>
+      <c r="S183" t="str">
+        <v/>
+      </c>
+      <c r="T183" t="str">
+        <v/>
+      </c>
+      <c r="U183" t="str">
+        <v/>
+      </c>
+      <c r="V183" t="str">
+        <v/>
+      </c>
+      <c r="W183" t="str">
+        <v/>
+      </c>
+      <c r="X183" t="str">
+        <v/>
+      </c>
+      <c r="Y183" t="str">
+        <v/>
+      </c>
+      <c r="Z183" t="str">
+        <v/>
+      </c>
+      <c r="AA183" t="str">
+        <v/>
+      </c>
+      <c r="AB183" t="str">
+        <v/>
+      </c>
+      <c r="AC183" t="str">
+        <v/>
+      </c>
+      <c r="AD183" t="str">
+        <v/>
+      </c>
+      <c r="AE183" t="str">
+        <v/>
+      </c>
+      <c r="AF183" t="str">
+        <v/>
+      </c>
+      <c r="AG183" t="str">
+        <v/>
+      </c>
+      <c r="AH183" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH182"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH183"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -18208,34 +18312,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB13"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "hænger" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH183"/>
+  <dimension ref="A1:AH184"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18301,9 +18301,113 @@
         <v/>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>30de1ca9-0b4c-43ce-9a12-d2691320d05e</v>
+      </c>
+      <c r="B184" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C184" t="str">
+        <v>hænger</v>
+      </c>
+      <c r="D184" t="str">
+        <v>hænger</v>
+      </c>
+      <c r="E184" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F184" t="str">
+        <v>en</v>
+      </c>
+      <c r="G184" t="str">
+        <v>-en, -e, -ne</v>
+      </c>
+      <c r="H184" t="str">
+        <v>[ˈhεŋʌ]</v>
+      </c>
+      <c r="I184" t="str">
+        <v>https://static.ordnet.dk/mp3/11022/11022247_1.mp3</v>
+      </c>
+      <c r="J184" t="str">
+        <v>kortform af anhænger</v>
+      </c>
+      <c r="K184" t="str">
+        <v>hangs</v>
+      </c>
+      <c r="L184" t="str">
+        <v>Mens salget af ellastbiler hænger i bremsen, klemmer Volvos nye model med otte batteripakker frem for seks op til 700 kilometers rækkevidde ud af en enkelt opladning.</v>
+      </c>
+      <c r="M184" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N184" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O184" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=h%C3%A6nger</v>
+      </c>
+      <c r="P184" t="str">
+        <v/>
+      </c>
+      <c r="Q184" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R184" t="str">
+        <v/>
+      </c>
+      <c r="S184" t="str">
+        <v/>
+      </c>
+      <c r="T184" t="str">
+        <v/>
+      </c>
+      <c r="U184" t="str">
+        <v/>
+      </c>
+      <c r="V184" t="str">
+        <v/>
+      </c>
+      <c r="W184" t="str">
+        <v/>
+      </c>
+      <c r="X184" t="str">
+        <v/>
+      </c>
+      <c r="Y184" t="str">
+        <v/>
+      </c>
+      <c r="Z184" t="str">
+        <v/>
+      </c>
+      <c r="AA184" t="str">
+        <v/>
+      </c>
+      <c r="AB184" t="str">
+        <v/>
+      </c>
+      <c r="AC184" t="str">
+        <v/>
+      </c>
+      <c r="AD184" t="str">
+        <v/>
+      </c>
+      <c r="AE184" t="str">
+        <v/>
+      </c>
+      <c r="AF184" t="str">
+        <v/>
+      </c>
+      <c r="AG184" t="str">
+        <v/>
+      </c>
+      <c r="AH184" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH183"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH184"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bremsen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH184"/>
+  <dimension ref="A1:AH185"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18405,9 +18405,113 @@
         <v/>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>30f74584-6045-482b-a43d-ede2326b858a</v>
+      </c>
+      <c r="B185" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C185" t="str">
+        <v>bremsen</v>
+      </c>
+      <c r="D185" t="str">
+        <v>bremse</v>
+      </c>
+      <c r="E185" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F185" t="str">
+        <v>en</v>
+      </c>
+      <c r="G185" t="str">
+        <v>bremsen, bremser, bremserne</v>
+      </c>
+      <c r="H185" t="str">
+        <v>[ˈbʁamsə]</v>
+      </c>
+      <c r="I185" t="str">
+        <v>https://static.ordnet.dk/mp3/11006/11006101_1.mp3</v>
+      </c>
+      <c r="J185" t="str">
+        <v>behåret, stuefluelignende insekt som lægger æg på dyr, især heste og kvæg</v>
+      </c>
+      <c r="K185" t="str">
+        <v>the brake</v>
+      </c>
+      <c r="L185" t="str">
+        <v>Mens salget af ellastbiler hænger i bremsen, klemmer Volvos nye model med otte batteripakker frem for seks op til 700 kilometers rækkevidde ud af en enkelt opladning.</v>
+      </c>
+      <c r="M185" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N185" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O185" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=bremsen</v>
+      </c>
+      <c r="P185" t="str">
+        <v/>
+      </c>
+      <c r="Q185" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R185" t="str">
+        <v/>
+      </c>
+      <c r="S185" t="str">
+        <v/>
+      </c>
+      <c r="T185" t="str">
+        <v/>
+      </c>
+      <c r="U185" t="str">
+        <v/>
+      </c>
+      <c r="V185" t="str">
+        <v/>
+      </c>
+      <c r="W185" t="str">
+        <v/>
+      </c>
+      <c r="X185" t="str">
+        <v/>
+      </c>
+      <c r="Y185" t="str">
+        <v/>
+      </c>
+      <c r="Z185" t="str">
+        <v/>
+      </c>
+      <c r="AA185" t="str">
+        <v/>
+      </c>
+      <c r="AB185" t="str">
+        <v/>
+      </c>
+      <c r="AC185" t="str">
+        <v/>
+      </c>
+      <c r="AD185" t="str">
+        <v/>
+      </c>
+      <c r="AE185" t="str">
+        <v/>
+      </c>
+      <c r="AF185" t="str">
+        <v/>
+      </c>
+      <c r="AG185" t="str">
+        <v/>
+      </c>
+      <c r="AH185" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH184"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH185"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "klemmer" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH185"/>
+  <dimension ref="A1:AH186"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18509,9 +18509,113 @@
         <v/>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>e9fa2c00-3211-4ee2-932d-290d88eff8f3</v>
+      </c>
+      <c r="B186" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C186" t="str">
+        <v>klemmer</v>
+      </c>
+      <c r="D186" t="str">
+        <v>klemme</v>
+      </c>
+      <c r="E186" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F186" t="str">
+        <v>en</v>
+      </c>
+      <c r="G186" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H186" t="str">
+        <v>[ˈklεmə]</v>
+      </c>
+      <c r="I186" t="str">
+        <v>https://static.ordnet.dk/mp3/11026/11026260_1.mp3</v>
+      </c>
+      <c r="J186" t="str">
+        <v>redskab som ved hjælp af en fjederanordning klemmer sammen om noget og holder det fast i en bestemt position eller på et bestemt sted</v>
+      </c>
+      <c r="K186" t="str">
+        <v>Clamps</v>
+      </c>
+      <c r="L186" t="str">
+        <v>Mens salget af ellastbiler hænger i bremsen, klemmer Volvos nye model med otte batteripakker frem for seks op til 700 kilometers rækkevidde ud af en enkelt opladning.</v>
+      </c>
+      <c r="M186" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N186" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O186" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=klemmer</v>
+      </c>
+      <c r="P186" t="str">
+        <v/>
+      </c>
+      <c r="Q186" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R186" t="str">
+        <v/>
+      </c>
+      <c r="S186" t="str">
+        <v/>
+      </c>
+      <c r="T186" t="str">
+        <v/>
+      </c>
+      <c r="U186" t="str">
+        <v/>
+      </c>
+      <c r="V186" t="str">
+        <v/>
+      </c>
+      <c r="W186" t="str">
+        <v/>
+      </c>
+      <c r="X186" t="str">
+        <v/>
+      </c>
+      <c r="Y186" t="str">
+        <v/>
+      </c>
+      <c r="Z186" t="str">
+        <v/>
+      </c>
+      <c r="AA186" t="str">
+        <v/>
+      </c>
+      <c r="AB186" t="str">
+        <v/>
+      </c>
+      <c r="AC186" t="str">
+        <v/>
+      </c>
+      <c r="AD186" t="str">
+        <v/>
+      </c>
+      <c r="AE186" t="str">
+        <v/>
+      </c>
+      <c r="AF186" t="str">
+        <v/>
+      </c>
+      <c r="AG186" t="str">
+        <v/>
+      </c>
+      <c r="AH186" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH185"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH186"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "opladning" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH186"/>
+  <dimension ref="A1:AH187"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18613,9 +18613,113 @@
         <v/>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>e3c1f11f-a855-459c-8f03-0b789a2e8f39</v>
+      </c>
+      <c r="B187" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C187" t="str">
+        <v>opladning</v>
+      </c>
+      <c r="D187" t="str">
+        <v>opladning</v>
+      </c>
+      <c r="E187" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F187" t="str">
+        <v>en</v>
+      </c>
+      <c r="G187" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H187" t="str">
+        <v>[-ˌlæðˀneŋ]</v>
+      </c>
+      <c r="I187" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037532_1.mp3</v>
+      </c>
+      <c r="J187" t="str">
+        <v>tilførsel af elektrisk ladning til fx et batteri</v>
+      </c>
+      <c r="K187" t="str">
+        <v>charging</v>
+      </c>
+      <c r="L187" t="str">
+        <v>Mens salget af ellastbiler hænger i bremsen, klemmer Volvos nye model med otte batteripakker frem for seks op til 700 kilometers rækkevidde ud af en enkelt opladning.</v>
+      </c>
+      <c r="M187" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N187" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O187" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=opladning</v>
+      </c>
+      <c r="P187" t="str">
+        <v/>
+      </c>
+      <c r="Q187" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R187" t="str">
+        <v/>
+      </c>
+      <c r="S187" t="str">
+        <v/>
+      </c>
+      <c r="T187" t="str">
+        <v/>
+      </c>
+      <c r="U187" t="str">
+        <v/>
+      </c>
+      <c r="V187" t="str">
+        <v/>
+      </c>
+      <c r="W187" t="str">
+        <v/>
+      </c>
+      <c r="X187" t="str">
+        <v/>
+      </c>
+      <c r="Y187" t="str">
+        <v/>
+      </c>
+      <c r="Z187" t="str">
+        <v/>
+      </c>
+      <c r="AA187" t="str">
+        <v/>
+      </c>
+      <c r="AB187" t="str">
+        <v/>
+      </c>
+      <c r="AC187" t="str">
+        <v/>
+      </c>
+      <c r="AD187" t="str">
+        <v/>
+      </c>
+      <c r="AE187" t="str">
+        <v/>
+      </c>
+      <c r="AF187" t="str">
+        <v/>
+      </c>
+      <c r="AG187" t="str">
+        <v/>
+      </c>
+      <c r="AH187" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH186"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH187"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Mens" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH187"/>
+  <dimension ref="A1:AH188"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18717,9 +18717,113 @@
         <v/>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>648060e1-c449-47a9-b97b-3279f22fb263</v>
+      </c>
+      <c r="B188" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C188" t="str">
+        <v>Mens</v>
+      </c>
+      <c r="D188" t="str">
+        <v>mens</v>
+      </c>
+      <c r="E188" t="str">
+        <v>konjunktion</v>
+      </c>
+      <c r="F188" t="str">
+        <v/>
+      </c>
+      <c r="G188" t="str">
+        <v/>
+      </c>
+      <c r="H188" t="str">
+        <v>[ˈmεnˀs]</v>
+      </c>
+      <c r="I188" t="str">
+        <v>https://static.ordnet.dk/mp3/11033/11033235_1.mp3</v>
+      </c>
+      <c r="J188" t="str">
+        <v>samtidig med eller i løbet af det tidsrum hvor</v>
+      </c>
+      <c r="K188" t="str">
+        <v>While</v>
+      </c>
+      <c r="L188" t="str">
+        <v>Mens salget af ellastbiler hænger i bremsen, klemmer Volvos nye model med otte batteripakker frem for seks op til 700 kilometers rækkevidde ud af en enkelt opladning.</v>
+      </c>
+      <c r="M188" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N188" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O188" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=Mens</v>
+      </c>
+      <c r="P188" t="str">
+        <v/>
+      </c>
+      <c r="Q188" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R188" t="str">
+        <v/>
+      </c>
+      <c r="S188" t="str">
+        <v/>
+      </c>
+      <c r="T188" t="str">
+        <v/>
+      </c>
+      <c r="U188" t="str">
+        <v/>
+      </c>
+      <c r="V188" t="str">
+        <v/>
+      </c>
+      <c r="W188" t="str">
+        <v/>
+      </c>
+      <c r="X188" t="str">
+        <v/>
+      </c>
+      <c r="Y188" t="str">
+        <v/>
+      </c>
+      <c r="Z188" t="str">
+        <v/>
+      </c>
+      <c r="AA188" t="str">
+        <v/>
+      </c>
+      <c r="AB188" t="str">
+        <v/>
+      </c>
+      <c r="AC188" t="str">
+        <v/>
+      </c>
+      <c r="AD188" t="str">
+        <v/>
+      </c>
+      <c r="AE188" t="str">
+        <v/>
+      </c>
+      <c r="AF188" t="str">
+        <v/>
+      </c>
+      <c r="AG188" t="str">
+        <v/>
+      </c>
+      <c r="AH188" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH187"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH188"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "frem for" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -196,40 +196,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH188"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18830,36 +18830,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AB14"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19839,9 +19839,95 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>7397d92f-48f4-4873-b935-529c85c56f94</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C14" t="str">
+        <v>frem for</v>
+      </c>
+      <c r="D14" t="str">
+        <v>frem=forward · for=for</v>
+      </c>
+      <c r="E14" t="str">
+        <v>instead of</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Mens salget af ellastbiler hænger i bremsen, klemmer Volvos nye model med otte batteripakker frem for seks op til 700 kilometers rækkevidde ud af en enkelt opladning.</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="H14" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="I14" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=frem%20for</v>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14" t="str">
+        <v/>
+      </c>
+      <c r="Z14" t="str">
+        <v/>
+      </c>
+      <c r="AA14" t="str">
+        <v/>
+      </c>
+      <c r="AB14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update translation of "klemmer" in Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -18541,7 +18541,7 @@
         <v>redskab som ved hjælp af en fjederanordning klemmer sammen om noget og holder det fast i en bestemt position eller på et bestemt sted</v>
       </c>
       <c r="K186" t="str">
-        <v>Clamps</v>
+        <v>Clamps/squeezes</v>
       </c>
       <c r="L186" t="str">
         <v>Mens salget af ellastbiler hænger i bremsen, klemmer Volvos nye model med otte batteripakker frem for seks op til 700 kilometers rækkevidde ud af en enkelt opladning.</v>
@@ -18832,34 +18832,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB14"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "tomt" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,42 +194,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH188"/>
+  <dimension ref="A1:AH189"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18821,9 +18821,113 @@
         <v/>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>228ea53a-7d74-4ace-adf7-e6afeab9be07</v>
+      </c>
+      <c r="B189" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C189" t="str">
+        <v>tomt</v>
+      </c>
+      <c r="D189" t="str">
+        <v>tomt</v>
+      </c>
+      <c r="E189" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F189" t="str">
+        <v>en</v>
+      </c>
+      <c r="G189" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H189" t="str">
+        <v>[ˈtʌmˀd]</v>
+      </c>
+      <c r="I189" t="str">
+        <v>https://static.ordnet.dk/mp3/12001/12001728_1.mp3</v>
+      </c>
+      <c r="J189" t="str">
+        <v>jordstykke hvor der har ligget en bygning, eller hvor der skal opføres en bygning</v>
+      </c>
+      <c r="K189" t="str">
+        <v>empty</v>
+      </c>
+      <c r="L189" t="str">
+        <v>Fra fabrikken i Gøteborg kan Volvos nye ellastbil på blot én opladning køre ned til Øresundsbroen, hen over Sjælland og helt til Hamborg, før batteriet er tomt. Ved at frigøre plads til ekstra batterier kan den klimavenlige lastbil, FH Aero Electric, nemlig på én enkelt opladning køre op til 700 kilometer.</v>
+      </c>
+      <c r="M189" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N189" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O189" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=tomt</v>
+      </c>
+      <c r="P189" t="str">
+        <v/>
+      </c>
+      <c r="Q189" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R189" t="str">
+        <v/>
+      </c>
+      <c r="S189" t="str">
+        <v/>
+      </c>
+      <c r="T189" t="str">
+        <v/>
+      </c>
+      <c r="U189" t="str">
+        <v/>
+      </c>
+      <c r="V189" t="str">
+        <v/>
+      </c>
+      <c r="W189" t="str">
+        <v/>
+      </c>
+      <c r="X189" t="str">
+        <v/>
+      </c>
+      <c r="Y189" t="str">
+        <v/>
+      </c>
+      <c r="Z189" t="str">
+        <v/>
+      </c>
+      <c r="AA189" t="str">
+        <v/>
+      </c>
+      <c r="AB189" t="str">
+        <v/>
+      </c>
+      <c r="AC189" t="str">
+        <v/>
+      </c>
+      <c r="AD189" t="str">
+        <v/>
+      </c>
+      <c r="AE189" t="str">
+        <v/>
+      </c>
+      <c r="AF189" t="str">
+        <v/>
+      </c>
+      <c r="AG189" t="str">
+        <v/>
+      </c>
+      <c r="AH189" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH188"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH189"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "frigøre" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH189"/>
+  <dimension ref="A1:AH190"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18925,9 +18925,113 @@
         <v/>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>7d1b5cbe-ad5f-4a4e-bc26-f27f61ec964e</v>
+      </c>
+      <c r="B190" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C190" t="str">
+        <v>frigøre</v>
+      </c>
+      <c r="D190" t="str">
+        <v>frigøre</v>
+      </c>
+      <c r="E190" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F190" t="str">
+        <v/>
+      </c>
+      <c r="G190" t="str">
+        <v>frigør, frigjorde, frigjort</v>
+      </c>
+      <c r="H190" t="str">
+        <v>[ˈfʁiˌgɶˀʌ]</v>
+      </c>
+      <c r="I190" t="str">
+        <v>https://static.ordnet.dk/mp3/11016/11016025_1.mp3</v>
+      </c>
+      <c r="J190" t="str">
+        <v>gøre (sig) fri og uafhængig af noget eller nogen der hæmmer, begrænser eller undertrykker</v>
+      </c>
+      <c r="K190" t="str">
+        <v>release</v>
+      </c>
+      <c r="L190" t="str">
+        <v>Fra fabrikken i Gøteborg kan Volvos nye ellastbil på blot én opladning køre ned til Øresundsbroen, hen over Sjælland og helt til Hamborg, før batteriet er tomt. Ved at frigøre plads til ekstra batterier kan den klimavenlige lastbil, FH Aero Electric, nemlig på én enkelt opladning køre op til 700 kilometer.</v>
+      </c>
+      <c r="M190" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N190" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O190" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=frig%C3%B8re</v>
+      </c>
+      <c r="P190" t="str">
+        <v/>
+      </c>
+      <c r="Q190" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R190" t="str">
+        <v/>
+      </c>
+      <c r="S190" t="str">
+        <v/>
+      </c>
+      <c r="T190" t="str">
+        <v/>
+      </c>
+      <c r="U190" t="str">
+        <v/>
+      </c>
+      <c r="V190" t="str">
+        <v/>
+      </c>
+      <c r="W190" t="str">
+        <v/>
+      </c>
+      <c r="X190" t="str">
+        <v/>
+      </c>
+      <c r="Y190" t="str">
+        <v/>
+      </c>
+      <c r="Z190" t="str">
+        <v/>
+      </c>
+      <c r="AA190" t="str">
+        <v/>
+      </c>
+      <c r="AB190" t="str">
+        <v/>
+      </c>
+      <c r="AC190" t="str">
+        <v/>
+      </c>
+      <c r="AD190" t="str">
+        <v/>
+      </c>
+      <c r="AE190" t="str">
+        <v/>
+      </c>
+      <c r="AF190" t="str">
+        <v/>
+      </c>
+      <c r="AG190" t="str">
+        <v/>
+      </c>
+      <c r="AH190" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH189"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH190"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "sat gang" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -196,40 +196,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH190"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19038,36 +19038,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB14"/>
+  <dimension ref="A1:AB15"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20133,9 +20133,95 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>75cd9609-f9da-46e7-8844-b903b335f8f2</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C15" t="str">
+        <v>sat gang</v>
+      </c>
+      <c r="D15" t="str">
+        <v>sat=SAT · gang=walk</v>
+      </c>
+      <c r="E15" t="str">
+        <v>set off</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Volvo har netop sat gang i samlebåndsproduktionen og holder sig ikke tilbage med at knytte store ord til den nye lastbil med rekordhurtig opladning. Volvo Trucks øverste chef, Roger Alm, kalder den for »den bedste i branchen«, mens det ifølge ham »aldrig har været nemmere at udskifte diesellastbilerne«.</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="H15" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="I15" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=sat%20gang</v>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v/>
+      </c>
+      <c r="X15" t="str">
+        <v/>
+      </c>
+      <c r="Y15" t="str">
+        <v/>
+      </c>
+      <c r="Z15" t="str">
+        <v/>
+      </c>
+      <c r="AA15" t="str">
+        <v/>
+      </c>
+      <c r="AB15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB15"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "samlebåndsproduktionen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,42 +194,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH190"/>
+  <dimension ref="A1:AH191"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19029,9 +19029,113 @@
         <v/>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>444635df-08b2-4979-bd21-feae42cde287</v>
+      </c>
+      <c r="B191" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C191" t="str">
+        <v>samlebåndsproduktionen</v>
+      </c>
+      <c r="D191" t="str">
+        <v>samlebåndsproduktion</v>
+      </c>
+      <c r="E191" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F191" t="str">
+        <v>en</v>
+      </c>
+      <c r="G191" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H191" t="str">
+        <v/>
+      </c>
+      <c r="I191" t="str">
+        <v/>
+      </c>
+      <c r="J191" t="str">
+        <v>sammensat af samlebånds + produktion</v>
+      </c>
+      <c r="K191" t="str">
+        <v>assembly line production</v>
+      </c>
+      <c r="L191" t="str">
+        <v>Volvo har netop sat gang i samlebåndsproduktionen og holder sig ikke tilbage med at knytte store ord til den nye lastbil med rekordhurtig opladning. Volvo Trucks øverste chef, Roger Alm, kalder den for »den bedste i branchen«, mens det ifølge ham »aldrig har været nemmere at udskifte diesellastbilerne«.</v>
+      </c>
+      <c r="M191" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N191" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O191" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=samleb%C3%A5ndsproduktionen</v>
+      </c>
+      <c r="P191" t="str">
+        <v/>
+      </c>
+      <c r="Q191" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R191" t="str">
+        <v/>
+      </c>
+      <c r="S191" t="str">
+        <v/>
+      </c>
+      <c r="T191" t="str">
+        <v/>
+      </c>
+      <c r="U191" t="str">
+        <v/>
+      </c>
+      <c r="V191" t="str">
+        <v/>
+      </c>
+      <c r="W191" t="str">
+        <v/>
+      </c>
+      <c r="X191" t="str">
+        <v/>
+      </c>
+      <c r="Y191" t="str">
+        <v/>
+      </c>
+      <c r="Z191" t="str">
+        <v/>
+      </c>
+      <c r="AA191" t="str">
+        <v/>
+      </c>
+      <c r="AB191" t="str">
+        <v/>
+      </c>
+      <c r="AC191" t="str">
+        <v/>
+      </c>
+      <c r="AD191" t="str">
+        <v/>
+      </c>
+      <c r="AE191" t="str">
+        <v/>
+      </c>
+      <c r="AF191" t="str">
+        <v/>
+      </c>
+      <c r="AG191" t="str">
+        <v/>
+      </c>
+      <c r="AH191" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH190"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH191"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -19040,34 +19144,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB15"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "knytte" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH191"/>
+  <dimension ref="A1:AH192"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19133,9 +19133,113 @@
         <v/>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>567548aa-fe15-4362-aa34-285c2e53d14b</v>
+      </c>
+      <c r="B192" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C192" t="str">
+        <v>knytte</v>
+      </c>
+      <c r="D192" t="str">
+        <v>knytte</v>
+      </c>
+      <c r="E192" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F192" t="str">
+        <v>et</v>
+      </c>
+      <c r="G192" t="str">
+        <v>-t, -r, -rne</v>
+      </c>
+      <c r="H192" t="str">
+        <v>[ˈknydə]</v>
+      </c>
+      <c r="I192" t="str">
+        <v>https://static.ordnet.dk/mp3/11026/11026720_1.mp3</v>
+      </c>
+      <c r="J192" t="str">
+        <v>stykke stof der er bundet sammen korsvis i hjørnerne, og som bruges til at bære tøj eller småting i</v>
+      </c>
+      <c r="K192" t="str">
+        <v>attach</v>
+      </c>
+      <c r="L192" t="str">
+        <v>Volvo har netop sat gang i samlebåndsproduktionen og holder sig ikke tilbage med at knytte store ord til den nye lastbil med rekordhurtig opladning. Volvo Trucks øverste chef, Roger Alm, kalder den for »den bedste i branchen«, mens det ifølge ham »aldrig har været nemmere at udskifte diesellastbilerne«.</v>
+      </c>
+      <c r="M192" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N192" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O192" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=knytte</v>
+      </c>
+      <c r="P192" t="str">
+        <v/>
+      </c>
+      <c r="Q192" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R192" t="str">
+        <v/>
+      </c>
+      <c r="S192" t="str">
+        <v/>
+      </c>
+      <c r="T192" t="str">
+        <v/>
+      </c>
+      <c r="U192" t="str">
+        <v/>
+      </c>
+      <c r="V192" t="str">
+        <v/>
+      </c>
+      <c r="W192" t="str">
+        <v/>
+      </c>
+      <c r="X192" t="str">
+        <v/>
+      </c>
+      <c r="Y192" t="str">
+        <v/>
+      </c>
+      <c r="Z192" t="str">
+        <v/>
+      </c>
+      <c r="AA192" t="str">
+        <v/>
+      </c>
+      <c r="AB192" t="str">
+        <v/>
+      </c>
+      <c r="AC192" t="str">
+        <v/>
+      </c>
+      <c r="AD192" t="str">
+        <v/>
+      </c>
+      <c r="AE192" t="str">
+        <v/>
+      </c>
+      <c r="AF192" t="str">
+        <v/>
+      </c>
+      <c r="AG192" t="str">
+        <v/>
+      </c>
+      <c r="AH192" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH191"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH192"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "rekordhurtig" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH192"/>
+  <dimension ref="A1:AH193"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19237,9 +19237,113 @@
         <v/>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>80ea0846-837b-49f1-b5b9-d0b0e10b77f5</v>
+      </c>
+      <c r="B193" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C193" t="str">
+        <v>rekordhurtig</v>
+      </c>
+      <c r="D193" t="str">
+        <v>rekordhurtig</v>
+      </c>
+      <c r="E193" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F193" t="str">
+        <v/>
+      </c>
+      <c r="G193" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H193" t="str">
+        <v/>
+      </c>
+      <c r="I193" t="str">
+        <v/>
+      </c>
+      <c r="J193" t="str">
+        <v>sammensat af rekord + hurtig</v>
+      </c>
+      <c r="K193" t="str">
+        <v>Record fast</v>
+      </c>
+      <c r="L193" t="str">
+        <v>Volvo har netop sat gang i samlebåndsproduktionen og holder sig ikke tilbage med at knytte store ord til den nye lastbil med rekordhurtig opladning. Volvo Trucks øverste chef, Roger Alm, kalder den for »den bedste i branchen«, mens det ifølge ham »aldrig har været nemmere at udskifte diesellastbilerne«.</v>
+      </c>
+      <c r="M193" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N193" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O193" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=rekordhurtig</v>
+      </c>
+      <c r="P193" t="str">
+        <v/>
+      </c>
+      <c r="Q193" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R193" t="str">
+        <v/>
+      </c>
+      <c r="S193" t="str">
+        <v/>
+      </c>
+      <c r="T193" t="str">
+        <v/>
+      </c>
+      <c r="U193" t="str">
+        <v/>
+      </c>
+      <c r="V193" t="str">
+        <v/>
+      </c>
+      <c r="W193" t="str">
+        <v/>
+      </c>
+      <c r="X193" t="str">
+        <v/>
+      </c>
+      <c r="Y193" t="str">
+        <v/>
+      </c>
+      <c r="Z193" t="str">
+        <v/>
+      </c>
+      <c r="AA193" t="str">
+        <v/>
+      </c>
+      <c r="AB193" t="str">
+        <v/>
+      </c>
+      <c r="AC193" t="str">
+        <v/>
+      </c>
+      <c r="AD193" t="str">
+        <v/>
+      </c>
+      <c r="AE193" t="str">
+        <v/>
+      </c>
+      <c r="AF193" t="str">
+        <v/>
+      </c>
+      <c r="AG193" t="str">
+        <v/>
+      </c>
+      <c r="AH193" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH192"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH193"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "udskifte" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH193"/>
+  <dimension ref="A1:AH194"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19341,9 +19341,113 @@
         <v/>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>8b72c7a2-1390-4292-90e2-287f666e0295</v>
+      </c>
+      <c r="B194" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C194" t="str">
+        <v>udskifte</v>
+      </c>
+      <c r="D194" t="str">
+        <v>udskifte</v>
+      </c>
+      <c r="E194" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F194" t="str">
+        <v/>
+      </c>
+      <c r="G194" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H194" t="str">
+        <v>[ˈuðˌsgifdə]</v>
+      </c>
+      <c r="I194" t="str">
+        <v>https://static.ordnet.dk/mp3/12004/12004099_1.mp3</v>
+      </c>
+      <c r="J194" t="str">
+        <v>fjerne og erstatte med noget andet</v>
+      </c>
+      <c r="K194" t="str">
+        <v>replace</v>
+      </c>
+      <c r="L194" t="str">
+        <v>Volvo har netop sat gang i samlebåndsproduktionen og holder sig ikke tilbage med at knytte store ord til den nye lastbil med rekordhurtig opladning. Volvo Trucks øverste chef, Roger Alm, kalder den for »den bedste i branchen«, mens det ifølge ham »aldrig har været nemmere at udskifte diesellastbilerne«.</v>
+      </c>
+      <c r="M194" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N194" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O194" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=udskifte</v>
+      </c>
+      <c r="P194" t="str">
+        <v/>
+      </c>
+      <c r="Q194" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R194" t="str">
+        <v/>
+      </c>
+      <c r="S194" t="str">
+        <v/>
+      </c>
+      <c r="T194" t="str">
+        <v/>
+      </c>
+      <c r="U194" t="str">
+        <v/>
+      </c>
+      <c r="V194" t="str">
+        <v/>
+      </c>
+      <c r="W194" t="str">
+        <v/>
+      </c>
+      <c r="X194" t="str">
+        <v/>
+      </c>
+      <c r="Y194" t="str">
+        <v/>
+      </c>
+      <c r="Z194" t="str">
+        <v/>
+      </c>
+      <c r="AA194" t="str">
+        <v/>
+      </c>
+      <c r="AB194" t="str">
+        <v/>
+      </c>
+      <c r="AC194" t="str">
+        <v/>
+      </c>
+      <c r="AD194" t="str">
+        <v/>
+      </c>
+      <c r="AE194" t="str">
+        <v/>
+      </c>
+      <c r="AF194" t="str">
+        <v/>
+      </c>
+      <c r="AG194" t="str">
+        <v/>
+      </c>
+      <c r="AH194" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH193"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH194"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "omsætter" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH194"/>
+  <dimension ref="A1:AH195"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19445,9 +19445,113 @@
         <v/>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>aba91dbe-079d-4b48-a098-4fecb02d9b3b</v>
+      </c>
+      <c r="B195" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C195" t="str">
+        <v>omsætter</v>
+      </c>
+      <c r="D195" t="str">
+        <v>omsætte</v>
+      </c>
+      <c r="E195" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F195" t="str">
+        <v/>
+      </c>
+      <c r="G195" t="str">
+        <v>-r, omsatte, omsat</v>
+      </c>
+      <c r="H195" t="str">
+        <v>[ˈʌmˌsεdə]</v>
+      </c>
+      <c r="I195" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037255_1.mp3</v>
+      </c>
+      <c r="J195" t="str">
+        <v>få til at overgå fra en form til en anden ved hjælp af en proces, en bearbejdning el.lign.</v>
+      </c>
+      <c r="K195" t="str">
+        <v>Translating</v>
+      </c>
+      <c r="L195" t="str">
+        <v>»Vi omsætter nu banebrydende teknologi til industriel virkelighed,« siger han i en pressemeddelelse.</v>
+      </c>
+      <c r="M195" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N195" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O195" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=oms%C3%A6tter</v>
+      </c>
+      <c r="P195" t="str">
+        <v/>
+      </c>
+      <c r="Q195" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R195" t="str">
+        <v/>
+      </c>
+      <c r="S195" t="str">
+        <v/>
+      </c>
+      <c r="T195" t="str">
+        <v/>
+      </c>
+      <c r="U195" t="str">
+        <v/>
+      </c>
+      <c r="V195" t="str">
+        <v/>
+      </c>
+      <c r="W195" t="str">
+        <v/>
+      </c>
+      <c r="X195" t="str">
+        <v/>
+      </c>
+      <c r="Y195" t="str">
+        <v/>
+      </c>
+      <c r="Z195" t="str">
+        <v/>
+      </c>
+      <c r="AA195" t="str">
+        <v/>
+      </c>
+      <c r="AB195" t="str">
+        <v/>
+      </c>
+      <c r="AC195" t="str">
+        <v/>
+      </c>
+      <c r="AD195" t="str">
+        <v/>
+      </c>
+      <c r="AE195" t="str">
+        <v/>
+      </c>
+      <c r="AF195" t="str">
+        <v/>
+      </c>
+      <c r="AG195" t="str">
+        <v/>
+      </c>
+      <c r="AH195" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH194"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH195"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "banebrydende" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH195"/>
+  <dimension ref="A1:AH196"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19549,9 +19549,113 @@
         <v/>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>6d7cd41b-c161-4c81-854f-eb61aae9f814</v>
+      </c>
+      <c r="B196" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C196" t="str">
+        <v>banebrydende</v>
+      </c>
+      <c r="D196" t="str">
+        <v>banebrydende</v>
+      </c>
+      <c r="E196" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F196" t="str">
+        <v/>
+      </c>
+      <c r="G196" t="str">
+        <v>-, -</v>
+      </c>
+      <c r="H196" t="str">
+        <v>[-ˌbʁyˀðənə]</v>
+      </c>
+      <c r="I196" t="str">
+        <v>https://static.ordnet.dk/mp3/11003/11003383_1.mp3</v>
+      </c>
+      <c r="J196" t="str">
+        <v>markant anderledes og nyskabende i forhold til det alment kendte og accepterede</v>
+      </c>
+      <c r="K196" t="str">
+        <v>Pioneering</v>
+      </c>
+      <c r="L196" t="str">
+        <v>»Vi omsætter nu banebrydende teknologi til industriel virkelighed,« siger han i en pressemeddelelse.</v>
+      </c>
+      <c r="M196" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N196" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O196" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=banebrydende</v>
+      </c>
+      <c r="P196" t="str">
+        <v/>
+      </c>
+      <c r="Q196" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R196" t="str">
+        <v/>
+      </c>
+      <c r="S196" t="str">
+        <v/>
+      </c>
+      <c r="T196" t="str">
+        <v/>
+      </c>
+      <c r="U196" t="str">
+        <v/>
+      </c>
+      <c r="V196" t="str">
+        <v/>
+      </c>
+      <c r="W196" t="str">
+        <v/>
+      </c>
+      <c r="X196" t="str">
+        <v/>
+      </c>
+      <c r="Y196" t="str">
+        <v/>
+      </c>
+      <c r="Z196" t="str">
+        <v/>
+      </c>
+      <c r="AA196" t="str">
+        <v/>
+      </c>
+      <c r="AB196" t="str">
+        <v/>
+      </c>
+      <c r="AC196" t="str">
+        <v/>
+      </c>
+      <c r="AD196" t="str">
+        <v/>
+      </c>
+      <c r="AE196" t="str">
+        <v/>
+      </c>
+      <c r="AF196" t="str">
+        <v/>
+      </c>
+      <c r="AG196" t="str">
+        <v/>
+      </c>
+      <c r="AH196" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH195"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH196"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "virkelighed" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH196"/>
+  <dimension ref="A1:AH197"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19653,9 +19653,113 @@
         <v/>
       </c>
     </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>b876d74c-ab6c-4e19-aa35-ee18fc559b0e</v>
+      </c>
+      <c r="B197" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C197" t="str">
+        <v>virkelighed</v>
+      </c>
+      <c r="D197" t="str">
+        <v>virkelighed</v>
+      </c>
+      <c r="E197" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F197" t="str">
+        <v>en</v>
+      </c>
+      <c r="G197" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H197" t="str">
+        <v>[ˈviɐ̯gəliˌheðˀ]</v>
+      </c>
+      <c r="I197" t="str">
+        <v>https://static.ordnet.dk/mp3/12007/12007014_1.mp3</v>
+      </c>
+      <c r="J197" t="str">
+        <v>sammenfatning af de ting, forhold eller omstændigheder som rent faktisk findes eller gør sig gældende (på et bestemt tidspunkt) i modsætning til det mulige, sandsynlige, ideale eller til det der (kun) findes i fantasien, drømmene el.lign.</v>
+      </c>
+      <c r="K197" t="str">
+        <v>reality</v>
+      </c>
+      <c r="L197" t="str">
+        <v>»Vi omsætter nu banebrydende teknologi til industriel virkelighed,« siger han i en pressemeddelelse.</v>
+      </c>
+      <c r="M197" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N197" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O197" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=virkelighed</v>
+      </c>
+      <c r="P197" t="str">
+        <v/>
+      </c>
+      <c r="Q197" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R197" t="str">
+        <v/>
+      </c>
+      <c r="S197" t="str">
+        <v/>
+      </c>
+      <c r="T197" t="str">
+        <v/>
+      </c>
+      <c r="U197" t="str">
+        <v/>
+      </c>
+      <c r="V197" t="str">
+        <v/>
+      </c>
+      <c r="W197" t="str">
+        <v/>
+      </c>
+      <c r="X197" t="str">
+        <v/>
+      </c>
+      <c r="Y197" t="str">
+        <v/>
+      </c>
+      <c r="Z197" t="str">
+        <v/>
+      </c>
+      <c r="AA197" t="str">
+        <v/>
+      </c>
+      <c r="AB197" t="str">
+        <v/>
+      </c>
+      <c r="AC197" t="str">
+        <v/>
+      </c>
+      <c r="AD197" t="str">
+        <v/>
+      </c>
+      <c r="AE197" t="str">
+        <v/>
+      </c>
+      <c r="AF197" t="str">
+        <v/>
+      </c>
+      <c r="AG197" t="str">
+        <v/>
+      </c>
+      <c r="AH197" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH196"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH197"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "pressemeddelelse" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH197"/>
+  <dimension ref="A1:AH198"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19757,9 +19757,113 @@
         <v/>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>63d7b873-4250-4143-b1cf-35d3c7c310c5</v>
+      </c>
+      <c r="B198" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C198" t="str">
+        <v>pressemeddelelse</v>
+      </c>
+      <c r="D198" t="str">
+        <v>pressemeddelelse</v>
+      </c>
+      <c r="E198" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F198" t="str">
+        <v>en</v>
+      </c>
+      <c r="G198" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H198" t="str">
+        <v/>
+      </c>
+      <c r="I198" t="str">
+        <v>https://static.ordnet.dk/mp3/11040/11040738_1.mp3</v>
+      </c>
+      <c r="J198" t="str">
+        <v>meddelelse som man sender ud til pressen og andre medier i håb om at opnå offentliggørelse eller anden opfølgning fra pressens side</v>
+      </c>
+      <c r="K198" t="str">
+        <v>press release</v>
+      </c>
+      <c r="L198" t="str">
+        <v>»Vi omsætter nu banebrydende teknologi til industriel virkelighed,« siger han i en pressemeddelelse.</v>
+      </c>
+      <c r="M198" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N198" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O198" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=pressemeddelelse</v>
+      </c>
+      <c r="P198" t="str">
+        <v/>
+      </c>
+      <c r="Q198" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R198" t="str">
+        <v/>
+      </c>
+      <c r="S198" t="str">
+        <v/>
+      </c>
+      <c r="T198" t="str">
+        <v/>
+      </c>
+      <c r="U198" t="str">
+        <v/>
+      </c>
+      <c r="V198" t="str">
+        <v/>
+      </c>
+      <c r="W198" t="str">
+        <v/>
+      </c>
+      <c r="X198" t="str">
+        <v/>
+      </c>
+      <c r="Y198" t="str">
+        <v/>
+      </c>
+      <c r="Z198" t="str">
+        <v/>
+      </c>
+      <c r="AA198" t="str">
+        <v/>
+      </c>
+      <c r="AB198" t="str">
+        <v/>
+      </c>
+      <c r="AC198" t="str">
+        <v/>
+      </c>
+      <c r="AD198" t="str">
+        <v/>
+      </c>
+      <c r="AE198" t="str">
+        <v/>
+      </c>
+      <c r="AF198" t="str">
+        <v/>
+      </c>
+      <c r="AG198" t="str">
+        <v/>
+      </c>
+      <c r="AH198" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH197"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH198"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "skud" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH198"/>
+  <dimension ref="A1:AH199"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19861,9 +19861,113 @@
         <v/>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>c8115a69-e84b-447c-9d4b-c44130ad770e</v>
+      </c>
+      <c r="B199" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C199" t="str">
+        <v>skud</v>
+      </c>
+      <c r="D199" t="str">
+        <v>skud</v>
+      </c>
+      <c r="E199" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F199" t="str">
+        <v>et</v>
+      </c>
+      <c r="G199" t="str">
+        <v>-det, -, -dene</v>
+      </c>
+      <c r="H199" t="str">
+        <v>[ˈsguð]</v>
+      </c>
+      <c r="I199" t="str">
+        <v>https://static.ordnet.dk/mp3/11047/11047131_1.mp3</v>
+      </c>
+      <c r="J199" t="str">
+        <v>affyring af et projektil</v>
+      </c>
+      <c r="K199" t="str">
+        <v>shot</v>
+      </c>
+      <c r="L199" t="str">
+        <v>Volvos nye skud på stammen overflødiggør ikke alene ture til tankstationer, der på grund af krigene i Mellemøsten sælger diesel dyrere end nogensinde før. Den har en længere rækkevidde end konkurrenternes, såsom ellastbilerne fra Scania og Renault, der kører 400-660 kilometer per fuld opladning.</v>
+      </c>
+      <c r="M199" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N199" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O199" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=skud</v>
+      </c>
+      <c r="P199" t="str">
+        <v/>
+      </c>
+      <c r="Q199" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R199" t="str">
+        <v/>
+      </c>
+      <c r="S199" t="str">
+        <v/>
+      </c>
+      <c r="T199" t="str">
+        <v/>
+      </c>
+      <c r="U199" t="str">
+        <v/>
+      </c>
+      <c r="V199" t="str">
+        <v/>
+      </c>
+      <c r="W199" t="str">
+        <v/>
+      </c>
+      <c r="X199" t="str">
+        <v/>
+      </c>
+      <c r="Y199" t="str">
+        <v/>
+      </c>
+      <c r="Z199" t="str">
+        <v/>
+      </c>
+      <c r="AA199" t="str">
+        <v/>
+      </c>
+      <c r="AB199" t="str">
+        <v/>
+      </c>
+      <c r="AC199" t="str">
+        <v/>
+      </c>
+      <c r="AD199" t="str">
+        <v/>
+      </c>
+      <c r="AE199" t="str">
+        <v/>
+      </c>
+      <c r="AF199" t="str">
+        <v/>
+      </c>
+      <c r="AG199" t="str">
+        <v/>
+      </c>
+      <c r="AH199" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH198"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH199"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "stammen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH199"/>
+  <dimension ref="A1:AH200"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19965,9 +19965,113 @@
         <v/>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>eabf6724-1b66-465f-92d1-d519d4cb677b</v>
+      </c>
+      <c r="B200" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C200" t="str">
+        <v>stammen</v>
+      </c>
+      <c r="D200" t="str">
+        <v>stammen</v>
+      </c>
+      <c r="E200" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F200" t="str">
+        <v>en</v>
+      </c>
+      <c r="G200" t="str">
+        <v/>
+      </c>
+      <c r="H200" t="str">
+        <v>[ˈsdɑmən]</v>
+      </c>
+      <c r="I200" t="str">
+        <v>https://static.ordnet.dk/mp3/51002/51002421_1.mp3</v>
+      </c>
+      <c r="J200" t="str">
+        <v>krampagtige sammentrækninger i taleorganerne der bevirker at lyde eller ord gentages stødvis</v>
+      </c>
+      <c r="K200" t="str">
+        <v>The tribe</v>
+      </c>
+      <c r="L200" t="str">
+        <v>Volvos nye skud på stammen overflødiggør ikke alene ture til tankstationer, der på grund af krigene i Mellemøsten sælger diesel dyrere end nogensinde før. Den har en længere rækkevidde end konkurrenternes, såsom ellastbilerne fra Scania og Renault, der kører 400-660 kilometer per fuld opladning.</v>
+      </c>
+      <c r="M200" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N200" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O200" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=stammen</v>
+      </c>
+      <c r="P200" t="str">
+        <v/>
+      </c>
+      <c r="Q200" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R200" t="str">
+        <v/>
+      </c>
+      <c r="S200" t="str">
+        <v/>
+      </c>
+      <c r="T200" t="str">
+        <v/>
+      </c>
+      <c r="U200" t="str">
+        <v/>
+      </c>
+      <c r="V200" t="str">
+        <v/>
+      </c>
+      <c r="W200" t="str">
+        <v/>
+      </c>
+      <c r="X200" t="str">
+        <v/>
+      </c>
+      <c r="Y200" t="str">
+        <v/>
+      </c>
+      <c r="Z200" t="str">
+        <v/>
+      </c>
+      <c r="AA200" t="str">
+        <v/>
+      </c>
+      <c r="AB200" t="str">
+        <v/>
+      </c>
+      <c r="AC200" t="str">
+        <v/>
+      </c>
+      <c r="AD200" t="str">
+        <v/>
+      </c>
+      <c r="AE200" t="str">
+        <v/>
+      </c>
+      <c r="AF200" t="str">
+        <v/>
+      </c>
+      <c r="AG200" t="str">
+        <v/>
+      </c>
+      <c r="AH200" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH199"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH200"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "overflødiggør" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH200"/>
+  <dimension ref="A1:AH201"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20069,9 +20069,113 @@
         <v/>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>cbe3ae65-00a5-47e6-97f8-1c1ff05b80c5</v>
+      </c>
+      <c r="B201" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C201" t="str">
+        <v>overflødiggør</v>
+      </c>
+      <c r="D201" t="str">
+        <v>overflødiggøre</v>
+      </c>
+      <c r="E201" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F201" t="str">
+        <v/>
+      </c>
+      <c r="G201" t="str">
+        <v>..gør, ..gjorde, ..gjort</v>
+      </c>
+      <c r="H201" t="str">
+        <v>[-ˌgɶˀʌ]</v>
+      </c>
+      <c r="I201" t="str">
+        <v>https://static.ordnet.dk/mp3/11038/11038271_1.mp3</v>
+      </c>
+      <c r="J201" t="str">
+        <v>gøre overflødig</v>
+      </c>
+      <c r="K201" t="str">
+        <v>Makes redundant</v>
+      </c>
+      <c r="L201" t="str">
+        <v>Volvos nye skud på stammen overflødiggør ikke alene ture til tankstationer, der på grund af krigene i Mellemøsten sælger diesel dyrere end nogensinde før. Den har en længere rækkevidde end konkurrenternes, såsom ellastbilerne fra Scania og Renault, der kører 400-660 kilometer per fuld opladning.</v>
+      </c>
+      <c r="M201" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N201" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O201" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=overfl%C3%B8digg%C3%B8r</v>
+      </c>
+      <c r="P201" t="str">
+        <v/>
+      </c>
+      <c r="Q201" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R201" t="str">
+        <v/>
+      </c>
+      <c r="S201" t="str">
+        <v/>
+      </c>
+      <c r="T201" t="str">
+        <v/>
+      </c>
+      <c r="U201" t="str">
+        <v/>
+      </c>
+      <c r="V201" t="str">
+        <v/>
+      </c>
+      <c r="W201" t="str">
+        <v/>
+      </c>
+      <c r="X201" t="str">
+        <v/>
+      </c>
+      <c r="Y201" t="str">
+        <v/>
+      </c>
+      <c r="Z201" t="str">
+        <v/>
+      </c>
+      <c r="AA201" t="str">
+        <v/>
+      </c>
+      <c r="AB201" t="str">
+        <v/>
+      </c>
+      <c r="AC201" t="str">
+        <v/>
+      </c>
+      <c r="AD201" t="str">
+        <v/>
+      </c>
+      <c r="AE201" t="str">
+        <v/>
+      </c>
+      <c r="AF201" t="str">
+        <v/>
+      </c>
+      <c r="AG201" t="str">
+        <v/>
+      </c>
+      <c r="AH201" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH200"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH201"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "ture" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH201"/>
+  <dimension ref="A1:AH202"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20173,9 +20173,113 @@
         <v/>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>c0db822e-53c7-474f-baf2-24c570b98d3a</v>
+      </c>
+      <c r="B202" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C202" t="str">
+        <v>ture</v>
+      </c>
+      <c r="D202" t="str">
+        <v>ture</v>
+      </c>
+      <c r="E202" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F202" t="str">
+        <v/>
+      </c>
+      <c r="G202" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H202" t="str">
+        <v>[ˈtuːʌ]</v>
+      </c>
+      <c r="I202" t="str">
+        <v>https://static.ordnet.dk/mp3/12002/12002893_1.mp3</v>
+      </c>
+      <c r="J202" t="str">
+        <v>rejse planløst fra sted til sted</v>
+      </c>
+      <c r="K202" t="str">
+        <v>trips</v>
+      </c>
+      <c r="L202" t="str">
+        <v>Volvos nye skud på stammen overflødiggør ikke alene ture til tankstationer, der på grund af krigene i Mellemøsten sælger diesel dyrere end nogensinde før. Den har en længere rækkevidde end konkurrenternes, såsom ellastbilerne fra Scania og Renault, der kører 400-660 kilometer per fuld opladning.</v>
+      </c>
+      <c r="M202" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N202" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O202" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=ture</v>
+      </c>
+      <c r="P202" t="str">
+        <v/>
+      </c>
+      <c r="Q202" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R202" t="str">
+        <v/>
+      </c>
+      <c r="S202" t="str">
+        <v/>
+      </c>
+      <c r="T202" t="str">
+        <v/>
+      </c>
+      <c r="U202" t="str">
+        <v/>
+      </c>
+      <c r="V202" t="str">
+        <v/>
+      </c>
+      <c r="W202" t="str">
+        <v/>
+      </c>
+      <c r="X202" t="str">
+        <v/>
+      </c>
+      <c r="Y202" t="str">
+        <v/>
+      </c>
+      <c r="Z202" t="str">
+        <v/>
+      </c>
+      <c r="AA202" t="str">
+        <v/>
+      </c>
+      <c r="AB202" t="str">
+        <v/>
+      </c>
+      <c r="AC202" t="str">
+        <v/>
+      </c>
+      <c r="AD202" t="str">
+        <v/>
+      </c>
+      <c r="AE202" t="str">
+        <v/>
+      </c>
+      <c r="AF202" t="str">
+        <v/>
+      </c>
+      <c r="AG202" t="str">
+        <v/>
+      </c>
+      <c r="AH202" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH201"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH202"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "dyrere" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH202"/>
+  <dimension ref="A1:AH203"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20277,9 +20277,113 @@
         <v/>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>9f3298d5-dc0c-4cb3-89fb-cdb1a1c99dac</v>
+      </c>
+      <c r="B203" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C203" t="str">
+        <v>dyrere</v>
+      </c>
+      <c r="D203" t="str">
+        <v>dyr</v>
+      </c>
+      <c r="E203" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F203" t="str">
+        <v/>
+      </c>
+      <c r="G203" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H203" t="str">
+        <v>[ˈdyɐ̯ˀ]</v>
+      </c>
+      <c r="I203" t="str">
+        <v>https://static.ordnet.dk/mp3/11010/11010115_1.mp3</v>
+      </c>
+      <c r="J203" t="str">
+        <v>som koster forholdsvis mange penge at anskaffe, benytte, vedligeholde, opretholde, forsørge el.lign. fx om ting eller tjenesteydelse</v>
+      </c>
+      <c r="K203" t="str">
+        <v>more expensive</v>
+      </c>
+      <c r="L203" t="str">
+        <v>Volvos nye skud på stammen overflødiggør ikke alene ture til tankstationer, der på grund af krigene i Mellemøsten sælger diesel dyrere end nogensinde før. Den har en længere rækkevidde end konkurrenternes, såsom ellastbilerne fra Scania og Renault, der kører 400-660 kilometer per fuld opladning.</v>
+      </c>
+      <c r="M203" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N203" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O203" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=dyrere</v>
+      </c>
+      <c r="P203" t="str">
+        <v/>
+      </c>
+      <c r="Q203" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R203" t="str">
+        <v/>
+      </c>
+      <c r="S203" t="str">
+        <v/>
+      </c>
+      <c r="T203" t="str">
+        <v/>
+      </c>
+      <c r="U203" t="str">
+        <v/>
+      </c>
+      <c r="V203" t="str">
+        <v/>
+      </c>
+      <c r="W203" t="str">
+        <v/>
+      </c>
+      <c r="X203" t="str">
+        <v/>
+      </c>
+      <c r="Y203" t="str">
+        <v/>
+      </c>
+      <c r="Z203" t="str">
+        <v/>
+      </c>
+      <c r="AA203" t="str">
+        <v/>
+      </c>
+      <c r="AB203" t="str">
+        <v/>
+      </c>
+      <c r="AC203" t="str">
+        <v/>
+      </c>
+      <c r="AD203" t="str">
+        <v/>
+      </c>
+      <c r="AE203" t="str">
+        <v/>
+      </c>
+      <c r="AF203" t="str">
+        <v/>
+      </c>
+      <c r="AG203" t="str">
+        <v/>
+      </c>
+      <c r="AH203" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH202"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH203"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "konkurrenternes" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH203"/>
+  <dimension ref="A1:AH204"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20381,9 +20381,113 @@
         <v/>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>5ed784d0-79ae-432e-8202-cf8f51348be6</v>
+      </c>
+      <c r="B204" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C204" t="str">
+        <v>konkurrenternes</v>
+      </c>
+      <c r="D204" t="str">
+        <v>konkurrent</v>
+      </c>
+      <c r="E204" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F204" t="str">
+        <v>en</v>
+      </c>
+      <c r="G204" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H204" t="str">
+        <v>[kʌŋgoˈʁanˀd]</v>
+      </c>
+      <c r="I204" t="str">
+        <v>https://static.ordnet.dk/mp3/11027/11027357_1.mp3</v>
+      </c>
+      <c r="J204" t="str">
+        <v>modpart i en konkurrence eller kappestrid</v>
+      </c>
+      <c r="K204" t="str">
+        <v>competitors</v>
+      </c>
+      <c r="L204" t="str">
+        <v>Volvos nye skud på stammen overflødiggør ikke alene ture til tankstationer, der på grund af krigene i Mellemøsten sælger diesel dyrere end nogensinde før. Den har en længere rækkevidde end konkurrenternes, såsom ellastbilerne fra Scania og Renault, der kører 400-660 kilometer per fuld opladning.</v>
+      </c>
+      <c r="M204" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N204" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O204" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=konkurrenternes</v>
+      </c>
+      <c r="P204" t="str">
+        <v/>
+      </c>
+      <c r="Q204" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R204" t="str">
+        <v/>
+      </c>
+      <c r="S204" t="str">
+        <v/>
+      </c>
+      <c r="T204" t="str">
+        <v/>
+      </c>
+      <c r="U204" t="str">
+        <v/>
+      </c>
+      <c r="V204" t="str">
+        <v/>
+      </c>
+      <c r="W204" t="str">
+        <v/>
+      </c>
+      <c r="X204" t="str">
+        <v/>
+      </c>
+      <c r="Y204" t="str">
+        <v/>
+      </c>
+      <c r="Z204" t="str">
+        <v/>
+      </c>
+      <c r="AA204" t="str">
+        <v/>
+      </c>
+      <c r="AB204" t="str">
+        <v/>
+      </c>
+      <c r="AC204" t="str">
+        <v/>
+      </c>
+      <c r="AD204" t="str">
+        <v/>
+      </c>
+      <c r="AE204" t="str">
+        <v/>
+      </c>
+      <c r="AF204" t="str">
+        <v/>
+      </c>
+      <c r="AG204" t="str">
+        <v/>
+      </c>
+      <c r="AH204" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH203"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH204"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "såsom" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH204"/>
+  <dimension ref="A1:AH205"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20485,9 +20485,113 @@
         <v/>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>522f829f-fd5c-4fd5-b8a6-14b43c028452</v>
+      </c>
+      <c r="B205" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C205" t="str">
+        <v>såsom</v>
+      </c>
+      <c r="D205" t="str">
+        <v>såsom</v>
+      </c>
+      <c r="E205" t="str">
+        <v>konjunktion</v>
+      </c>
+      <c r="F205" t="str">
+        <v/>
+      </c>
+      <c r="G205" t="str">
+        <v/>
+      </c>
+      <c r="H205" t="str">
+        <v>[ˈsɔˀsʌm]</v>
+      </c>
+      <c r="I205" t="str">
+        <v>https://static.ordnet.dk/mp3/11052/11052560_1.mp3</v>
+      </c>
+      <c r="J205" t="str">
+        <v>bruges til angivelse af et eller flere eksempler på noget</v>
+      </c>
+      <c r="K205" t="str">
+        <v>such as</v>
+      </c>
+      <c r="L205" t="str">
+        <v>Volvos nye skud på stammen overflødiggør ikke alene ture til tankstationer, der på grund af krigene i Mellemøsten sælger diesel dyrere end nogensinde før. Den har en længere rækkevidde end konkurrenternes, såsom ellastbilerne fra Scania og Renault, der kører 400-660 kilometer per fuld opladning.</v>
+      </c>
+      <c r="M205" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N205" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O205" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=s%C3%A5som</v>
+      </c>
+      <c r="P205" t="str">
+        <v/>
+      </c>
+      <c r="Q205" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R205" t="str">
+        <v/>
+      </c>
+      <c r="S205" t="str">
+        <v/>
+      </c>
+      <c r="T205" t="str">
+        <v/>
+      </c>
+      <c r="U205" t="str">
+        <v/>
+      </c>
+      <c r="V205" t="str">
+        <v/>
+      </c>
+      <c r="W205" t="str">
+        <v/>
+      </c>
+      <c r="X205" t="str">
+        <v/>
+      </c>
+      <c r="Y205" t="str">
+        <v/>
+      </c>
+      <c r="Z205" t="str">
+        <v/>
+      </c>
+      <c r="AA205" t="str">
+        <v/>
+      </c>
+      <c r="AB205" t="str">
+        <v/>
+      </c>
+      <c r="AC205" t="str">
+        <v/>
+      </c>
+      <c r="AD205" t="str">
+        <v/>
+      </c>
+      <c r="AE205" t="str">
+        <v/>
+      </c>
+      <c r="AF205" t="str">
+        <v/>
+      </c>
+      <c r="AG205" t="str">
+        <v/>
+      </c>
+      <c r="AH205" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH204"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH205"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bagakslen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH205"/>
+  <dimension ref="A1:AH206"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20589,9 +20589,113 @@
         <v/>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>d91bb7ab-5138-4f54-a7cd-7beac906fb61</v>
+      </c>
+      <c r="B206" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C206" t="str">
+        <v>bagakslen</v>
+      </c>
+      <c r="D206" t="str">
+        <v>bagaksel</v>
+      </c>
+      <c r="E206" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F206" t="str">
+        <v>en</v>
+      </c>
+      <c r="G206" t="str">
+        <v>bagakslen (eller uofficiel form: -en), bagaksler, bagakslerne Se bøjning i skema</v>
+      </c>
+      <c r="H206" t="str">
+        <v/>
+      </c>
+      <c r="I206" t="str">
+        <v>https://static.ordnet.dk/mp3/11003/11003079_1.mp3</v>
+      </c>
+      <c r="J206" t="str">
+        <v>aksel som er placeret i den bageste del af et køretøj</v>
+      </c>
+      <c r="K206" t="str">
+        <v>the rear axle</v>
+      </c>
+      <c r="L206" t="str">
+        <v>Ved at flytte motor og gearkasse til bagakslen har Volvo Trucks frigjort plads til ekstra batterier. Mens de tidligere elektriske lastbiler har 4-6 batteripakker med en batterikapacitet på 540 kWh, som rækker til op mod 470 kilometer, har FH Aero Electric otte batteripakker med samlet 725 kWh.</v>
+      </c>
+      <c r="M206" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N206" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O206" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=bagakslen</v>
+      </c>
+      <c r="P206" t="str">
+        <v/>
+      </c>
+      <c r="Q206" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R206" t="str">
+        <v/>
+      </c>
+      <c r="S206" t="str">
+        <v/>
+      </c>
+      <c r="T206" t="str">
+        <v/>
+      </c>
+      <c r="U206" t="str">
+        <v/>
+      </c>
+      <c r="V206" t="str">
+        <v/>
+      </c>
+      <c r="W206" t="str">
+        <v/>
+      </c>
+      <c r="X206" t="str">
+        <v/>
+      </c>
+      <c r="Y206" t="str">
+        <v/>
+      </c>
+      <c r="Z206" t="str">
+        <v/>
+      </c>
+      <c r="AA206" t="str">
+        <v/>
+      </c>
+      <c r="AB206" t="str">
+        <v/>
+      </c>
+      <c r="AC206" t="str">
+        <v/>
+      </c>
+      <c r="AD206" t="str">
+        <v/>
+      </c>
+      <c r="AE206" t="str">
+        <v/>
+      </c>
+      <c r="AF206" t="str">
+        <v/>
+      </c>
+      <c r="AG206" t="str">
+        <v/>
+      </c>
+      <c r="AH206" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH205"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH206"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Trægt" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH206"/>
+  <dimension ref="A1:AH207"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20693,9 +20693,113 @@
         <v/>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>fdea3d30-2094-4c25-840c-73470cd27c07</v>
+      </c>
+      <c r="B207" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="C207" t="str">
+        <v>Trægt</v>
+      </c>
+      <c r="D207" t="str">
+        <v>træg</v>
+      </c>
+      <c r="E207" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F207" t="str">
+        <v/>
+      </c>
+      <c r="G207" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H207" t="str">
+        <v>[ˈtʁεˀj]</v>
+      </c>
+      <c r="I207" t="str">
+        <v>https://static.ordnet.dk/mp3/12002/12002646_1.mp3</v>
+      </c>
+      <c r="J207" t="str">
+        <v>præget af langsommelighed eller mangel på aktivitet og engagement om person, handling el.lign.</v>
+      </c>
+      <c r="K207" t="str">
+        <v>sluggish</v>
+      </c>
+      <c r="L207" t="str">
+        <v>Trægt salg af ellastbiler</v>
+      </c>
+      <c r="M207" t="str">
+        <v>Volvo knækker kode: El-lastbil med rækkevidde på 700 kilometer rammer gaden | Ingeniøren</v>
+      </c>
+      <c r="N207" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden</v>
+      </c>
+      <c r="O207" t="str">
+        <v>https://ing.dk/artikel/volvo-knaekker-kode-el-lastbil-med-raekkevidde-paa-700-kilometer-rammer-gaden#:~:text=Tr%C3%A6gt</v>
+      </c>
+      <c r="P207" t="str">
+        <v/>
+      </c>
+      <c r="Q207" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R207" t="str">
+        <v/>
+      </c>
+      <c r="S207" t="str">
+        <v/>
+      </c>
+      <c r="T207" t="str">
+        <v/>
+      </c>
+      <c r="U207" t="str">
+        <v/>
+      </c>
+      <c r="V207" t="str">
+        <v/>
+      </c>
+      <c r="W207" t="str">
+        <v/>
+      </c>
+      <c r="X207" t="str">
+        <v/>
+      </c>
+      <c r="Y207" t="str">
+        <v/>
+      </c>
+      <c r="Z207" t="str">
+        <v/>
+      </c>
+      <c r="AA207" t="str">
+        <v/>
+      </c>
+      <c r="AB207" t="str">
+        <v/>
+      </c>
+      <c r="AC207" t="str">
+        <v/>
+      </c>
+      <c r="AD207" t="str">
+        <v/>
+      </c>
+      <c r="AE207" t="str">
+        <v/>
+      </c>
+      <c r="AF207" t="str">
+        <v/>
+      </c>
+      <c r="AG207" t="str">
+        <v/>
+      </c>
+      <c r="AH207" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH206"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH207"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: add 1 in Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH207"/>
+  <dimension ref="A1:AH208"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20797,9 +20797,113 @@
         <v/>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>54c22739-f9be-41dc-962d-63934ab7759a</v>
+      </c>
+      <c r="B208" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="C208" t="str">
+        <v>nedbrud</v>
+      </c>
+      <c r="D208" t="str">
+        <v/>
+      </c>
+      <c r="E208" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F208" t="str">
+        <v>et</v>
+      </c>
+      <c r="G208" t="str">
+        <v>-det, -, -dene</v>
+      </c>
+      <c r="H208" t="str">
+        <v>[ˈneðˌbʁuð]</v>
+      </c>
+      <c r="I208" t="str">
+        <v>https://static.ordnet.dk/mp3/11035/11035622_1.mp3</v>
+      </c>
+      <c r="J208" t="str">
+        <v>det at noget bryder ned eller bryder sammen</v>
+      </c>
+      <c r="K208" t="str">
+        <v>breakdown</v>
+      </c>
+      <c r="L208" t="str">
+        <v>En kvart milliard skal sikre 800.000 husstande mod strømnedbrud: »Det er især truslen fra fysiske angreb«</v>
+      </c>
+      <c r="M208" t="str">
+        <v>En kvart milliard skal sikre 800.000 husstande mod strømnedbrud: »Det er især truslen fra fysiske angreb« | Ingeniøren</v>
+      </c>
+      <c r="N208" t="str">
+        <v>https://ing.dk/artikel/en-kvart-milliard-skal-sikre-800000-husstande-mod-stroemnedbrud-det-er-isaer-truslen-fra-fysiske</v>
+      </c>
+      <c r="O208" t="str">
+        <v>https://ing.dk/artikel/en-kvart-milliard-skal-sikre-800000-husstande-mod-stroemnedbrud-det-er-isaer-truslen-fra-fysiske#:~:text=nedbrud</v>
+      </c>
+      <c r="P208" t="str">
+        <v/>
+      </c>
+      <c r="Q208" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R208" t="str">
+        <v/>
+      </c>
+      <c r="S208" t="str">
+        <v/>
+      </c>
+      <c r="T208">
+        <v>0</v>
+      </c>
+      <c r="U208" t="str">
+        <v/>
+      </c>
+      <c r="V208">
+        <v>0</v>
+      </c>
+      <c r="W208">
+        <v>0</v>
+      </c>
+      <c r="X208" t="str">
+        <v/>
+      </c>
+      <c r="Y208">
+        <v>0</v>
+      </c>
+      <c r="Z208" t="str">
+        <v/>
+      </c>
+      <c r="AA208">
+        <v>0</v>
+      </c>
+      <c r="AB208">
+        <v>0</v>
+      </c>
+      <c r="AC208" t="str">
+        <v/>
+      </c>
+      <c r="AD208" t="str">
+        <v/>
+      </c>
+      <c r="AE208" t="str">
+        <v/>
+      </c>
+      <c r="AF208" t="str">
+        <v/>
+      </c>
+      <c r="AG208" t="str">
+        <v/>
+      </c>
+      <c r="AH208" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH207"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH208"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "såret" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH209"/>
+  <dimension ref="A1:AH210"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21005,9 +21005,113 @@
         <v/>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>10b11507-1253-4899-a3b1-110a693babb9</v>
+      </c>
+      <c r="B210" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="C210" t="str">
+        <v>såret</v>
+      </c>
+      <c r="D210" t="str">
+        <v>sår</v>
+      </c>
+      <c r="E210" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F210" t="str">
+        <v>et</v>
+      </c>
+      <c r="G210" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H210" t="str">
+        <v>[ˈsɒˀ]</v>
+      </c>
+      <c r="I210" t="str">
+        <v>https://static.ordnet.dk/mp3/11052/11052554_1.mp3</v>
+      </c>
+      <c r="J210" t="str">
+        <v>hul på hud eller slimhinde som blodet kan trænge ud gennem, og som evt. blotlægger dybereliggende væv eller organer også om et sådant hul som er ved at hele op og er dækket af en tør hinde eller en skorpe</v>
+      </c>
+      <c r="K210" t="str">
+        <v>hurt</v>
+      </c>
+      <c r="L210" t="str">
+        <v>Kampfly styrtede tirsdag ned nær den amerikanske Spangdahlem-luftbase i det vestlige Tyskland. Piloten overlevede ved at skyde sig ud med katapultsædet, mens én person på jorden blev såret.</v>
+      </c>
+      <c r="M210" t="str">
+        <v>Pilot hoppede ud med katapult: Amerikansk F-16-kampfly styrter ned i Tyskland | Ingeniøren</v>
+      </c>
+      <c r="N210" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+      </c>
+      <c r="O210" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=s%C3%A5ret</v>
+      </c>
+      <c r="P210" t="str">
+        <v/>
+      </c>
+      <c r="Q210" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R210" t="str">
+        <v/>
+      </c>
+      <c r="S210" t="str">
+        <v/>
+      </c>
+      <c r="T210" t="str">
+        <v/>
+      </c>
+      <c r="U210" t="str">
+        <v/>
+      </c>
+      <c r="V210" t="str">
+        <v/>
+      </c>
+      <c r="W210" t="str">
+        <v/>
+      </c>
+      <c r="X210" t="str">
+        <v/>
+      </c>
+      <c r="Y210" t="str">
+        <v/>
+      </c>
+      <c r="Z210" t="str">
+        <v/>
+      </c>
+      <c r="AA210" t="str">
+        <v/>
+      </c>
+      <c r="AB210" t="str">
+        <v/>
+      </c>
+      <c r="AC210" t="str">
+        <v/>
+      </c>
+      <c r="AD210" t="str">
+        <v/>
+      </c>
+      <c r="AE210" t="str">
+        <v/>
+      </c>
+      <c r="AF210" t="str">
+        <v/>
+      </c>
+      <c r="AG210" t="str">
+        <v/>
+      </c>
+      <c r="AH210" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH209"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH210"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kampfly" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH210"/>
+  <dimension ref="A1:AH211"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21109,9 +21109,113 @@
         <v/>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>9fbf26ed-a230-410a-95ad-72d098cf9be7</v>
+      </c>
+      <c r="B211" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="C211" t="str">
+        <v>kampfly</v>
+      </c>
+      <c r="D211" t="str">
+        <v>kampfly</v>
+      </c>
+      <c r="E211" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F211" t="str">
+        <v>et</v>
+      </c>
+      <c r="G211" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H211" t="str">
+        <v/>
+      </c>
+      <c r="I211" t="str">
+        <v>https://static.ordnet.dk/mp3/11025/11025150_1.mp3</v>
+      </c>
+      <c r="J211" t="str">
+        <v>mindre, bevæbnet, meget manøvredygtigt og hurtigt militært fly, især beregnet til angreb på mål på landjorden eller havet</v>
+      </c>
+      <c r="K211" t="str">
+        <v>Fighting aircraft</v>
+      </c>
+      <c r="L211" t="str">
+        <v>Et kampfly af typen F-16 fra det amerikanske luftvåben styrtede ned tirsdag eftermiddag tæt på Spangdahlem-luftbasen i det vestlige Tyskland. Det skriver mediet Deutsche Welle.</v>
+      </c>
+      <c r="M211" t="str">
+        <v>Pilot hoppede ud med katapult: Amerikansk F-16-kampfly styrter ned i Tyskland | Ingeniøren</v>
+      </c>
+      <c r="N211" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+      </c>
+      <c r="O211" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=kampfly</v>
+      </c>
+      <c r="P211" t="str">
+        <v/>
+      </c>
+      <c r="Q211" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R211" t="str">
+        <v/>
+      </c>
+      <c r="S211" t="str">
+        <v/>
+      </c>
+      <c r="T211" t="str">
+        <v/>
+      </c>
+      <c r="U211" t="str">
+        <v/>
+      </c>
+      <c r="V211" t="str">
+        <v/>
+      </c>
+      <c r="W211" t="str">
+        <v/>
+      </c>
+      <c r="X211" t="str">
+        <v/>
+      </c>
+      <c r="Y211" t="str">
+        <v/>
+      </c>
+      <c r="Z211" t="str">
+        <v/>
+      </c>
+      <c r="AA211" t="str">
+        <v/>
+      </c>
+      <c r="AB211" t="str">
+        <v/>
+      </c>
+      <c r="AC211" t="str">
+        <v/>
+      </c>
+      <c r="AD211" t="str">
+        <v/>
+      </c>
+      <c r="AE211" t="str">
+        <v/>
+      </c>
+      <c r="AF211" t="str">
+        <v/>
+      </c>
+      <c r="AG211" t="str">
+        <v/>
+      </c>
+      <c r="AH211" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH210"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH211"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "luftvåben" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH211"/>
+  <dimension ref="A1:AH212"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21213,9 +21213,113 @@
         <v/>
       </c>
     </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>1060b12b-42a0-4488-a6ad-b6520b2e5b0b</v>
+      </c>
+      <c r="B212" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="C212" t="str">
+        <v>luftvåben</v>
+      </c>
+      <c r="D212" t="str">
+        <v>luftvåben</v>
+      </c>
+      <c r="E212" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F212" t="str">
+        <v>et</v>
+      </c>
+      <c r="G212" t="str">
+        <v>..våbnet eller -et, -, ..våbnene Se bøjning i skema</v>
+      </c>
+      <c r="H212" t="str">
+        <v/>
+      </c>
+      <c r="I212" t="str">
+        <v>https://static.ordnet.dk/mp3/11031/11031142_1.mp3</v>
+      </c>
+      <c r="J212" t="str">
+        <v>den del af et lands militær som er udrustet til at føre krig ved hjælp af krigsfly, helikoptere, luftværnsraketter m.m.</v>
+      </c>
+      <c r="K212" t="str">
+        <v>Air Force</v>
+      </c>
+      <c r="L212" t="str">
+        <v>Et kampfly af typen F-16 fra det amerikanske luftvåben styrtede ned tirsdag eftermiddag tæt på Spangdahlem-luftbasen i det vestlige Tyskland. Det skriver mediet Deutsche Welle.</v>
+      </c>
+      <c r="M212" t="str">
+        <v>Pilot hoppede ud med katapult: Amerikansk F-16-kampfly styrter ned i Tyskland | Ingeniøren</v>
+      </c>
+      <c r="N212" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+      </c>
+      <c r="O212" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=luftv%C3%A5ben</v>
+      </c>
+      <c r="P212" t="str">
+        <v/>
+      </c>
+      <c r="Q212" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R212" t="str">
+        <v/>
+      </c>
+      <c r="S212" t="str">
+        <v/>
+      </c>
+      <c r="T212" t="str">
+        <v/>
+      </c>
+      <c r="U212" t="str">
+        <v/>
+      </c>
+      <c r="V212" t="str">
+        <v/>
+      </c>
+      <c r="W212" t="str">
+        <v/>
+      </c>
+      <c r="X212" t="str">
+        <v/>
+      </c>
+      <c r="Y212" t="str">
+        <v/>
+      </c>
+      <c r="Z212" t="str">
+        <v/>
+      </c>
+      <c r="AA212" t="str">
+        <v/>
+      </c>
+      <c r="AB212" t="str">
+        <v/>
+      </c>
+      <c r="AC212" t="str">
+        <v/>
+      </c>
+      <c r="AD212" t="str">
+        <v/>
+      </c>
+      <c r="AE212" t="str">
+        <v/>
+      </c>
+      <c r="AF212" t="str">
+        <v/>
+      </c>
+      <c r="AG212" t="str">
+        <v/>
+      </c>
+      <c r="AH212" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH211"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH212"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "jagereskadre" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH212"/>
+  <dimension ref="A1:AH213"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21317,9 +21317,113 @@
         <v/>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>e7892f22-ea70-49ce-a698-c7635960ec5b</v>
+      </c>
+      <c r="B213" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="C213" t="str">
+        <v>jagereskadre</v>
+      </c>
+      <c r="D213" t="str">
+        <v>jagereskadre</v>
+      </c>
+      <c r="E213" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F213" t="str">
+        <v>en</v>
+      </c>
+      <c r="G213" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H213" t="str">
+        <v/>
+      </c>
+      <c r="I213" t="str">
+        <v/>
+      </c>
+      <c r="J213" t="str">
+        <v>sammensat af jageres + kadre</v>
+      </c>
+      <c r="K213" t="str">
+        <v>Fighter squadron</v>
+      </c>
+      <c r="L213" t="str">
+        <v>Det drejer sig om et F-16 Fighting Falcon-fly fra det amerikanske luftvåbens 52. jagereskadre. Efter at være undsluppet ved hjælp af flyets katapultsystem blev piloten transporteret til lægebehandling.</v>
+      </c>
+      <c r="M213" t="str">
+        <v>Pilot hoppede ud med katapult: Amerikansk F-16-kampfly styrter ned i Tyskland | Ingeniøren</v>
+      </c>
+      <c r="N213" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+      </c>
+      <c r="O213" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=jagereskadre</v>
+      </c>
+      <c r="P213" t="str">
+        <v/>
+      </c>
+      <c r="Q213" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R213" t="str">
+        <v/>
+      </c>
+      <c r="S213" t="str">
+        <v/>
+      </c>
+      <c r="T213" t="str">
+        <v/>
+      </c>
+      <c r="U213" t="str">
+        <v/>
+      </c>
+      <c r="V213" t="str">
+        <v/>
+      </c>
+      <c r="W213" t="str">
+        <v/>
+      </c>
+      <c r="X213" t="str">
+        <v/>
+      </c>
+      <c r="Y213" t="str">
+        <v/>
+      </c>
+      <c r="Z213" t="str">
+        <v/>
+      </c>
+      <c r="AA213" t="str">
+        <v/>
+      </c>
+      <c r="AB213" t="str">
+        <v/>
+      </c>
+      <c r="AC213" t="str">
+        <v/>
+      </c>
+      <c r="AD213" t="str">
+        <v/>
+      </c>
+      <c r="AE213" t="str">
+        <v/>
+      </c>
+      <c r="AF213" t="str">
+        <v/>
+      </c>
+      <c r="AG213" t="str">
+        <v/>
+      </c>
+      <c r="AH213" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH212"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH213"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "behandling" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH213"/>
+  <dimension ref="A1:AH214"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21421,9 +21421,113 @@
         <v/>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>8b92b412-4d76-4407-bba7-c9e3fdf6c5b3</v>
+      </c>
+      <c r="B214" t="str">
+        <v>2026-09-23</v>
+      </c>
+      <c r="C214" t="str">
+        <v>behandling</v>
+      </c>
+      <c r="D214" t="str">
+        <v>behandling</v>
+      </c>
+      <c r="E214" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F214" t="str">
+        <v>en</v>
+      </c>
+      <c r="G214" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H214" t="str">
+        <v>[beˈhanˀleŋ]</v>
+      </c>
+      <c r="I214" t="str">
+        <v>https://static.ordnet.dk/mp3/11003/11003905_1.mp3</v>
+      </c>
+      <c r="J214" t="str">
+        <v>foranstaltning som man iværksætter for at helbrede nogen eller afhjælpe et helbredsmæssigt problem</v>
+      </c>
+      <c r="K214" t="str">
+        <v>treatment</v>
+      </c>
+      <c r="L214" t="str">
+        <v>Det drejer sig om et F-16 Fighting Falcon-fly fra det amerikanske luftvåbens 52. jagereskadre. Efter at være undsluppet ved hjælp af flyets katapultsystem blev piloten transporteret til lægebehandling.</v>
+      </c>
+      <c r="M214" t="str">
+        <v>Pilot hoppede ud med katapult: Amerikansk F-16-kampfly styrter ned i Tyskland | Ingeniøren</v>
+      </c>
+      <c r="N214" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+      </c>
+      <c r="O214" t="str">
+        <v>https://ing.dk/artikel/pilot-hoppede-ud-med-katapult-amerikansk-f-16-kampfly-styrter-ned-i-tyskland?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=behandling</v>
+      </c>
+      <c r="P214" t="str">
+        <v/>
+      </c>
+      <c r="Q214" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R214" t="str">
+        <v/>
+      </c>
+      <c r="S214" t="str">
+        <v/>
+      </c>
+      <c r="T214" t="str">
+        <v/>
+      </c>
+      <c r="U214" t="str">
+        <v/>
+      </c>
+      <c r="V214" t="str">
+        <v/>
+      </c>
+      <c r="W214" t="str">
+        <v/>
+      </c>
+      <c r="X214" t="str">
+        <v/>
+      </c>
+      <c r="Y214" t="str">
+        <v/>
+      </c>
+      <c r="Z214" t="str">
+        <v/>
+      </c>
+      <c r="AA214" t="str">
+        <v/>
+      </c>
+      <c r="AB214" t="str">
+        <v/>
+      </c>
+      <c r="AC214" t="str">
+        <v/>
+      </c>
+      <c r="AD214" t="str">
+        <v/>
+      </c>
+      <c r="AE214" t="str">
+        <v/>
+      </c>
+      <c r="AF214" t="str">
+        <v/>
+      </c>
+      <c r="AG214" t="str">
+        <v/>
+      </c>
+      <c r="AH214" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH213"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH214"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Vådt" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH214"/>
+  <dimension ref="A1:AH215"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21525,9 +21525,113 @@
         <v/>
       </c>
     </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>5eb6d04d-675f-4b05-af4d-a58828db5289</v>
+      </c>
+      <c r="B215" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Vådt</v>
+      </c>
+      <c r="D215" t="str">
+        <v>våd</v>
+      </c>
+      <c r="E215" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F215" t="str">
+        <v>et</v>
+      </c>
+      <c r="G215" t="str">
+        <v>-t, -e -ere, -est</v>
+      </c>
+      <c r="H215" t="str">
+        <v>[ˈvɔˀð]</v>
+      </c>
+      <c r="I215" t="str">
+        <v>https://static.ordnet.dk/mp3/12007/12007623_1.mp3</v>
+      </c>
+      <c r="J215" t="str">
+        <v>helt dækket eller fuld af vand, sved eller anden væske</v>
+      </c>
+      <c r="K215" t="str">
+        <v>Wet</v>
+      </c>
+      <c r="L215" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme</v>
+      </c>
+      <c r="M215" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N215" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O215" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=V%C3%A5dt</v>
+      </c>
+      <c r="P215" t="str">
+        <v/>
+      </c>
+      <c r="Q215" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R215" t="str">
+        <v/>
+      </c>
+      <c r="S215" t="str">
+        <v/>
+      </c>
+      <c r="T215" t="str">
+        <v/>
+      </c>
+      <c r="U215" t="str">
+        <v/>
+      </c>
+      <c r="V215" t="str">
+        <v/>
+      </c>
+      <c r="W215" t="str">
+        <v/>
+      </c>
+      <c r="X215" t="str">
+        <v/>
+      </c>
+      <c r="Y215" t="str">
+        <v/>
+      </c>
+      <c r="Z215" t="str">
+        <v/>
+      </c>
+      <c r="AA215" t="str">
+        <v/>
+      </c>
+      <c r="AB215" t="str">
+        <v/>
+      </c>
+      <c r="AC215" t="str">
+        <v/>
+      </c>
+      <c r="AD215" t="str">
+        <v/>
+      </c>
+      <c r="AE215" t="str">
+        <v/>
+      </c>
+      <c r="AF215" t="str">
+        <v/>
+      </c>
+      <c r="AG215" t="str">
+        <v/>
+      </c>
+      <c r="AH215" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH214"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH215"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "forsyning" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH215"/>
+  <dimension ref="A1:AH216"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21629,9 +21629,113 @@
         <v/>
       </c>
     </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>11193e61-65ef-4892-a213-3e9f64b7429f</v>
+      </c>
+      <c r="B216" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C216" t="str">
+        <v>forsyning</v>
+      </c>
+      <c r="D216" t="str">
+        <v>forsyning</v>
+      </c>
+      <c r="E216" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F216" t="str">
+        <v>en</v>
+      </c>
+      <c r="G216" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H216" t="str">
+        <v>[fʌˈsyˀneŋ]</v>
+      </c>
+      <c r="I216" t="str">
+        <v>https://static.ordnet.dk/mp3/11015/11015271_1.mp3</v>
+      </c>
+      <c r="J216" t="str">
+        <v>varer og andre fornødenheder der er til rådighed</v>
+      </c>
+      <c r="K216" t="str">
+        <v>supply</v>
+      </c>
+      <c r="L216" t="str">
+        <v>I Silkeborg har den lokale forsyning skåret en fjerdedel af deres CO2-udledning fra fjernvarmen til de 55.000 kunder med en utraditionel combo af tekniske løsninger, der med deres egne ord udnytter nogle »helt særlige synergier«, skriver Ingeniørens GridTech.</v>
+      </c>
+      <c r="M216" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N216" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O216" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=forsyning</v>
+      </c>
+      <c r="P216" t="str">
+        <v/>
+      </c>
+      <c r="Q216" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R216" t="str">
+        <v/>
+      </c>
+      <c r="S216" t="str">
+        <v/>
+      </c>
+      <c r="T216" t="str">
+        <v/>
+      </c>
+      <c r="U216" t="str">
+        <v/>
+      </c>
+      <c r="V216" t="str">
+        <v/>
+      </c>
+      <c r="W216" t="str">
+        <v/>
+      </c>
+      <c r="X216" t="str">
+        <v/>
+      </c>
+      <c r="Y216" t="str">
+        <v/>
+      </c>
+      <c r="Z216" t="str">
+        <v/>
+      </c>
+      <c r="AA216" t="str">
+        <v/>
+      </c>
+      <c r="AB216" t="str">
+        <v/>
+      </c>
+      <c r="AC216" t="str">
+        <v/>
+      </c>
+      <c r="AD216" t="str">
+        <v/>
+      </c>
+      <c r="AE216" t="str">
+        <v/>
+      </c>
+      <c r="AF216" t="str">
+        <v/>
+      </c>
+      <c r="AG216" t="str">
+        <v/>
+      </c>
+      <c r="AH216" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH215"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH216"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "skåret" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH216"/>
+  <dimension ref="A1:AH217"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21733,9 +21733,113 @@
         <v/>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>4c0b50a3-8bbc-457f-8820-5b0e4b8c7688</v>
+      </c>
+      <c r="B217" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C217" t="str">
+        <v>skåret</v>
+      </c>
+      <c r="D217" t="str">
+        <v>skåret</v>
+      </c>
+      <c r="E217" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F217" t="str">
+        <v/>
+      </c>
+      <c r="G217" t="str">
+        <v>-, skårede</v>
+      </c>
+      <c r="H217" t="str">
+        <v>[ˈsgɒːɒð]</v>
+      </c>
+      <c r="I217" t="str">
+        <v>https://static.ordnet.dk/mp3/11047/11047533_1.mp3</v>
+      </c>
+      <c r="J217" t="str">
+        <v>som der er slået skår af om genstand af glas, porcelæn el.lign.</v>
+      </c>
+      <c r="K217" t="str">
+        <v>cut</v>
+      </c>
+      <c r="L217" t="str">
+        <v>I Silkeborg har den lokale forsyning skåret en fjerdedel af deres CO2-udledning fra fjernvarmen til de 55.000 kunder med en utraditionel combo af tekniske løsninger, der med deres egne ord udnytter nogle »helt særlige synergier«, skriver Ingeniørens GridTech.</v>
+      </c>
+      <c r="M217" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N217" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O217" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=sk%C3%A5ret</v>
+      </c>
+      <c r="P217" t="str">
+        <v/>
+      </c>
+      <c r="Q217" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R217" t="str">
+        <v/>
+      </c>
+      <c r="S217" t="str">
+        <v/>
+      </c>
+      <c r="T217" t="str">
+        <v/>
+      </c>
+      <c r="U217" t="str">
+        <v/>
+      </c>
+      <c r="V217" t="str">
+        <v/>
+      </c>
+      <c r="W217" t="str">
+        <v/>
+      </c>
+      <c r="X217" t="str">
+        <v/>
+      </c>
+      <c r="Y217" t="str">
+        <v/>
+      </c>
+      <c r="Z217" t="str">
+        <v/>
+      </c>
+      <c r="AA217" t="str">
+        <v/>
+      </c>
+      <c r="AB217" t="str">
+        <v/>
+      </c>
+      <c r="AC217" t="str">
+        <v/>
+      </c>
+      <c r="AD217" t="str">
+        <v/>
+      </c>
+      <c r="AE217" t="str">
+        <v/>
+      </c>
+      <c r="AF217" t="str">
+        <v/>
+      </c>
+      <c r="AG217" t="str">
+        <v/>
+      </c>
+      <c r="AH217" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH216"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH217"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "fjerdedel" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH217"/>
+  <dimension ref="A1:AH218"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21837,9 +21837,113 @@
         <v/>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>babe3736-ea26-40ca-85fa-90383361c580</v>
+      </c>
+      <c r="B218" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C218" t="str">
+        <v>fjerdedel</v>
+      </c>
+      <c r="D218" t="str">
+        <v>fjerdedel</v>
+      </c>
+      <c r="E218" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F218" t="str">
+        <v>en</v>
+      </c>
+      <c r="G218" t="str">
+        <v>-en, -e, -ene</v>
+      </c>
+      <c r="H218" t="str">
+        <v>[ˈfjεːʌˌdeˀl]</v>
+      </c>
+      <c r="I218" t="str">
+        <v>https://static.ordnet.dk/mp3/11013/11013337_1.mp3</v>
+      </c>
+      <c r="J218" t="str">
+        <v>hver af fire lige store dele som en helhed kan deles op i fx tre fjerdedele = 3/4</v>
+      </c>
+      <c r="K218" t="str">
+        <v>quarter</v>
+      </c>
+      <c r="L218" t="str">
+        <v>I Silkeborg har den lokale forsyning skåret en fjerdedel af deres CO2-udledning fra fjernvarmen til de 55.000 kunder med en utraditionel combo af tekniske løsninger, der med deres egne ord udnytter nogle »helt særlige synergier«, skriver Ingeniørens GridTech.</v>
+      </c>
+      <c r="M218" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N218" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O218" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=fjerdedel</v>
+      </c>
+      <c r="P218" t="str">
+        <v/>
+      </c>
+      <c r="Q218" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R218" t="str">
+        <v/>
+      </c>
+      <c r="S218" t="str">
+        <v/>
+      </c>
+      <c r="T218" t="str">
+        <v/>
+      </c>
+      <c r="U218" t="str">
+        <v/>
+      </c>
+      <c r="V218" t="str">
+        <v/>
+      </c>
+      <c r="W218" t="str">
+        <v/>
+      </c>
+      <c r="X218" t="str">
+        <v/>
+      </c>
+      <c r="Y218" t="str">
+        <v/>
+      </c>
+      <c r="Z218" t="str">
+        <v/>
+      </c>
+      <c r="AA218" t="str">
+        <v/>
+      </c>
+      <c r="AB218" t="str">
+        <v/>
+      </c>
+      <c r="AC218" t="str">
+        <v/>
+      </c>
+      <c r="AD218" t="str">
+        <v/>
+      </c>
+      <c r="AE218" t="str">
+        <v/>
+      </c>
+      <c r="AF218" t="str">
+        <v/>
+      </c>
+      <c r="AG218" t="str">
+        <v/>
+      </c>
+      <c r="AH218" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH217"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH218"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "udledning" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH218"/>
+  <dimension ref="A1:AH219"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21941,9 +21941,113 @@
         <v/>
       </c>
     </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>407994d3-b085-4722-85a3-a2c3538657e6</v>
+      </c>
+      <c r="B219" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C219" t="str">
+        <v>udledning</v>
+      </c>
+      <c r="D219" t="str">
+        <v>udledning</v>
+      </c>
+      <c r="E219" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F219" t="str">
+        <v>en</v>
+      </c>
+      <c r="G219" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H219" t="str">
+        <v>[-ˌleðˀneŋ]</v>
+      </c>
+      <c r="I219" t="str">
+        <v>https://static.ordnet.dk/mp3/12003/12003939_1.mp3</v>
+      </c>
+      <c r="J219" t="str">
+        <v>det at lede noget, som regel spildevand, ud i naturen</v>
+      </c>
+      <c r="K219" t="str">
+        <v>discharge</v>
+      </c>
+      <c r="L219" t="str">
+        <v>I Silkeborg har den lokale forsyning skåret en fjerdedel af deres CO2-udledning fra fjernvarmen til de 55.000 kunder med en utraditionel combo af tekniske løsninger, der med deres egne ord udnytter nogle »helt særlige synergier«, skriver Ingeniørens GridTech.</v>
+      </c>
+      <c r="M219" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N219" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O219" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=udledning</v>
+      </c>
+      <c r="P219" t="str">
+        <v/>
+      </c>
+      <c r="Q219" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R219" t="str">
+        <v/>
+      </c>
+      <c r="S219" t="str">
+        <v/>
+      </c>
+      <c r="T219" t="str">
+        <v/>
+      </c>
+      <c r="U219" t="str">
+        <v/>
+      </c>
+      <c r="V219" t="str">
+        <v/>
+      </c>
+      <c r="W219" t="str">
+        <v/>
+      </c>
+      <c r="X219" t="str">
+        <v/>
+      </c>
+      <c r="Y219" t="str">
+        <v/>
+      </c>
+      <c r="Z219" t="str">
+        <v/>
+      </c>
+      <c r="AA219" t="str">
+        <v/>
+      </c>
+      <c r="AB219" t="str">
+        <v/>
+      </c>
+      <c r="AC219" t="str">
+        <v/>
+      </c>
+      <c r="AD219" t="str">
+        <v/>
+      </c>
+      <c r="AE219" t="str">
+        <v/>
+      </c>
+      <c r="AF219" t="str">
+        <v/>
+      </c>
+      <c r="AG219" t="str">
+        <v/>
+      </c>
+      <c r="AH219" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH218"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH219"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "fjernvarmen" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH219"/>
+  <dimension ref="A1:AH220"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22045,9 +22045,113 @@
         <v/>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>b9ed5fb3-a85a-4d3d-83dd-2e60f88c26fd</v>
+      </c>
+      <c r="B220" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C220" t="str">
+        <v>fjernvarmen</v>
+      </c>
+      <c r="D220" t="str">
+        <v>fjernvarme</v>
+      </c>
+      <c r="E220" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F220" t="str">
+        <v>en</v>
+      </c>
+      <c r="G220" t="str">
+        <v>-n</v>
+      </c>
+      <c r="H220" t="str">
+        <v/>
+      </c>
+      <c r="I220" t="str">
+        <v>https://static.ordnet.dk/mp3/11013/11013373_1.mp3</v>
+      </c>
+      <c r="J220" t="str">
+        <v>forsyning med varme i form af varmt vand der i et net af nedgravede rør føres rundt til de tilsluttede huse og tilbage til varmeværket</v>
+      </c>
+      <c r="K220" t="str">
+        <v>the district heating</v>
+      </c>
+      <c r="L220" t="str">
+        <v>I Silkeborg har den lokale forsyning skåret en fjerdedel af deres CO2-udledning fra fjernvarmen til de 55.000 kunder med en utraditionel combo af tekniske løsninger, der med deres egne ord udnytter nogle »helt særlige synergier«, skriver Ingeniørens GridTech.</v>
+      </c>
+      <c r="M220" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N220" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O220" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=fjernvarmen</v>
+      </c>
+      <c r="P220" t="str">
+        <v/>
+      </c>
+      <c r="Q220" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R220" t="str">
+        <v/>
+      </c>
+      <c r="S220" t="str">
+        <v/>
+      </c>
+      <c r="T220" t="str">
+        <v/>
+      </c>
+      <c r="U220" t="str">
+        <v/>
+      </c>
+      <c r="V220" t="str">
+        <v/>
+      </c>
+      <c r="W220" t="str">
+        <v/>
+      </c>
+      <c r="X220" t="str">
+        <v/>
+      </c>
+      <c r="Y220" t="str">
+        <v/>
+      </c>
+      <c r="Z220" t="str">
+        <v/>
+      </c>
+      <c r="AA220" t="str">
+        <v/>
+      </c>
+      <c r="AB220" t="str">
+        <v/>
+      </c>
+      <c r="AC220" t="str">
+        <v/>
+      </c>
+      <c r="AD220" t="str">
+        <v/>
+      </c>
+      <c r="AE220" t="str">
+        <v/>
+      </c>
+      <c r="AF220" t="str">
+        <v/>
+      </c>
+      <c r="AG220" t="str">
+        <v/>
+      </c>
+      <c r="AH220" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH219"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH220"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "udnytter" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH220"/>
+  <dimension ref="A1:AH221"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22149,9 +22149,113 @@
         <v/>
       </c>
     </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>4344de3c-f8c8-4af4-a375-3215c480db7b</v>
+      </c>
+      <c r="B221" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C221" t="str">
+        <v>udnytter</v>
+      </c>
+      <c r="D221" t="str">
+        <v>udnytte</v>
+      </c>
+      <c r="E221" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F221" t="str">
+        <v/>
+      </c>
+      <c r="G221" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H221" t="str">
+        <v/>
+      </c>
+      <c r="I221" t="str">
+        <v>https://static.ordnet.dk/mp3/12004/12004007_1.mp3</v>
+      </c>
+      <c r="J221" t="str">
+        <v>gøre brug af en eksisterende resurse til et hensigtsmæssigt formål</v>
+      </c>
+      <c r="K221" t="str">
+        <v>Utilizes</v>
+      </c>
+      <c r="L221" t="str">
+        <v>I Silkeborg har den lokale forsyning skåret en fjerdedel af deres CO2-udledning fra fjernvarmen til de 55.000 kunder med en utraditionel combo af tekniske løsninger, der med deres egne ord udnytter nogle »helt særlige synergier«, skriver Ingeniørens GridTech.</v>
+      </c>
+      <c r="M221" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N221" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O221" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=udnytter</v>
+      </c>
+      <c r="P221" t="str">
+        <v/>
+      </c>
+      <c r="Q221" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R221" t="str">
+        <v/>
+      </c>
+      <c r="S221" t="str">
+        <v/>
+      </c>
+      <c r="T221" t="str">
+        <v/>
+      </c>
+      <c r="U221" t="str">
+        <v/>
+      </c>
+      <c r="V221" t="str">
+        <v/>
+      </c>
+      <c r="W221" t="str">
+        <v/>
+      </c>
+      <c r="X221" t="str">
+        <v/>
+      </c>
+      <c r="Y221" t="str">
+        <v/>
+      </c>
+      <c r="Z221" t="str">
+        <v/>
+      </c>
+      <c r="AA221" t="str">
+        <v/>
+      </c>
+      <c r="AB221" t="str">
+        <v/>
+      </c>
+      <c r="AC221" t="str">
+        <v/>
+      </c>
+      <c r="AD221" t="str">
+        <v/>
+      </c>
+      <c r="AE221" t="str">
+        <v/>
+      </c>
+      <c r="AF221" t="str">
+        <v/>
+      </c>
+      <c r="AG221" t="str">
+        <v/>
+      </c>
+      <c r="AH221" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH220"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH221"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "udforsket" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH221"/>
+  <dimension ref="A1:AH222"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22253,9 +22253,113 @@
         <v/>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>bd699994-ee45-4598-a7c4-4899c6758ddc</v>
+      </c>
+      <c r="B222" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C222" t="str">
+        <v>udforsket</v>
+      </c>
+      <c r="D222" t="str">
+        <v>udforske</v>
+      </c>
+      <c r="E222" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F222" t="str">
+        <v/>
+      </c>
+      <c r="G222" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H222" t="str">
+        <v>[-ˌfɒːsgə]</v>
+      </c>
+      <c r="I222" t="str">
+        <v>https://static.ordnet.dk/mp3/12003/12003812_1.mp3</v>
+      </c>
+      <c r="J222" t="str">
+        <v>undersøge eller skaffe sig oplysninger om ved hjælp af videnskabelige metoder</v>
+      </c>
+      <c r="K222" t="str">
+        <v>explored</v>
+      </c>
+      <c r="L222" t="str">
+        <v>Hvor de fleste forsyninger driver hhv. deres varmepumper og biomasseanlæg i separate systemer, har man hos Silkeborg Forsyning udforsket en ny vej og bundet deres termiske kredsløb tæt sammen.</v>
+      </c>
+      <c r="M222" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N222" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O222" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=udforsket</v>
+      </c>
+      <c r="P222" t="str">
+        <v/>
+      </c>
+      <c r="Q222" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R222" t="str">
+        <v/>
+      </c>
+      <c r="S222" t="str">
+        <v/>
+      </c>
+      <c r="T222" t="str">
+        <v/>
+      </c>
+      <c r="U222" t="str">
+        <v/>
+      </c>
+      <c r="V222" t="str">
+        <v/>
+      </c>
+      <c r="W222" t="str">
+        <v/>
+      </c>
+      <c r="X222" t="str">
+        <v/>
+      </c>
+      <c r="Y222" t="str">
+        <v/>
+      </c>
+      <c r="Z222" t="str">
+        <v/>
+      </c>
+      <c r="AA222" t="str">
+        <v/>
+      </c>
+      <c r="AB222" t="str">
+        <v/>
+      </c>
+      <c r="AC222" t="str">
+        <v/>
+      </c>
+      <c r="AD222" t="str">
+        <v/>
+      </c>
+      <c r="AE222" t="str">
+        <v/>
+      </c>
+      <c r="AF222" t="str">
+        <v/>
+      </c>
+      <c r="AG222" t="str">
+        <v/>
+      </c>
+      <c r="AH222" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH221"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH222"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kredsløb" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH222"/>
+  <dimension ref="A1:AH223"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22357,9 +22357,113 @@
         <v/>
       </c>
     </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>57229d86-107e-4ee1-8ea2-e6c572fdffad</v>
+      </c>
+      <c r="B223" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C223" t="str">
+        <v>kredsløb</v>
+      </c>
+      <c r="D223" t="str">
+        <v>kredsløb</v>
+      </c>
+      <c r="E223" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F223" t="str">
+        <v>et</v>
+      </c>
+      <c r="G223" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H223" t="str">
+        <v>[ˈkʁεːsˌløˀb]</v>
+      </c>
+      <c r="I223" t="str">
+        <v>https://static.ordnet.dk/mp3/11028/11028005_1.mp3</v>
+      </c>
+      <c r="J223" t="str">
+        <v>gentagen og ubrudt bevægelse i en kredsformet bane omkring et centrum</v>
+      </c>
+      <c r="K223" t="str">
+        <v>circuit</v>
+      </c>
+      <c r="L223" t="str">
+        <v>Hvor de fleste forsyninger driver hhv. deres varmepumper og biomasseanlæg i separate systemer, har man hos Silkeborg Forsyning udforsket en ny vej og bundet deres termiske kredsløb tæt sammen.</v>
+      </c>
+      <c r="M223" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N223" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O223" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=kredsl%C3%B8b</v>
+      </c>
+      <c r="P223" t="str">
+        <v/>
+      </c>
+      <c r="Q223" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R223" t="str">
+        <v/>
+      </c>
+      <c r="S223" t="str">
+        <v/>
+      </c>
+      <c r="T223" t="str">
+        <v/>
+      </c>
+      <c r="U223" t="str">
+        <v/>
+      </c>
+      <c r="V223" t="str">
+        <v/>
+      </c>
+      <c r="W223" t="str">
+        <v/>
+      </c>
+      <c r="X223" t="str">
+        <v/>
+      </c>
+      <c r="Y223" t="str">
+        <v/>
+      </c>
+      <c r="Z223" t="str">
+        <v/>
+      </c>
+      <c r="AA223" t="str">
+        <v/>
+      </c>
+      <c r="AB223" t="str">
+        <v/>
+      </c>
+      <c r="AC223" t="str">
+        <v/>
+      </c>
+      <c r="AD223" t="str">
+        <v/>
+      </c>
+      <c r="AE223" t="str">
+        <v/>
+      </c>
+      <c r="AF223" t="str">
+        <v/>
+      </c>
+      <c r="AG223" t="str">
+        <v/>
+      </c>
+      <c r="AH223" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH222"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH223"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "termiske" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH223"/>
+  <dimension ref="A1:AH224"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22461,9 +22461,113 @@
         <v/>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>9cdc3d1a-205a-470f-a5df-83d8daf346a0</v>
+      </c>
+      <c r="B224" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C224" t="str">
+        <v>termiske</v>
+      </c>
+      <c r="D224" t="str">
+        <v>termisk</v>
+      </c>
+      <c r="E224" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F224" t="str">
+        <v/>
+      </c>
+      <c r="G224" t="str">
+        <v>-, -e</v>
+      </c>
+      <c r="H224" t="str">
+        <v>[ˈtæɐ̯ˀmisg]</v>
+      </c>
+      <c r="I224" t="str">
+        <v>https://static.ordnet.dk/mp3/12000/12000753_1.mp3</v>
+      </c>
+      <c r="J224" t="str">
+        <v>vedrørende varme eller temperatur</v>
+      </c>
+      <c r="K224" t="str">
+        <v>Thermal</v>
+      </c>
+      <c r="L224" t="str">
+        <v>Hvor de fleste forsyninger driver hhv. deres varmepumper og biomasseanlæg i separate systemer, har man hos Silkeborg Forsyning udforsket en ny vej og bundet deres termiske kredsløb tæt sammen.</v>
+      </c>
+      <c r="M224" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N224" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O224" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=termiske</v>
+      </c>
+      <c r="P224" t="str">
+        <v/>
+      </c>
+      <c r="Q224" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R224" t="str">
+        <v/>
+      </c>
+      <c r="S224" t="str">
+        <v/>
+      </c>
+      <c r="T224" t="str">
+        <v/>
+      </c>
+      <c r="U224" t="str">
+        <v/>
+      </c>
+      <c r="V224" t="str">
+        <v/>
+      </c>
+      <c r="W224" t="str">
+        <v/>
+      </c>
+      <c r="X224" t="str">
+        <v/>
+      </c>
+      <c r="Y224" t="str">
+        <v/>
+      </c>
+      <c r="Z224" t="str">
+        <v/>
+      </c>
+      <c r="AA224" t="str">
+        <v/>
+      </c>
+      <c r="AB224" t="str">
+        <v/>
+      </c>
+      <c r="AC224" t="str">
+        <v/>
+      </c>
+      <c r="AD224" t="str">
+        <v/>
+      </c>
+      <c r="AE224" t="str">
+        <v/>
+      </c>
+      <c r="AF224" t="str">
+        <v/>
+      </c>
+      <c r="AG224" t="str">
+        <v/>
+      </c>
+      <c r="AH224" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH223"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH224"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "etableret" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH224"/>
+  <dimension ref="A1:AH225"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22565,9 +22565,113 @@
         <v/>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>92f243fc-f401-4dab-9967-93c8f07ab5af</v>
+      </c>
+      <c r="B225" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C225" t="str">
+        <v>etableret</v>
+      </c>
+      <c r="D225" t="str">
+        <v>etableret</v>
+      </c>
+      <c r="E225" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F225" t="str">
+        <v/>
+      </c>
+      <c r="G225" t="str">
+        <v>-, etablerede</v>
+      </c>
+      <c r="H225" t="str">
+        <v>[etaˈbleˀʌð]</v>
+      </c>
+      <c r="I225" t="str">
+        <v>https://static.ordnet.dk/mp3/11011/11011824_1.mp3</v>
+      </c>
+      <c r="J225" t="str">
+        <v>som har eksisteret eller været i brug gennem længere tid og derfor er almindeligt anerkendt og accepteret fx om en institution eller en retning inden for kunst eller videnskab</v>
+      </c>
+      <c r="K225" t="str">
+        <v>established</v>
+      </c>
+      <c r="L225" t="str">
+        <v>Tricket er en dedikeret 6 MW koldtvandskreds, som ingeniørerne har etableret direkte på den store luft-til-vand-varmepumpe. I stedet for at lade køleeffekten gå til spilde, cirkuleres det kolde vand internt på matriklen og ledes blandt andet ind i 'røgvaskemaskinen' – skrubberen – på forsyningens nye biomasseforgasningsanlæg.</v>
+      </c>
+      <c r="M225" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N225" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O225" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=etableret</v>
+      </c>
+      <c r="P225" t="str">
+        <v/>
+      </c>
+      <c r="Q225" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R225" t="str">
+        <v/>
+      </c>
+      <c r="S225" t="str">
+        <v/>
+      </c>
+      <c r="T225" t="str">
+        <v/>
+      </c>
+      <c r="U225" t="str">
+        <v/>
+      </c>
+      <c r="V225" t="str">
+        <v/>
+      </c>
+      <c r="W225" t="str">
+        <v/>
+      </c>
+      <c r="X225" t="str">
+        <v/>
+      </c>
+      <c r="Y225" t="str">
+        <v/>
+      </c>
+      <c r="Z225" t="str">
+        <v/>
+      </c>
+      <c r="AA225" t="str">
+        <v/>
+      </c>
+      <c r="AB225" t="str">
+        <v/>
+      </c>
+      <c r="AC225" t="str">
+        <v/>
+      </c>
+      <c r="AD225" t="str">
+        <v/>
+      </c>
+      <c r="AE225" t="str">
+        <v/>
+      </c>
+      <c r="AF225" t="str">
+        <v/>
+      </c>
+      <c r="AG225" t="str">
+        <v/>
+      </c>
+      <c r="AH225" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH224"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH225"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "lade" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH225"/>
+  <dimension ref="A1:AH226"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22669,9 +22669,113 @@
         <v/>
       </c>
     </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>56a91f71-2209-4f81-9825-fd5fa3418342</v>
+      </c>
+      <c r="B226" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C226" t="str">
+        <v>lade</v>
+      </c>
+      <c r="D226" t="str">
+        <v>lade</v>
+      </c>
+      <c r="E226" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F226" t="str">
+        <v>en</v>
+      </c>
+      <c r="G226" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H226" t="str">
+        <v>[ˈlæːðə]</v>
+      </c>
+      <c r="I226" t="str">
+        <v>https://static.ordnet.dk/mp3/11029/11029410_1.mp3</v>
+      </c>
+      <c r="J226" t="str">
+        <v>stor landbrugsbygning beregnet til opbevaring af afgrøder, foder, redskaber osv.</v>
+      </c>
+      <c r="K226" t="str">
+        <v>let</v>
+      </c>
+      <c r="L226" t="str">
+        <v>Tricket er en dedikeret 6 MW koldtvandskreds, som ingeniørerne har etableret direkte på den store luft-til-vand-varmepumpe. I stedet for at lade køleeffekten gå til spilde, cirkuleres det kolde vand internt på matriklen og ledes blandt andet ind i 'røgvaskemaskinen' – skrubberen – på forsyningens nye biomasseforgasningsanlæg.</v>
+      </c>
+      <c r="M226" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N226" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O226" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=lade</v>
+      </c>
+      <c r="P226" t="str">
+        <v/>
+      </c>
+      <c r="Q226" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R226" t="str">
+        <v/>
+      </c>
+      <c r="S226" t="str">
+        <v/>
+      </c>
+      <c r="T226" t="str">
+        <v/>
+      </c>
+      <c r="U226" t="str">
+        <v/>
+      </c>
+      <c r="V226" t="str">
+        <v/>
+      </c>
+      <c r="W226" t="str">
+        <v/>
+      </c>
+      <c r="X226" t="str">
+        <v/>
+      </c>
+      <c r="Y226" t="str">
+        <v/>
+      </c>
+      <c r="Z226" t="str">
+        <v/>
+      </c>
+      <c r="AA226" t="str">
+        <v/>
+      </c>
+      <c r="AB226" t="str">
+        <v/>
+      </c>
+      <c r="AC226" t="str">
+        <v/>
+      </c>
+      <c r="AD226" t="str">
+        <v/>
+      </c>
+      <c r="AE226" t="str">
+        <v/>
+      </c>
+      <c r="AF226" t="str">
+        <v/>
+      </c>
+      <c r="AG226" t="str">
+        <v/>
+      </c>
+      <c r="AH226" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH225"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH226"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "køleeffekten" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH226"/>
+  <dimension ref="A1:AH227"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22773,9 +22773,113 @@
         <v/>
       </c>
     </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>f823b7a7-a88b-4608-b219-e37552feab2b</v>
+      </c>
+      <c r="B227" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C227" t="str">
+        <v>køleeffekten</v>
+      </c>
+      <c r="D227" t="str">
+        <v>køleeffekt</v>
+      </c>
+      <c r="E227" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F227" t="str">
+        <v>en</v>
+      </c>
+      <c r="G227" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H227" t="str">
+        <v/>
+      </c>
+      <c r="I227" t="str">
+        <v/>
+      </c>
+      <c r="J227" t="str">
+        <v>sammensat af køle + effekt</v>
+      </c>
+      <c r="K227" t="str">
+        <v>the cooling effect</v>
+      </c>
+      <c r="L227" t="str">
+        <v>Tricket er en dedikeret 6 MW koldtvandskreds, som ingeniørerne har etableret direkte på den store luft-til-vand-varmepumpe. I stedet for at lade køleeffekten gå til spilde, cirkuleres det kolde vand internt på matriklen og ledes blandt andet ind i 'røgvaskemaskinen' – skrubberen – på forsyningens nye biomasseforgasningsanlæg.</v>
+      </c>
+      <c r="M227" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N227" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O227" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=k%C3%B8leeffekten</v>
+      </c>
+      <c r="P227" t="str">
+        <v/>
+      </c>
+      <c r="Q227" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R227" t="str">
+        <v/>
+      </c>
+      <c r="S227" t="str">
+        <v/>
+      </c>
+      <c r="T227" t="str">
+        <v/>
+      </c>
+      <c r="U227" t="str">
+        <v/>
+      </c>
+      <c r="V227" t="str">
+        <v/>
+      </c>
+      <c r="W227" t="str">
+        <v/>
+      </c>
+      <c r="X227" t="str">
+        <v/>
+      </c>
+      <c r="Y227" t="str">
+        <v/>
+      </c>
+      <c r="Z227" t="str">
+        <v/>
+      </c>
+      <c r="AA227" t="str">
+        <v/>
+      </c>
+      <c r="AB227" t="str">
+        <v/>
+      </c>
+      <c r="AC227" t="str">
+        <v/>
+      </c>
+      <c r="AD227" t="str">
+        <v/>
+      </c>
+      <c r="AE227" t="str">
+        <v/>
+      </c>
+      <c r="AF227" t="str">
+        <v/>
+      </c>
+      <c r="AG227" t="str">
+        <v/>
+      </c>
+      <c r="AH227" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH226"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH227"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "spilde" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH227"/>
+  <dimension ref="A1:AH228"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22877,9 +22877,113 @@
         <v/>
       </c>
     </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>fbbad778-6001-437e-b195-23d44383023f</v>
+      </c>
+      <c r="B228" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C228" t="str">
+        <v>spilde</v>
+      </c>
+      <c r="D228" t="str">
+        <v>spilde</v>
+      </c>
+      <c r="E228" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F228" t="str">
+        <v>et</v>
+      </c>
+      <c r="G228" t="str">
+        <v/>
+      </c>
+      <c r="H228" t="str">
+        <v>[ˈsbilə]</v>
+      </c>
+      <c r="I228" t="str">
+        <v>https://static.ordnet.dk/mp3/11049/11049132_1.mp3</v>
+      </c>
+      <c r="J228" t="str">
+        <v>kun i udtrykket:</v>
+      </c>
+      <c r="K228" t="str">
+        <v>spill</v>
+      </c>
+      <c r="L228" t="str">
+        <v>Tricket er en dedikeret 6 MW koldtvandskreds, som ingeniørerne har etableret direkte på den store luft-til-vand-varmepumpe. I stedet for at lade køleeffekten gå til spilde, cirkuleres det kolde vand internt på matriklen og ledes blandt andet ind i 'røgvaskemaskinen' – skrubberen – på forsyningens nye biomasseforgasningsanlæg.</v>
+      </c>
+      <c r="M228" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N228" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O228" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=spilde</v>
+      </c>
+      <c r="P228" t="str">
+        <v/>
+      </c>
+      <c r="Q228" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R228" t="str">
+        <v/>
+      </c>
+      <c r="S228" t="str">
+        <v/>
+      </c>
+      <c r="T228" t="str">
+        <v/>
+      </c>
+      <c r="U228" t="str">
+        <v/>
+      </c>
+      <c r="V228" t="str">
+        <v/>
+      </c>
+      <c r="W228" t="str">
+        <v/>
+      </c>
+      <c r="X228" t="str">
+        <v/>
+      </c>
+      <c r="Y228" t="str">
+        <v/>
+      </c>
+      <c r="Z228" t="str">
+        <v/>
+      </c>
+      <c r="AA228" t="str">
+        <v/>
+      </c>
+      <c r="AB228" t="str">
+        <v/>
+      </c>
+      <c r="AC228" t="str">
+        <v/>
+      </c>
+      <c r="AD228" t="str">
+        <v/>
+      </c>
+      <c r="AE228" t="str">
+        <v/>
+      </c>
+      <c r="AF228" t="str">
+        <v/>
+      </c>
+      <c r="AG228" t="str">
+        <v/>
+      </c>
+      <c r="AH228" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH227"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH228"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "indbyrdes" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH228"/>
+  <dimension ref="A1:AH229"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22981,9 +22981,113 @@
         <v/>
       </c>
     </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>50347e64-88bf-4841-a8c0-ad5096f8d827</v>
+      </c>
+      <c r="B229" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C229" t="str">
+        <v>indbyrdes</v>
+      </c>
+      <c r="D229" t="str">
+        <v>indbyrdes</v>
+      </c>
+      <c r="E229" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F229" t="str">
+        <v/>
+      </c>
+      <c r="G229" t="str">
+        <v>-, -</v>
+      </c>
+      <c r="H229" t="str">
+        <v>[-ˌbyɐ̯ˀdəs]</v>
+      </c>
+      <c r="I229" t="str">
+        <v>https://static.ordnet.dk/mp3/11023/11023152_1.mp3</v>
+      </c>
+      <c r="J229" t="str">
+        <v>som foregår eller eksisterer gensidigt mellem to eller flere parter, begreber eller ting</v>
+      </c>
+      <c r="K229" t="str">
+        <v>mutual</v>
+      </c>
+      <c r="L229" t="str">
+        <v>»Vi har skabt nogle helt særlige synergier ved at udnytte anlæggenes indbyrdes placering. Varmepumpen bruges ikke kun til at producere varme til nettet; vi udnytter også den kulde, som processen genererer, til at øge effektiviteten på vores biomasseværk,« forklarer Mogens Lyhne, projektchef for Varme i Silkeborg Forsyning.</v>
+      </c>
+      <c r="M229" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N229" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O229" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=indbyrdes</v>
+      </c>
+      <c r="P229" t="str">
+        <v/>
+      </c>
+      <c r="Q229" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R229" t="str">
+        <v/>
+      </c>
+      <c r="S229" t="str">
+        <v/>
+      </c>
+      <c r="T229" t="str">
+        <v/>
+      </c>
+      <c r="U229" t="str">
+        <v/>
+      </c>
+      <c r="V229" t="str">
+        <v/>
+      </c>
+      <c r="W229" t="str">
+        <v/>
+      </c>
+      <c r="X229" t="str">
+        <v/>
+      </c>
+      <c r="Y229" t="str">
+        <v/>
+      </c>
+      <c r="Z229" t="str">
+        <v/>
+      </c>
+      <c r="AA229" t="str">
+        <v/>
+      </c>
+      <c r="AB229" t="str">
+        <v/>
+      </c>
+      <c r="AC229" t="str">
+        <v/>
+      </c>
+      <c r="AD229" t="str">
+        <v/>
+      </c>
+      <c r="AE229" t="str">
+        <v/>
+      </c>
+      <c r="AF229" t="str">
+        <v/>
+      </c>
+      <c r="AG229" t="str">
+        <v/>
+      </c>
+      <c r="AH229" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH228"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH229"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "placering" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH229"/>
+  <dimension ref="A1:AH230"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -23085,9 +23085,113 @@
         <v/>
       </c>
     </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>52919c58-ad37-4ed0-903d-524f16d94f5b</v>
+      </c>
+      <c r="B230" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="C230" t="str">
+        <v>placering</v>
+      </c>
+      <c r="D230" t="str">
+        <v>placering</v>
+      </c>
+      <c r="E230" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F230" t="str">
+        <v>en</v>
+      </c>
+      <c r="G230" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H230" t="str">
+        <v>[plaˈseˀɐ̯eŋ]</v>
+      </c>
+      <c r="I230" t="str">
+        <v>https://static.ordnet.dk/mp3/11039/11039919_1.mp3</v>
+      </c>
+      <c r="J230" t="str">
+        <v>sted hvor noget eller nogen befinder sig eller kommer til at befinde sig</v>
+      </c>
+      <c r="K230" t="str">
+        <v>Location</v>
+      </c>
+      <c r="L230" t="str">
+        <v>»Vi har skabt nogle helt særlige synergier ved at udnytte anlæggenes indbyrdes placering. Varmepumpen bruges ikke kun til at producere varme til nettet; vi udnytter også den kulde, som processen genererer, til at øge effektiviteten på vores biomasseværk,« forklarer Mogens Lyhne, projektchef for Varme i Silkeborg Forsyning.</v>
+      </c>
+      <c r="M230" t="str">
+        <v>Jyde-trick hiver ekstra energi ud: Vådt haveaffald forvandles til varme | Ingeniøren</v>
+      </c>
+      <c r="N230" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme</v>
+      </c>
+      <c r="O230" t="str">
+        <v>https://ing.dk/artikel/jyde-trick-hiver-ekstra-energi-ud-vaadt-haveaffald-forvandles-til-varme#:~:text=placering</v>
+      </c>
+      <c r="P230" t="str">
+        <v/>
+      </c>
+      <c r="Q230" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R230" t="str">
+        <v/>
+      </c>
+      <c r="S230" t="str">
+        <v/>
+      </c>
+      <c r="T230" t="str">
+        <v/>
+      </c>
+      <c r="U230" t="str">
+        <v/>
+      </c>
+      <c r="V230" t="str">
+        <v/>
+      </c>
+      <c r="W230" t="str">
+        <v/>
+      </c>
+      <c r="X230" t="str">
+        <v/>
+      </c>
+      <c r="Y230" t="str">
+        <v/>
+      </c>
+      <c r="Z230" t="str">
+        <v/>
+      </c>
+      <c r="AA230" t="str">
+        <v/>
+      </c>
+      <c r="AB230" t="str">
+        <v/>
+      </c>
+      <c r="AC230" t="str">
+        <v/>
+      </c>
+      <c r="AD230" t="str">
+        <v/>
+      </c>
+      <c r="AE230" t="str">
+        <v/>
+      </c>
+      <c r="AF230" t="str">
+        <v/>
+      </c>
+      <c r="AG230" t="str">
+        <v/>
+      </c>
+      <c r="AH230" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH229"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH230"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "opnåede" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH230"/>
+  <dimension ref="A1:AH231"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -23189,9 +23189,113 @@
         <v/>
       </c>
     </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>2888be8f-56aa-40c8-8911-4880dc03f229</v>
+      </c>
+      <c r="B231" t="str">
+        <v>2026-10-06</v>
+      </c>
+      <c r="C231" t="str">
+        <v>opnåede</v>
+      </c>
+      <c r="D231" t="str">
+        <v>opnå</v>
+      </c>
+      <c r="E231" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F231" t="str">
+        <v/>
+      </c>
+      <c r="G231" t="str">
+        <v>-r, -ede, -et</v>
+      </c>
+      <c r="H231" t="str">
+        <v>[ˈʌbˌnɔˀ]</v>
+      </c>
+      <c r="I231" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037592_1.mp3</v>
+      </c>
+      <c r="J231" t="str">
+        <v>få, skaffe eller sikre sig, tilfældigt eller som resultat af en indsats</v>
+      </c>
+      <c r="K231" t="str">
+        <v>achieved</v>
+      </c>
+      <c r="L231" t="str">
+        <v>Hvad er din højest opnåede uddannelse?</v>
+      </c>
+      <c r="M231" t="str">
+        <v>Audience - DK - PC - TPC</v>
+      </c>
+      <c r="N231" t="str">
+        <v>https://gasurvey.gemius.com/recruiting/index.php</v>
+      </c>
+      <c r="O231" t="str">
+        <v>https://gasurvey.gemius.com/recruiting/index.php#:~:text=opn%C3%A5ede</v>
+      </c>
+      <c r="P231" t="str">
+        <v/>
+      </c>
+      <c r="Q231" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R231" t="str">
+        <v/>
+      </c>
+      <c r="S231" t="str">
+        <v/>
+      </c>
+      <c r="T231" t="str">
+        <v/>
+      </c>
+      <c r="U231" t="str">
+        <v/>
+      </c>
+      <c r="V231" t="str">
+        <v/>
+      </c>
+      <c r="W231" t="str">
+        <v/>
+      </c>
+      <c r="X231" t="str">
+        <v/>
+      </c>
+      <c r="Y231" t="str">
+        <v/>
+      </c>
+      <c r="Z231" t="str">
+        <v/>
+      </c>
+      <c r="AA231" t="str">
+        <v/>
+      </c>
+      <c r="AB231" t="str">
+        <v/>
+      </c>
+      <c r="AC231" t="str">
+        <v/>
+      </c>
+      <c r="AD231" t="str">
+        <v/>
+      </c>
+      <c r="AE231" t="str">
+        <v/>
+      </c>
+      <c r="AF231" t="str">
+        <v/>
+      </c>
+      <c r="AG231" t="str">
+        <v/>
+      </c>
+      <c r="AH231" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH230"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH231"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Angiv" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH231"/>
+  <dimension ref="A1:AH232"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -23293,9 +23293,113 @@
         <v/>
       </c>
     </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>e95c02ed-1f15-420f-b6e3-3f876eb75588</v>
+      </c>
+      <c r="B232" t="str">
+        <v>2026-10-06</v>
+      </c>
+      <c r="C232" t="str">
+        <v>Angiv</v>
+      </c>
+      <c r="D232" t="str">
+        <v>angive</v>
+      </c>
+      <c r="E232" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F232" t="str">
+        <v/>
+      </c>
+      <c r="G232" t="str">
+        <v>-r, angav, -t</v>
+      </c>
+      <c r="H232" t="str">
+        <v>[ˈanˌgiˀ]</v>
+      </c>
+      <c r="I232" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001769_1.mp3</v>
+      </c>
+      <c r="J232" t="str">
+        <v>oplyse eller meddele skriftligt eller mundtligt</v>
+      </c>
+      <c r="K232" t="str">
+        <v>Indicate</v>
+      </c>
+      <c r="L232" t="str">
+        <v>Angiv din boligform?</v>
+      </c>
+      <c r="M232" t="str">
+        <v>Audience - DK - PC - TPC</v>
+      </c>
+      <c r="N232" t="str">
+        <v>https://gasurvey.gemius.com/recruiting/index.php</v>
+      </c>
+      <c r="O232" t="str">
+        <v>https://gasurvey.gemius.com/recruiting/index.php#:~:text=Angiv</v>
+      </c>
+      <c r="P232" t="str">
+        <v/>
+      </c>
+      <c r="Q232" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R232" t="str">
+        <v/>
+      </c>
+      <c r="S232" t="str">
+        <v/>
+      </c>
+      <c r="T232" t="str">
+        <v/>
+      </c>
+      <c r="U232" t="str">
+        <v/>
+      </c>
+      <c r="V232" t="str">
+        <v/>
+      </c>
+      <c r="W232" t="str">
+        <v/>
+      </c>
+      <c r="X232" t="str">
+        <v/>
+      </c>
+      <c r="Y232" t="str">
+        <v/>
+      </c>
+      <c r="Z232" t="str">
+        <v/>
+      </c>
+      <c r="AA232" t="str">
+        <v/>
+      </c>
+      <c r="AB232" t="str">
+        <v/>
+      </c>
+      <c r="AC232" t="str">
+        <v/>
+      </c>
+      <c r="AD232" t="str">
+        <v/>
+      </c>
+      <c r="AE232" t="str">
+        <v/>
+      </c>
+      <c r="AF232" t="str">
+        <v/>
+      </c>
+      <c r="AG232" t="str">
+        <v/>
+      </c>
+      <c r="AH232" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH231"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH232"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bedes" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH232"/>
+  <dimension ref="A1:AH233"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -23397,9 +23397,113 @@
         <v/>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>9f2d1252-f3c4-4542-95c5-edabab6a93df</v>
+      </c>
+      <c r="B233" t="str">
+        <v>2026-10-06</v>
+      </c>
+      <c r="C233" t="str">
+        <v>bedes</v>
+      </c>
+      <c r="D233" t="str">
+        <v>bed</v>
+      </c>
+      <c r="E233" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F233" t="str">
+        <v>et</v>
+      </c>
+      <c r="G233" t="str">
+        <v>-et, -e, -ene</v>
+      </c>
+      <c r="H233" t="str">
+        <v>[ˈbeð]</v>
+      </c>
+      <c r="I233" t="str">
+        <v>https://static.ordnet.dk/mp3/11003/11003712_1.mp3</v>
+      </c>
+      <c r="J233" t="str">
+        <v>mindre, afgrænset område i en have hvor der vokser planter ofte en bestemt slags, fx roser, jordbær eller kål</v>
+      </c>
+      <c r="K233" t="str">
+        <v>please</v>
+      </c>
+      <c r="L233" t="str">
+        <v>Nedenfor bedes du anføre hvilke områder du er interesseret i (angiv gerne flere):</v>
+      </c>
+      <c r="M233" t="str">
+        <v>Audience - DK - PC - TPC</v>
+      </c>
+      <c r="N233" t="str">
+        <v>https://gasurvey.gemius.com/recruiting/index.php</v>
+      </c>
+      <c r="O233" t="str">
+        <v>https://gasurvey.gemius.com/recruiting/index.php#:~:text=bedes</v>
+      </c>
+      <c r="P233" t="str">
+        <v/>
+      </c>
+      <c r="Q233" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R233" t="str">
+        <v/>
+      </c>
+      <c r="S233" t="str">
+        <v/>
+      </c>
+      <c r="T233" t="str">
+        <v/>
+      </c>
+      <c r="U233" t="str">
+        <v/>
+      </c>
+      <c r="V233" t="str">
+        <v/>
+      </c>
+      <c r="W233" t="str">
+        <v/>
+      </c>
+      <c r="X233" t="str">
+        <v/>
+      </c>
+      <c r="Y233" t="str">
+        <v/>
+      </c>
+      <c r="Z233" t="str">
+        <v/>
+      </c>
+      <c r="AA233" t="str">
+        <v/>
+      </c>
+      <c r="AB233" t="str">
+        <v/>
+      </c>
+      <c r="AC233" t="str">
+        <v/>
+      </c>
+      <c r="AD233" t="str">
+        <v/>
+      </c>
+      <c r="AE233" t="str">
+        <v/>
+      </c>
+      <c r="AF233" t="str">
+        <v/>
+      </c>
+      <c r="AG233" t="str">
+        <v/>
+      </c>
+      <c r="AH233" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH232"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH233"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "anføre" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH233"/>
+  <dimension ref="A1:AH234"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -23501,9 +23501,113 @@
         <v/>
       </c>
     </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>f1cba31a-e269-47ef-9b9c-12ff5aadd72b</v>
+      </c>
+      <c r="B234" t="str">
+        <v>2026-10-06</v>
+      </c>
+      <c r="C234" t="str">
+        <v>anføre</v>
+      </c>
+      <c r="D234" t="str">
+        <v>anføre</v>
+      </c>
+      <c r="E234" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F234" t="str">
+        <v/>
+      </c>
+      <c r="G234" t="str">
+        <v>-r, anførte, anført</v>
+      </c>
+      <c r="H234" t="str">
+        <v>[ˈanˌføˀʌ]</v>
+      </c>
+      <c r="I234" t="str">
+        <v>https://static.ordnet.dk/mp3/11001/11001753_1.mp3</v>
+      </c>
+      <c r="J234" t="str">
+        <v>give en skriftlig oplysning, fx på et skema eller i en redegørelse</v>
+      </c>
+      <c r="K234" t="str">
+        <v>state</v>
+      </c>
+      <c r="L234" t="str">
+        <v>Nedenfor bedes du anføre hvilke områder du er interesseret i (angiv gerne flere):</v>
+      </c>
+      <c r="M234" t="str">
+        <v>Audience - DK - PC - TPC</v>
+      </c>
+      <c r="N234" t="str">
+        <v>https://gasurvey.gemius.com/recruiting/index.php</v>
+      </c>
+      <c r="O234" t="str">
+        <v>https://gasurvey.gemius.com/recruiting/index.php#:~:text=anf%C3%B8re</v>
+      </c>
+      <c r="P234" t="str">
+        <v/>
+      </c>
+      <c r="Q234" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R234" t="str">
+        <v/>
+      </c>
+      <c r="S234" t="str">
+        <v/>
+      </c>
+      <c r="T234" t="str">
+        <v/>
+      </c>
+      <c r="U234" t="str">
+        <v/>
+      </c>
+      <c r="V234" t="str">
+        <v/>
+      </c>
+      <c r="W234" t="str">
+        <v/>
+      </c>
+      <c r="X234" t="str">
+        <v/>
+      </c>
+      <c r="Y234" t="str">
+        <v/>
+      </c>
+      <c r="Z234" t="str">
+        <v/>
+      </c>
+      <c r="AA234" t="str">
+        <v/>
+      </c>
+      <c r="AB234" t="str">
+        <v/>
+      </c>
+      <c r="AC234" t="str">
+        <v/>
+      </c>
+      <c r="AD234" t="str">
+        <v/>
+      </c>
+      <c r="AE234" t="str">
+        <v/>
+      </c>
+      <c r="AF234" t="str">
+        <v/>
+      </c>
+      <c r="AG234" t="str">
+        <v/>
+      </c>
+      <c r="AH234" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH233"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH234"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "mængde" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH234"/>
+  <dimension ref="A1:AH235"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -23605,9 +23605,113 @@
         <v/>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>b1db9c05-3471-4808-94b5-f5e5647076a5</v>
+      </c>
+      <c r="B235" t="str">
+        <v>2026-10-06</v>
+      </c>
+      <c r="C235" t="str">
+        <v>mængde</v>
+      </c>
+      <c r="D235" t="str">
+        <v>mængde</v>
+      </c>
+      <c r="E235" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F235" t="str">
+        <v>en</v>
+      </c>
+      <c r="G235" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H235" t="str">
+        <v>[ˈmεŋˀdə]</v>
+      </c>
+      <c r="I235" t="str">
+        <v>https://static.ordnet.dk/mp3/11034/11034942_1.mp3</v>
+      </c>
+      <c r="J235" t="str">
+        <v>størrelsen af en tællelig eller målelig forekomst af et materiale eller af enheder, individer, fænomener el.lign.</v>
+      </c>
+      <c r="K235" t="str">
+        <v>quantity</v>
+      </c>
+      <c r="L235" t="str">
+        <v>Siden download af den store mængde data er foregået i september, så tyder meget på, at det først er gået op for specialisterne i Forsknings-, Uddannelse- og Digitaliseringsministeriet, at næsten alle danskeres oplysninger er blevet lænset, efter det er sket.</v>
+      </c>
+      <c r="M235" t="str">
+        <v>Erfaren hacker undrer sig: Her burde alarmen være gået i 10 dages CPR-tyveri | Ingeniøren</v>
+      </c>
+      <c r="N235" t="str">
+        <v>https://ing.dk/artikel/erfaren-hacker-undrer-sig-her-burde-alarmen-vaere-gaaet-i-10-dages-cpr-tyveri</v>
+      </c>
+      <c r="O235" t="str">
+        <v>https://ing.dk/artikel/erfaren-hacker-undrer-sig-her-burde-alarmen-vaere-gaaet-i-10-dages-cpr-tyveri#:~:text=m%C3%A6ngde</v>
+      </c>
+      <c r="P235" t="str">
+        <v/>
+      </c>
+      <c r="Q235" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R235" t="str">
+        <v/>
+      </c>
+      <c r="S235" t="str">
+        <v/>
+      </c>
+      <c r="T235" t="str">
+        <v/>
+      </c>
+      <c r="U235" t="str">
+        <v/>
+      </c>
+      <c r="V235" t="str">
+        <v/>
+      </c>
+      <c r="W235" t="str">
+        <v/>
+      </c>
+      <c r="X235" t="str">
+        <v/>
+      </c>
+      <c r="Y235" t="str">
+        <v/>
+      </c>
+      <c r="Z235" t="str">
+        <v/>
+      </c>
+      <c r="AA235" t="str">
+        <v/>
+      </c>
+      <c r="AB235" t="str">
+        <v/>
+      </c>
+      <c r="AC235" t="str">
+        <v/>
+      </c>
+      <c r="AD235" t="str">
+        <v/>
+      </c>
+      <c r="AE235" t="str">
+        <v/>
+      </c>
+      <c r="AF235" t="str">
+        <v/>
+      </c>
+      <c r="AG235" t="str">
+        <v/>
+      </c>
+      <c r="AH235" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH234"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH235"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "enestående" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH235"/>
+  <dimension ref="A1:AH236"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -23709,9 +23709,113 @@
         <v/>
       </c>
     </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>95e84f47-2dd7-4437-aa17-b812f864f98f</v>
+      </c>
+      <c r="B236" t="str">
+        <v>2026-10-12</v>
+      </c>
+      <c r="C236" t="str">
+        <v>enestående</v>
+      </c>
+      <c r="D236" t="str">
+        <v>enestående</v>
+      </c>
+      <c r="E236" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F236" t="str">
+        <v/>
+      </c>
+      <c r="G236" t="str">
+        <v>-, -</v>
+      </c>
+      <c r="H236" t="str">
+        <v>[-ˌsdɔˀənə]</v>
+      </c>
+      <c r="I236" t="str">
+        <v>https://static.ordnet.dk/mp3/11011/11011389_1.mp3</v>
+      </c>
+      <c r="J236" t="str">
+        <v>som i en eller anden henseende er i en klasse for sig i forhold til det meste andet af samme art; som er særlig god, smuk, fordelagtig osv.</v>
+      </c>
+      <c r="K236" t="str">
+        <v>unique</v>
+      </c>
+      <c r="L236" t="str">
+        <v>Lurpak® er globalt anerkendt for enestående kvalitet og smag. Et ry, der er opbygget og fortsat styrkes, gennem hårdt arbejde, dedikation og sans for detaljen.</v>
+      </c>
+      <c r="M236" t="str">
+        <v>Vi fejrer 125 år med Lurpak® | Lurpak®</v>
+      </c>
+      <c r="N236" t="str">
+        <v>https://www.lurpak.com/da/vores-historie/?utm_source=fbig&amp;utm_medium=paid&amp;utm_campaign=26_dk_lurp_125anniversary_41_44_reach%3A3300101308_organic-boost&amp;utm_content=dk_lurp_125anniversary_price_vid31+_4x5_fbig_da_b9cc60&amp;utm_id=120251060710430429&amp;utm_term=120251060727290429&amp;fbclid=IwY2xjawU5nsVleHRuA2FlbQEwAHBkb2YBYWRpZAGrN7PgWKhdYnJpZBEwdHp1cVJLdXJrc2w1TmM5RHNydGMGYXBwX2lkEDIyMjAzOTE3ODgyMDA4OTIAAR6hSFwEorfWq7-fUHZs_z1s1ydyprPUuSau1MqxfsNJ6bRdVTiwkCUvyrEv5A_aem_l9OGtSb8-zhk4MsUGbViIA&amp;campaign_id=120251060710430429&amp;ad_id=120251060727320429</v>
+      </c>
+      <c r="O236" t="str">
+        <v>https://www.lurpak.com/da/vores-historie/?utm_source=fbig&amp;utm_medium=paid&amp;utm_campaign=26_dk_lurp_125anniversary_41_44_reach%3A3300101308_organic-boost&amp;utm_content=dk_lurp_125anniversary_price_vid31+_4x5_fbig_da_b9cc60&amp;utm_id=120251060710430429&amp;utm_term=120251060727290429&amp;fbclid=IwY2xjawU5nsVleHRuA2FlbQEwAHBkb2YBYWRpZAGrN7PgWKhdYnJpZBEwdHp1cVJLdXJrc2w1TmM5RHNydGMGYXBwX2lkEDIyMjAzOTE3ODgyMDA4OTIAAR6hSFwEorfWq7-fUHZs_z1s1ydyprPUuSau1MqxfsNJ6bRdVTiwkCUvyrEv5A_aem_l9OGtSb8-zhk4MsUGbViIA&amp;campaign_id=120251060710430429&amp;ad_id=120251060727320429#:~:text=enest%C3%A5ende</v>
+      </c>
+      <c r="P236" t="str">
+        <v/>
+      </c>
+      <c r="Q236" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R236" t="str">
+        <v/>
+      </c>
+      <c r="S236" t="str">
+        <v/>
+      </c>
+      <c r="T236" t="str">
+        <v/>
+      </c>
+      <c r="U236" t="str">
+        <v/>
+      </c>
+      <c r="V236" t="str">
+        <v/>
+      </c>
+      <c r="W236" t="str">
+        <v/>
+      </c>
+      <c r="X236" t="str">
+        <v/>
+      </c>
+      <c r="Y236" t="str">
+        <v/>
+      </c>
+      <c r="Z236" t="str">
+        <v/>
+      </c>
+      <c r="AA236" t="str">
+        <v/>
+      </c>
+      <c r="AB236" t="str">
+        <v/>
+      </c>
+      <c r="AC236" t="str">
+        <v/>
+      </c>
+      <c r="AD236" t="str">
+        <v/>
+      </c>
+      <c r="AE236" t="str">
+        <v/>
+      </c>
+      <c r="AF236" t="str">
+        <v/>
+      </c>
+      <c r="AG236" t="str">
+        <v/>
+      </c>
+      <c r="AH236" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH235"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH236"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Samfund" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH236"/>
+  <dimension ref="A1:AH237"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -23813,9 +23813,113 @@
         <v/>
       </c>
     </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>c9ff0bda-4dd7-46f1-84a4-7d195d9e5f81</v>
+      </c>
+      <c r="B237" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="C237" t="str">
+        <v>Samfund</v>
+      </c>
+      <c r="D237" t="str">
+        <v>samfund</v>
+      </c>
+      <c r="E237" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F237" t="str">
+        <v>et</v>
+      </c>
+      <c r="G237" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H237" t="str">
+        <v>[ˈsɑmˌfɔnˀ]</v>
+      </c>
+      <c r="I237" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044593_1.mp3</v>
+      </c>
+      <c r="J237" t="str">
+        <v>større gruppe mennesker der bor inden for et afgrænset område og er knyttet sammen gennem organiseret samvær og indbyrdes afhængighed, evt. også af tilhørsforholdet til en bestemt nationalstat</v>
+      </c>
+      <c r="K237" t="str">
+        <v>Society</v>
+      </c>
+      <c r="L237" t="str">
+        <v>Sex og Samfund</v>
+      </c>
+      <c r="M237" t="str">
+        <v>(1) Facebook</v>
+      </c>
+      <c r="N237" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O237" t="str">
+        <v>https://www.facebook.com/#:~:text=Samfund</v>
+      </c>
+      <c r="P237" t="str">
+        <v/>
+      </c>
+      <c r="Q237" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R237" t="str">
+        <v/>
+      </c>
+      <c r="S237" t="str">
+        <v/>
+      </c>
+      <c r="T237" t="str">
+        <v/>
+      </c>
+      <c r="U237" t="str">
+        <v/>
+      </c>
+      <c r="V237" t="str">
+        <v/>
+      </c>
+      <c r="W237" t="str">
+        <v/>
+      </c>
+      <c r="X237" t="str">
+        <v/>
+      </c>
+      <c r="Y237" t="str">
+        <v/>
+      </c>
+      <c r="Z237" t="str">
+        <v/>
+      </c>
+      <c r="AA237" t="str">
+        <v/>
+      </c>
+      <c r="AB237" t="str">
+        <v/>
+      </c>
+      <c r="AC237" t="str">
+        <v/>
+      </c>
+      <c r="AD237" t="str">
+        <v/>
+      </c>
+      <c r="AE237" t="str">
+        <v/>
+      </c>
+      <c r="AF237" t="str">
+        <v/>
+      </c>
+      <c r="AG237" t="str">
+        <v/>
+      </c>
+      <c r="AH237" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH236"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH237"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "uenig" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH237"/>
+  <dimension ref="A1:AH238"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -23917,9 +23917,113 @@
         <v/>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>a7ca019e-179d-4bff-8590-6783864a01cf</v>
+      </c>
+      <c r="B238" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="C238" t="str">
+        <v>uenig</v>
+      </c>
+      <c r="D238" t="str">
+        <v>uenig</v>
+      </c>
+      <c r="E238" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F238" t="str">
+        <v/>
+      </c>
+      <c r="G238" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H238" t="str">
+        <v>[uˈeˀni]</v>
+      </c>
+      <c r="I238" t="str">
+        <v>https://static.ordnet.dk/mp3/12004/12004347_1.mp3</v>
+      </c>
+      <c r="J238" t="str">
+        <v>af indbyrdes forskellige, uforenelige opfattelser eller holdninger</v>
+      </c>
+      <c r="K238" t="str">
+        <v>Disagree</v>
+      </c>
+      <c r="L238" t="str">
+        <v>Forsker uenig med Musk: Indsamling af beskidte bleer er en god idé</v>
+      </c>
+      <c r="M238" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N238" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O238" t="str">
+        <v>https://ing.dk/#:~:text=uenig</v>
+      </c>
+      <c r="P238" t="str">
+        <v/>
+      </c>
+      <c r="Q238" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R238" t="str">
+        <v/>
+      </c>
+      <c r="S238" t="str">
+        <v/>
+      </c>
+      <c r="T238" t="str">
+        <v/>
+      </c>
+      <c r="U238" t="str">
+        <v/>
+      </c>
+      <c r="V238" t="str">
+        <v/>
+      </c>
+      <c r="W238" t="str">
+        <v/>
+      </c>
+      <c r="X238" t="str">
+        <v/>
+      </c>
+      <c r="Y238" t="str">
+        <v/>
+      </c>
+      <c r="Z238" t="str">
+        <v/>
+      </c>
+      <c r="AA238" t="str">
+        <v/>
+      </c>
+      <c r="AB238" t="str">
+        <v/>
+      </c>
+      <c r="AC238" t="str">
+        <v/>
+      </c>
+      <c r="AD238" t="str">
+        <v/>
+      </c>
+      <c r="AE238" t="str">
+        <v/>
+      </c>
+      <c r="AF238" t="str">
+        <v/>
+      </c>
+      <c r="AG238" t="str">
+        <v/>
+      </c>
+      <c r="AH238" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH237"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH238"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Indsamling" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH238"/>
+  <dimension ref="A1:AH239"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24021,9 +24021,113 @@
         <v/>
       </c>
     </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>62c54028-7164-4e58-be3c-c2938393fe4f</v>
+      </c>
+      <c r="B239" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="C239" t="str">
+        <v>Indsamling</v>
+      </c>
+      <c r="D239" t="str">
+        <v>indsamling</v>
+      </c>
+      <c r="E239" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F239" t="str">
+        <v>en</v>
+      </c>
+      <c r="G239" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H239" t="str">
+        <v>[-ˌsɑmˀleŋ]</v>
+      </c>
+      <c r="I239" t="str">
+        <v>https://static.ordnet.dk/mp3/11023/11023504_1.mp3</v>
+      </c>
+      <c r="J239" t="str">
+        <v>det at samle noget ind systematisk fx affald (til genbrug) eller oplysninger</v>
+      </c>
+      <c r="K239" t="str">
+        <v>Gathering</v>
+      </c>
+      <c r="L239" t="str">
+        <v>Forsker uenig med Musk: Indsamling af beskidte bleer er en god idé</v>
+      </c>
+      <c r="M239" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N239" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O239" t="str">
+        <v>https://ing.dk/#:~:text=Indsamling</v>
+      </c>
+      <c r="P239" t="str">
+        <v/>
+      </c>
+      <c r="Q239" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R239" t="str">
+        <v/>
+      </c>
+      <c r="S239" t="str">
+        <v/>
+      </c>
+      <c r="T239" t="str">
+        <v/>
+      </c>
+      <c r="U239" t="str">
+        <v/>
+      </c>
+      <c r="V239" t="str">
+        <v/>
+      </c>
+      <c r="W239" t="str">
+        <v/>
+      </c>
+      <c r="X239" t="str">
+        <v/>
+      </c>
+      <c r="Y239" t="str">
+        <v/>
+      </c>
+      <c r="Z239" t="str">
+        <v/>
+      </c>
+      <c r="AA239" t="str">
+        <v/>
+      </c>
+      <c r="AB239" t="str">
+        <v/>
+      </c>
+      <c r="AC239" t="str">
+        <v/>
+      </c>
+      <c r="AD239" t="str">
+        <v/>
+      </c>
+      <c r="AE239" t="str">
+        <v/>
+      </c>
+      <c r="AF239" t="str">
+        <v/>
+      </c>
+      <c r="AG239" t="str">
+        <v/>
+      </c>
+      <c r="AH239" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH238"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH239"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "beskidte" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH239"/>
+  <dimension ref="A1:AH240"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24125,9 +24125,113 @@
         <v/>
       </c>
     </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>88a1e010-34ac-444c-b5bc-288ea467451e</v>
+      </c>
+      <c r="B240" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="C240" t="str">
+        <v>beskidte</v>
+      </c>
+      <c r="D240" t="str">
+        <v>beskidt</v>
+      </c>
+      <c r="E240" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F240" t="str">
+        <v/>
+      </c>
+      <c r="G240" t="str">
+        <v>-, -e</v>
+      </c>
+      <c r="H240" t="str">
+        <v>[beˈsgid]</v>
+      </c>
+      <c r="I240" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004225_1.mp3</v>
+      </c>
+      <c r="J240" t="str">
+        <v>dækket af eller blandet med snavs; ikke helt ren</v>
+      </c>
+      <c r="K240" t="str">
+        <v>dirty</v>
+      </c>
+      <c r="L240" t="str">
+        <v>Forsker uenig med Musk: Indsamling af beskidte bleer er en god idé</v>
+      </c>
+      <c r="M240" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N240" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O240" t="str">
+        <v>https://ing.dk/#:~:text=beskidte</v>
+      </c>
+      <c r="P240" t="str">
+        <v/>
+      </c>
+      <c r="Q240" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R240" t="str">
+        <v/>
+      </c>
+      <c r="S240" t="str">
+        <v/>
+      </c>
+      <c r="T240" t="str">
+        <v/>
+      </c>
+      <c r="U240" t="str">
+        <v/>
+      </c>
+      <c r="V240" t="str">
+        <v/>
+      </c>
+      <c r="W240" t="str">
+        <v/>
+      </c>
+      <c r="X240" t="str">
+        <v/>
+      </c>
+      <c r="Y240" t="str">
+        <v/>
+      </c>
+      <c r="Z240" t="str">
+        <v/>
+      </c>
+      <c r="AA240" t="str">
+        <v/>
+      </c>
+      <c r="AB240" t="str">
+        <v/>
+      </c>
+      <c r="AC240" t="str">
+        <v/>
+      </c>
+      <c r="AD240" t="str">
+        <v/>
+      </c>
+      <c r="AE240" t="str">
+        <v/>
+      </c>
+      <c r="AF240" t="str">
+        <v/>
+      </c>
+      <c r="AG240" t="str">
+        <v/>
+      </c>
+      <c r="AH240" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH239"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH240"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bleer" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH240"/>
+  <dimension ref="A1:AH241"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24229,9 +24229,113 @@
         <v/>
       </c>
     </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>5951eda1-ee22-46a2-b005-c41edbb4ec65</v>
+      </c>
+      <c r="B241" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="C241" t="str">
+        <v>bleer</v>
+      </c>
+      <c r="D241" t="str">
+        <v>ble</v>
+      </c>
+      <c r="E241" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F241" t="str">
+        <v>en</v>
+      </c>
+      <c r="G241" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H241" t="str">
+        <v>[ˈbleˀ]</v>
+      </c>
+      <c r="I241" t="str">
+        <v>https://static.ordnet.dk/mp3/11005/11005063_1.mp3</v>
+      </c>
+      <c r="J241" t="str">
+        <v>stykke tykt papirmateriale eller ufarvet bomuldsstof til at fæstne om numsen (på småbørn) for at opsuge urin og afføring også om tilsvarende genstand til syge eller svagelige</v>
+      </c>
+      <c r="K241" t="str">
+        <v>Diapers</v>
+      </c>
+      <c r="L241" t="str">
+        <v>Forsker uenig med Musk: Indsamling af beskidte bleer er en god idé</v>
+      </c>
+      <c r="M241" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N241" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O241" t="str">
+        <v>https://ing.dk/#:~:text=bleer</v>
+      </c>
+      <c r="P241" t="str">
+        <v/>
+      </c>
+      <c r="Q241" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R241" t="str">
+        <v/>
+      </c>
+      <c r="S241" t="str">
+        <v/>
+      </c>
+      <c r="T241" t="str">
+        <v/>
+      </c>
+      <c r="U241" t="str">
+        <v/>
+      </c>
+      <c r="V241" t="str">
+        <v/>
+      </c>
+      <c r="W241" t="str">
+        <v/>
+      </c>
+      <c r="X241" t="str">
+        <v/>
+      </c>
+      <c r="Y241" t="str">
+        <v/>
+      </c>
+      <c r="Z241" t="str">
+        <v/>
+      </c>
+      <c r="AA241" t="str">
+        <v/>
+      </c>
+      <c r="AB241" t="str">
+        <v/>
+      </c>
+      <c r="AC241" t="str">
+        <v/>
+      </c>
+      <c r="AD241" t="str">
+        <v/>
+      </c>
+      <c r="AE241" t="str">
+        <v/>
+      </c>
+      <c r="AF241" t="str">
+        <v/>
+      </c>
+      <c r="AG241" t="str">
+        <v/>
+      </c>
+      <c r="AH241" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH240"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH241"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kortlagt" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH241"/>
+  <dimension ref="A1:AH242"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24333,9 +24333,113 @@
         <v/>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>55ef2464-3b97-4ebd-852d-6eada5c06335</v>
+      </c>
+      <c r="B242" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="C242" t="str">
+        <v>kortlagt</v>
+      </c>
+      <c r="D242" t="str">
+        <v>kortlægge</v>
+      </c>
+      <c r="E242" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F242" t="str">
+        <v/>
+      </c>
+      <c r="G242" t="str">
+        <v>-r, ..lagde, ..lagt</v>
+      </c>
+      <c r="H242" t="str">
+        <v/>
+      </c>
+      <c r="I242" t="str">
+        <v>https://static.ordnet.dk/mp3/11027/11027777_1.mp3</v>
+      </c>
+      <c r="J242" t="str">
+        <v>etablere et kort over et geografisk (eller astronomisk) område</v>
+      </c>
+      <c r="K242" t="str">
+        <v>mapped</v>
+      </c>
+      <c r="L242" t="str">
+        <v>Lækkede data afslører: Novo har kortlagt danske læger i hemmeligt kartotek</v>
+      </c>
+      <c r="M242" t="str">
+        <v>Lækkede data afslører: Novo har kortlagt danske læger i hemmeligt kartotek | Ingeniøren</v>
+      </c>
+      <c r="N242" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek</v>
+      </c>
+      <c r="O242" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek#:~:text=kortlagt</v>
+      </c>
+      <c r="P242" t="str">
+        <v/>
+      </c>
+      <c r="Q242" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R242" t="str">
+        <v/>
+      </c>
+      <c r="S242" t="str">
+        <v/>
+      </c>
+      <c r="T242" t="str">
+        <v/>
+      </c>
+      <c r="U242" t="str">
+        <v/>
+      </c>
+      <c r="V242" t="str">
+        <v/>
+      </c>
+      <c r="W242" t="str">
+        <v/>
+      </c>
+      <c r="X242" t="str">
+        <v/>
+      </c>
+      <c r="Y242" t="str">
+        <v/>
+      </c>
+      <c r="Z242" t="str">
+        <v/>
+      </c>
+      <c r="AA242" t="str">
+        <v/>
+      </c>
+      <c r="AB242" t="str">
+        <v/>
+      </c>
+      <c r="AC242" t="str">
+        <v/>
+      </c>
+      <c r="AD242" t="str">
+        <v/>
+      </c>
+      <c r="AE242" t="str">
+        <v/>
+      </c>
+      <c r="AF242" t="str">
+        <v/>
+      </c>
+      <c r="AG242" t="str">
+        <v/>
+      </c>
+      <c r="AH242" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH241"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH242"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "afslører" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH242"/>
+  <dimension ref="A1:AH243"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24437,9 +24437,113 @@
         <v/>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>92a1f319-bcf3-4dea-ae37-a447a0a038ad</v>
+      </c>
+      <c r="B243" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="C243" t="str">
+        <v>afslører</v>
+      </c>
+      <c r="D243" t="str">
+        <v>afsløre</v>
+      </c>
+      <c r="E243" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F243" t="str">
+        <v/>
+      </c>
+      <c r="G243" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H243" t="str">
+        <v>[-ˌsløˀʌ]</v>
+      </c>
+      <c r="I243" t="str">
+        <v>https://static.ordnet.dk/mp3/11000/11000720_1.mp3</v>
+      </c>
+      <c r="J243" t="str">
+        <v>opdage at nogen har begået en (kriminel eller uhæderlig) handling eller har en egenskab eller fortid som vedkommende har forsøgt at skjule</v>
+      </c>
+      <c r="K243" t="str">
+        <v>reveals</v>
+      </c>
+      <c r="L243" t="str">
+        <v>Lækkede data afslører: Novo har kortlagt danske læger i hemmeligt kartotek</v>
+      </c>
+      <c r="M243" t="str">
+        <v>Lækkede data afslører: Novo har kortlagt danske læger i hemmeligt kartotek | Ingeniøren</v>
+      </c>
+      <c r="N243" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek</v>
+      </c>
+      <c r="O243" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek#:~:text=afsl%C3%B8rer</v>
+      </c>
+      <c r="P243" t="str">
+        <v/>
+      </c>
+      <c r="Q243" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R243" t="str">
+        <v/>
+      </c>
+      <c r="S243" t="str">
+        <v/>
+      </c>
+      <c r="T243" t="str">
+        <v/>
+      </c>
+      <c r="U243" t="str">
+        <v/>
+      </c>
+      <c r="V243" t="str">
+        <v/>
+      </c>
+      <c r="W243" t="str">
+        <v/>
+      </c>
+      <c r="X243" t="str">
+        <v/>
+      </c>
+      <c r="Y243" t="str">
+        <v/>
+      </c>
+      <c r="Z243" t="str">
+        <v/>
+      </c>
+      <c r="AA243" t="str">
+        <v/>
+      </c>
+      <c r="AB243" t="str">
+        <v/>
+      </c>
+      <c r="AC243" t="str">
+        <v/>
+      </c>
+      <c r="AD243" t="str">
+        <v/>
+      </c>
+      <c r="AE243" t="str">
+        <v/>
+      </c>
+      <c r="AF243" t="str">
+        <v/>
+      </c>
+      <c r="AG243" t="str">
+        <v/>
+      </c>
+      <c r="AH243" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH242"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH243"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "hemmeligt" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH243"/>
+  <dimension ref="A1:AH244"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24541,9 +24541,113 @@
         <v/>
       </c>
     </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>8eadfac5-7cc5-4834-874b-5a38c6848806</v>
+      </c>
+      <c r="B244" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="C244" t="str">
+        <v>hemmeligt</v>
+      </c>
+      <c r="D244" t="str">
+        <v>hemmelig</v>
+      </c>
+      <c r="E244" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F244" t="str">
+        <v/>
+      </c>
+      <c r="G244" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H244" t="str">
+        <v>[ˈhεməli]</v>
+      </c>
+      <c r="I244" t="str">
+        <v>https://static.ordnet.dk/mp3/11020/11020389_1.mp3</v>
+      </c>
+      <c r="J244" t="str">
+        <v>som er skjult for alle uindviede; som kun en begrænset inderkreds eller nogle få fortrolige kender til eller må kende til</v>
+      </c>
+      <c r="K244" t="str">
+        <v>secretly</v>
+      </c>
+      <c r="L244" t="str">
+        <v>Lækkede data afslører: Novo har kortlagt danske læger i hemmeligt kartotek</v>
+      </c>
+      <c r="M244" t="str">
+        <v>Lækkede data afslører: Novo har kortlagt danske læger i hemmeligt kartotek | Ingeniøren</v>
+      </c>
+      <c r="N244" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek</v>
+      </c>
+      <c r="O244" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek#:~:text=hemmeligt</v>
+      </c>
+      <c r="P244" t="str">
+        <v/>
+      </c>
+      <c r="Q244" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R244" t="str">
+        <v/>
+      </c>
+      <c r="S244" t="str">
+        <v/>
+      </c>
+      <c r="T244" t="str">
+        <v/>
+      </c>
+      <c r="U244" t="str">
+        <v/>
+      </c>
+      <c r="V244" t="str">
+        <v/>
+      </c>
+      <c r="W244" t="str">
+        <v/>
+      </c>
+      <c r="X244" t="str">
+        <v/>
+      </c>
+      <c r="Y244" t="str">
+        <v/>
+      </c>
+      <c r="Z244" t="str">
+        <v/>
+      </c>
+      <c r="AA244" t="str">
+        <v/>
+      </c>
+      <c r="AB244" t="str">
+        <v/>
+      </c>
+      <c r="AC244" t="str">
+        <v/>
+      </c>
+      <c r="AD244" t="str">
+        <v/>
+      </c>
+      <c r="AE244" t="str">
+        <v/>
+      </c>
+      <c r="AF244" t="str">
+        <v/>
+      </c>
+      <c r="AG244" t="str">
+        <v/>
+      </c>
+      <c r="AH244" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH243"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH244"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kartotek" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH244"/>
+  <dimension ref="A1:AH245"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24645,9 +24645,113 @@
         <v/>
       </c>
     </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>6ebbcd1d-e189-4e49-bcf0-1750688d3f16</v>
+      </c>
+      <c r="B245" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="C245" t="str">
+        <v>kartotek</v>
+      </c>
+      <c r="D245" t="str">
+        <v>kartotek</v>
+      </c>
+      <c r="E245" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F245" t="str">
+        <v>et</v>
+      </c>
+      <c r="G245" t="str">
+        <v>-et, -er, -erne</v>
+      </c>
+      <c r="H245" t="str">
+        <v>[kɑdoˈteˀg]</v>
+      </c>
+      <c r="I245" t="str">
+        <v>https://static.ordnet.dk/mp3/11025/11025545_1.mp3</v>
+      </c>
+      <c r="J245" t="str">
+        <v>samling af kort som indeholder ensartede oplysninger om personer, genstande eller sager, og som er ordnet i alfabetisk eller systematisk rækkefølge så man hurtigt kan finde en oplysning</v>
+      </c>
+      <c r="K245" t="str">
+        <v>file</v>
+      </c>
+      <c r="L245" t="str">
+        <v>Lækkede data afslører: Novo har kortlagt danske læger i hemmeligt kartotek</v>
+      </c>
+      <c r="M245" t="str">
+        <v>Lækkede data afslører: Novo har kortlagt danske læger i hemmeligt kartotek | Ingeniøren</v>
+      </c>
+      <c r="N245" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek</v>
+      </c>
+      <c r="O245" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek#:~:text=kartotek</v>
+      </c>
+      <c r="P245" t="str">
+        <v/>
+      </c>
+      <c r="Q245" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R245" t="str">
+        <v/>
+      </c>
+      <c r="S245" t="str">
+        <v/>
+      </c>
+      <c r="T245" t="str">
+        <v/>
+      </c>
+      <c r="U245" t="str">
+        <v/>
+      </c>
+      <c r="V245" t="str">
+        <v/>
+      </c>
+      <c r="W245" t="str">
+        <v/>
+      </c>
+      <c r="X245" t="str">
+        <v/>
+      </c>
+      <c r="Y245" t="str">
+        <v/>
+      </c>
+      <c r="Z245" t="str">
+        <v/>
+      </c>
+      <c r="AA245" t="str">
+        <v/>
+      </c>
+      <c r="AB245" t="str">
+        <v/>
+      </c>
+      <c r="AC245" t="str">
+        <v/>
+      </c>
+      <c r="AD245" t="str">
+        <v/>
+      </c>
+      <c r="AE245" t="str">
+        <v/>
+      </c>
+      <c r="AF245" t="str">
+        <v/>
+      </c>
+      <c r="AG245" t="str">
+        <v/>
+      </c>
+      <c r="AH245" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH244"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH245"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "rangerer" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH245"/>
+  <dimension ref="A1:AH246"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24749,9 +24749,113 @@
         <v/>
       </c>
     </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>136c2d0e-dfca-4532-9414-a206ef932b69</v>
+      </c>
+      <c r="B246" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="C246" t="str">
+        <v>rangerer</v>
+      </c>
+      <c r="D246" t="str">
+        <v>rangere</v>
+      </c>
+      <c r="E246" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F246" t="str">
+        <v/>
+      </c>
+      <c r="G246" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H246" t="str">
+        <v>[ʁɑŋˈɕeˀʌ]</v>
+      </c>
+      <c r="I246" t="str">
+        <v>https://static.ordnet.dk/mp3/11042/11042127_1.mp3</v>
+      </c>
+      <c r="J246" t="str">
+        <v>have en bestemt status eller plads i en rangorden</v>
+      </c>
+      <c r="K246" t="str">
+        <v>ranks</v>
+      </c>
+      <c r="L246" t="str">
+        <v>Et datalæk viser, hvordan Novo fører et internt system på 46.000 sundhedspersoner, hvor de rangerer læger og sygeplejersker ud fra deres kommercielle værdi og loyalitet over for præparater som Ozempic og Wegovy.</v>
+      </c>
+      <c r="M246" t="str">
+        <v>Lækkede data afslører: Novo har kortlagt danske læger i hemmeligt kartotek | Ingeniøren</v>
+      </c>
+      <c r="N246" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek</v>
+      </c>
+      <c r="O246" t="str">
+        <v>https://ing.dk/artikel/laekkede-data-afsloerer-novo-har-kortlagt-danske-laeger-i-hemmeligt-kartotek#:~:text=rangerer</v>
+      </c>
+      <c r="P246" t="str">
+        <v/>
+      </c>
+      <c r="Q246" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R246" t="str">
+        <v/>
+      </c>
+      <c r="S246" t="str">
+        <v/>
+      </c>
+      <c r="T246" t="str">
+        <v/>
+      </c>
+      <c r="U246" t="str">
+        <v/>
+      </c>
+      <c r="V246" t="str">
+        <v/>
+      </c>
+      <c r="W246" t="str">
+        <v/>
+      </c>
+      <c r="X246" t="str">
+        <v/>
+      </c>
+      <c r="Y246" t="str">
+        <v/>
+      </c>
+      <c r="Z246" t="str">
+        <v/>
+      </c>
+      <c r="AA246" t="str">
+        <v/>
+      </c>
+      <c r="AB246" t="str">
+        <v/>
+      </c>
+      <c r="AC246" t="str">
+        <v/>
+      </c>
+      <c r="AD246" t="str">
+        <v/>
+      </c>
+      <c r="AE246" t="str">
+        <v/>
+      </c>
+      <c r="AF246" t="str">
+        <v/>
+      </c>
+      <c r="AG246" t="str">
+        <v/>
+      </c>
+      <c r="AH246" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH245"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH246"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Fjenden" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH246"/>
+  <dimension ref="A1:AH247"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24853,9 +24853,113 @@
         <v/>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>cea6e27d-07a2-4126-a714-f1656ab60cb9</v>
+      </c>
+      <c r="B247" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="C247" t="str">
+        <v>Fjenden</v>
+      </c>
+      <c r="D247" t="str">
+        <v>fjende</v>
+      </c>
+      <c r="E247" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F247" t="str">
+        <v>en</v>
+      </c>
+      <c r="G247" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H247" t="str">
+        <v>[ˈfjenə]</v>
+      </c>
+      <c r="I247" t="str">
+        <v>https://static.ordnet.dk/mp3/11013/11013323_1.mp3</v>
+      </c>
+      <c r="J247" t="str">
+        <v>person som aktivt søger at modarbejde, skade eller tilintetgøre en anden part</v>
+      </c>
+      <c r="K247" t="str">
+        <v>The enemy</v>
+      </c>
+      <c r="L247" t="str">
+        <v>Danmarks nye missiler kan nå dybt ind i Rusland: »Fjenden må ikke kunne skyde længere, end vi kan«</v>
+      </c>
+      <c r="M247" t="str">
+        <v>Danmarks nye missiler kan ramme dybt i Rusland - yihengldavid@gmail.com - Gmail</v>
+      </c>
+      <c r="N247" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+      </c>
+      <c r="O247" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=Fjenden</v>
+      </c>
+      <c r="P247" t="str">
+        <v/>
+      </c>
+      <c r="Q247" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R247" t="str">
+        <v/>
+      </c>
+      <c r="S247" t="str">
+        <v/>
+      </c>
+      <c r="T247" t="str">
+        <v/>
+      </c>
+      <c r="U247" t="str">
+        <v/>
+      </c>
+      <c r="V247" t="str">
+        <v/>
+      </c>
+      <c r="W247" t="str">
+        <v/>
+      </c>
+      <c r="X247" t="str">
+        <v/>
+      </c>
+      <c r="Y247" t="str">
+        <v/>
+      </c>
+      <c r="Z247" t="str">
+        <v/>
+      </c>
+      <c r="AA247" t="str">
+        <v/>
+      </c>
+      <c r="AB247" t="str">
+        <v/>
+      </c>
+      <c r="AC247" t="str">
+        <v/>
+      </c>
+      <c r="AD247" t="str">
+        <v/>
+      </c>
+      <c r="AE247" t="str">
+        <v/>
+      </c>
+      <c r="AF247" t="str">
+        <v/>
+      </c>
+      <c r="AG247" t="str">
+        <v/>
+      </c>
+      <c r="AH247" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH246"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH247"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "beskylder" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH247"/>
+  <dimension ref="A1:AH248"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24957,9 +24957,113 @@
         <v/>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>a19b1021-820d-40de-8cbc-f26832b73df4</v>
+      </c>
+      <c r="B248" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="C248" t="str">
+        <v>beskylder</v>
+      </c>
+      <c r="D248" t="str">
+        <v>beskylde</v>
+      </c>
+      <c r="E248" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F248" t="str">
+        <v/>
+      </c>
+      <c r="G248" t="str">
+        <v>-r, beskyldte, beskyldt</v>
+      </c>
+      <c r="H248" t="str">
+        <v>[beˈsgylˀə]</v>
+      </c>
+      <c r="I248" t="str">
+        <v>https://static.ordnet.dk/mp3/11004/11004237_1.mp3</v>
+      </c>
+      <c r="J248" t="str">
+        <v>påstå at nogen er skyldig i noget som man finder meget forkert</v>
+      </c>
+      <c r="K248" t="str">
+        <v>accusing</v>
+      </c>
+      <c r="L248" t="str">
+        <v>Donald Trump og Elon Musk beskylder hinanden for at stå bag den manglende satellitdækning til de kæmpende ukrainere, mens missilerne regner ned over landets største byer. Det har ikke uden grund rejst en del bekymring, at en lunefuld techmilliardær kan påvirke og måske afgøre væbnede konflikter efter for godt befindende.</v>
+      </c>
+      <c r="M248" t="str">
+        <v>Starlink tænder og slukker: Rumkrigen er startet, og en enkelt programmør kan afgøre den | Ingeniøren</v>
+      </c>
+      <c r="N248" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den</v>
+      </c>
+      <c r="O248" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den#:~:text=beskylder</v>
+      </c>
+      <c r="P248" t="str">
+        <v/>
+      </c>
+      <c r="Q248" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R248" t="str">
+        <v/>
+      </c>
+      <c r="S248" t="str">
+        <v/>
+      </c>
+      <c r="T248" t="str">
+        <v/>
+      </c>
+      <c r="U248" t="str">
+        <v/>
+      </c>
+      <c r="V248" t="str">
+        <v/>
+      </c>
+      <c r="W248" t="str">
+        <v/>
+      </c>
+      <c r="X248" t="str">
+        <v/>
+      </c>
+      <c r="Y248" t="str">
+        <v/>
+      </c>
+      <c r="Z248" t="str">
+        <v/>
+      </c>
+      <c r="AA248" t="str">
+        <v/>
+      </c>
+      <c r="AB248" t="str">
+        <v/>
+      </c>
+      <c r="AC248" t="str">
+        <v/>
+      </c>
+      <c r="AD248" t="str">
+        <v/>
+      </c>
+      <c r="AE248" t="str">
+        <v/>
+      </c>
+      <c r="AF248" t="str">
+        <v/>
+      </c>
+      <c r="AG248" t="str">
+        <v/>
+      </c>
+      <c r="AH248" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH247"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH248"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "manglende" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH248"/>
+  <dimension ref="A1:AH249"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -25061,9 +25061,113 @@
         <v/>
       </c>
     </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>753e84f7-9184-4bbe-949d-63580e1a492f</v>
+      </c>
+      <c r="B249" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="C249" t="str">
+        <v>manglende</v>
+      </c>
+      <c r="D249" t="str">
+        <v>mangle</v>
+      </c>
+      <c r="E249" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F249" t="str">
+        <v/>
+      </c>
+      <c r="G249" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H249" t="str">
+        <v>[ˈmɑŋlə]</v>
+      </c>
+      <c r="I249" t="str">
+        <v>https://static.ordnet.dk/mp3/11032/11032360_1.mp3</v>
+      </c>
+      <c r="J249" t="str">
+        <v>have behov for</v>
+      </c>
+      <c r="K249" t="str">
+        <v>missing</v>
+      </c>
+      <c r="L249" t="str">
+        <v>Donald Trump og Elon Musk beskylder hinanden for at stå bag den manglende satellitdækning til de kæmpende ukrainere, mens missilerne regner ned over landets største byer. Det har ikke uden grund rejst en del bekymring, at en lunefuld techmilliardær kan påvirke og måske afgøre væbnede konflikter efter for godt befindende.</v>
+      </c>
+      <c r="M249" t="str">
+        <v>Starlink tænder og slukker: Rumkrigen er startet, og en enkelt programmør kan afgøre den | Ingeniøren</v>
+      </c>
+      <c r="N249" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den</v>
+      </c>
+      <c r="O249" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den#:~:text=manglende</v>
+      </c>
+      <c r="P249" t="str">
+        <v/>
+      </c>
+      <c r="Q249" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R249" t="str">
+        <v/>
+      </c>
+      <c r="S249" t="str">
+        <v/>
+      </c>
+      <c r="T249" t="str">
+        <v/>
+      </c>
+      <c r="U249" t="str">
+        <v/>
+      </c>
+      <c r="V249" t="str">
+        <v/>
+      </c>
+      <c r="W249" t="str">
+        <v/>
+      </c>
+      <c r="X249" t="str">
+        <v/>
+      </c>
+      <c r="Y249" t="str">
+        <v/>
+      </c>
+      <c r="Z249" t="str">
+        <v/>
+      </c>
+      <c r="AA249" t="str">
+        <v/>
+      </c>
+      <c r="AB249" t="str">
+        <v/>
+      </c>
+      <c r="AC249" t="str">
+        <v/>
+      </c>
+      <c r="AD249" t="str">
+        <v/>
+      </c>
+      <c r="AE249" t="str">
+        <v/>
+      </c>
+      <c r="AF249" t="str">
+        <v/>
+      </c>
+      <c r="AG249" t="str">
+        <v/>
+      </c>
+      <c r="AH249" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH248"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH249"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "satellitdækning" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH249"/>
+  <dimension ref="A1:AH250"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -25165,9 +25165,113 @@
         <v/>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>a7a7d802-4350-4e6c-a73e-a5f776980a06</v>
+      </c>
+      <c r="B250" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="C250" t="str">
+        <v>satellitdækning</v>
+      </c>
+      <c r="D250" t="str">
+        <v>satellitdækning</v>
+      </c>
+      <c r="E250" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F250" t="str">
+        <v>en</v>
+      </c>
+      <c r="G250" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H250" t="str">
+        <v/>
+      </c>
+      <c r="I250" t="str">
+        <v/>
+      </c>
+      <c r="J250" t="str">
+        <v>sammensat af satellit + dækning</v>
+      </c>
+      <c r="K250" t="str">
+        <v>Satellite coverage</v>
+      </c>
+      <c r="L250" t="str">
+        <v>Donald Trump og Elon Musk beskylder hinanden for at stå bag den manglende satellitdækning til de kæmpende ukrainere, mens missilerne regner ned over landets største byer. Det har ikke uden grund rejst en del bekymring, at en lunefuld techmilliardær kan påvirke og måske afgøre væbnede konflikter efter for godt befindende.</v>
+      </c>
+      <c r="M250" t="str">
+        <v>Starlink tænder og slukker: Rumkrigen er startet, og en enkelt programmør kan afgøre den | Ingeniøren</v>
+      </c>
+      <c r="N250" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den</v>
+      </c>
+      <c r="O250" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den#:~:text=satellitd%C3%A6kning</v>
+      </c>
+      <c r="P250" t="str">
+        <v/>
+      </c>
+      <c r="Q250" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R250" t="str">
+        <v/>
+      </c>
+      <c r="S250" t="str">
+        <v/>
+      </c>
+      <c r="T250" t="str">
+        <v/>
+      </c>
+      <c r="U250" t="str">
+        <v/>
+      </c>
+      <c r="V250" t="str">
+        <v/>
+      </c>
+      <c r="W250" t="str">
+        <v/>
+      </c>
+      <c r="X250" t="str">
+        <v/>
+      </c>
+      <c r="Y250" t="str">
+        <v/>
+      </c>
+      <c r="Z250" t="str">
+        <v/>
+      </c>
+      <c r="AA250" t="str">
+        <v/>
+      </c>
+      <c r="AB250" t="str">
+        <v/>
+      </c>
+      <c r="AC250" t="str">
+        <v/>
+      </c>
+      <c r="AD250" t="str">
+        <v/>
+      </c>
+      <c r="AE250" t="str">
+        <v/>
+      </c>
+      <c r="AF250" t="str">
+        <v/>
+      </c>
+      <c r="AG250" t="str">
+        <v/>
+      </c>
+      <c r="AH250" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH249"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH250"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kæmpende" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH250"/>
+  <dimension ref="A1:AH251"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -25269,9 +25269,113 @@
         <v/>
       </c>
     </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>18654082-66fd-43cf-8137-c43031e93336</v>
+      </c>
+      <c r="B251" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="C251" t="str">
+        <v>kæmpende</v>
+      </c>
+      <c r="D251" t="str">
+        <v>kæmpe</v>
+      </c>
+      <c r="E251" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F251" t="str">
+        <v/>
+      </c>
+      <c r="G251" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H251" t="str">
+        <v>[ˈkεmbə]</v>
+      </c>
+      <c r="I251" t="str">
+        <v>https://static.ordnet.dk/mp3/11029/11029071_1.mp3</v>
+      </c>
+      <c r="J251" t="str">
+        <v>tage del i en voldelig konflikt; føre krig</v>
+      </c>
+      <c r="K251" t="str">
+        <v>Fighting</v>
+      </c>
+      <c r="L251" t="str">
+        <v>Donald Trump og Elon Musk beskylder hinanden for at stå bag den manglende satellitdækning til de kæmpende ukrainere, mens missilerne regner ned over landets største byer. Det har ikke uden grund rejst en del bekymring, at en lunefuld techmilliardær kan påvirke og måske afgøre væbnede konflikter efter for godt befindende.</v>
+      </c>
+      <c r="M251" t="str">
+        <v>Starlink tænder og slukker: Rumkrigen er startet, og en enkelt programmør kan afgøre den | Ingeniøren</v>
+      </c>
+      <c r="N251" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den</v>
+      </c>
+      <c r="O251" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den#:~:text=k%C3%A6mpende</v>
+      </c>
+      <c r="P251" t="str">
+        <v/>
+      </c>
+      <c r="Q251" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R251" t="str">
+        <v/>
+      </c>
+      <c r="S251" t="str">
+        <v/>
+      </c>
+      <c r="T251" t="str">
+        <v/>
+      </c>
+      <c r="U251" t="str">
+        <v/>
+      </c>
+      <c r="V251" t="str">
+        <v/>
+      </c>
+      <c r="W251" t="str">
+        <v/>
+      </c>
+      <c r="X251" t="str">
+        <v/>
+      </c>
+      <c r="Y251" t="str">
+        <v/>
+      </c>
+      <c r="Z251" t="str">
+        <v/>
+      </c>
+      <c r="AA251" t="str">
+        <v/>
+      </c>
+      <c r="AB251" t="str">
+        <v/>
+      </c>
+      <c r="AC251" t="str">
+        <v/>
+      </c>
+      <c r="AD251" t="str">
+        <v/>
+      </c>
+      <c r="AE251" t="str">
+        <v/>
+      </c>
+      <c r="AF251" t="str">
+        <v/>
+      </c>
+      <c r="AG251" t="str">
+        <v/>
+      </c>
+      <c r="AH251" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH250"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH251"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "rejst" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH251"/>
+  <dimension ref="A1:AH252"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -25373,9 +25373,113 @@
         <v/>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>180441f9-0b6d-4b6e-a129-614a0745506f</v>
+      </c>
+      <c r="B252" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="C252" t="str">
+        <v>rejst</v>
+      </c>
+      <c r="D252" t="str">
+        <v>rejse</v>
+      </c>
+      <c r="E252" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F252" t="str">
+        <v/>
+      </c>
+      <c r="G252" t="str">
+        <v>-r, rejste, rejst</v>
+      </c>
+      <c r="H252" t="str">
+        <v>[ˈʁɑjsə]</v>
+      </c>
+      <c r="I252" t="str">
+        <v>https://static.ordnet.dk/mp3/11042/11042622_1.mp3</v>
+      </c>
+      <c r="J252" t="str">
+        <v>få noget til at stå i opret, lodret stilling (i overensstemmelse med dets funktion)</v>
+      </c>
+      <c r="K252" t="str">
+        <v>Traveled</v>
+      </c>
+      <c r="L252" t="str">
+        <v>Donald Trump og Elon Musk beskylder hinanden for at stå bag den manglende satellitdækning til de kæmpende ukrainere, mens missilerne regner ned over landets største byer. Det har ikke uden grund rejst en del bekymring, at en lunefuld techmilliardær kan påvirke og måske afgøre væbnede konflikter efter for godt befindende.</v>
+      </c>
+      <c r="M252" t="str">
+        <v>Starlink tænder og slukker: Rumkrigen er startet, og en enkelt programmør kan afgøre den | Ingeniøren</v>
+      </c>
+      <c r="N252" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den</v>
+      </c>
+      <c r="O252" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den#:~:text=rejst</v>
+      </c>
+      <c r="P252" t="str">
+        <v/>
+      </c>
+      <c r="Q252" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R252" t="str">
+        <v/>
+      </c>
+      <c r="S252" t="str">
+        <v/>
+      </c>
+      <c r="T252" t="str">
+        <v/>
+      </c>
+      <c r="U252" t="str">
+        <v/>
+      </c>
+      <c r="V252" t="str">
+        <v/>
+      </c>
+      <c r="W252" t="str">
+        <v/>
+      </c>
+      <c r="X252" t="str">
+        <v/>
+      </c>
+      <c r="Y252" t="str">
+        <v/>
+      </c>
+      <c r="Z252" t="str">
+        <v/>
+      </c>
+      <c r="AA252" t="str">
+        <v/>
+      </c>
+      <c r="AB252" t="str">
+        <v/>
+      </c>
+      <c r="AC252" t="str">
+        <v/>
+      </c>
+      <c r="AD252" t="str">
+        <v/>
+      </c>
+      <c r="AE252" t="str">
+        <v/>
+      </c>
+      <c r="AF252" t="str">
+        <v/>
+      </c>
+      <c r="AG252" t="str">
+        <v/>
+      </c>
+      <c r="AH252" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH251"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH252"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bekymring" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH252"/>
+  <dimension ref="A1:AH253"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -25477,9 +25477,113 @@
         <v/>
       </c>
     </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>60bce890-c433-4af7-9bdf-aa22c8a96844</v>
+      </c>
+      <c r="B253" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="C253" t="str">
+        <v>bekymring</v>
+      </c>
+      <c r="D253" t="str">
+        <v>bekymring</v>
+      </c>
+      <c r="E253" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F253" t="str">
+        <v>en</v>
+      </c>
+      <c r="G253" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H253" t="str">
+        <v>[beˈkømˀʁεŋ]</v>
+      </c>
+      <c r="I253" t="str">
+        <v>https://static.ordnet.dk/mp3/11003/11003988_1.mp3</v>
+      </c>
+      <c r="J253" t="str">
+        <v>følelse af uro, nervøsitet eller ængstelse fx over aktuelle eller fremtidige problemer</v>
+      </c>
+      <c r="K253" t="str">
+        <v>concern</v>
+      </c>
+      <c r="L253" t="str">
+        <v>Donald Trump og Elon Musk beskylder hinanden for at stå bag den manglende satellitdækning til de kæmpende ukrainere, mens missilerne regner ned over landets største byer. Det har ikke uden grund rejst en del bekymring, at en lunefuld techmilliardær kan påvirke og måske afgøre væbnede konflikter efter for godt befindende.</v>
+      </c>
+      <c r="M253" t="str">
+        <v>Starlink tænder og slukker: Rumkrigen er startet, og en enkelt programmør kan afgøre den | Ingeniøren</v>
+      </c>
+      <c r="N253" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den</v>
+      </c>
+      <c r="O253" t="str">
+        <v>https://ing.dk/artikel/starlink-taender-og-slukker-rumkrigen-er-startet-og-en-enkelt-programmoer-kan-afgoere-den#:~:text=bekymring</v>
+      </c>
+      <c r="P253" t="str">
+        <v/>
+      </c>
+      <c r="Q253" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R253" t="str">
+        <v/>
+      </c>
+      <c r="S253" t="str">
+        <v/>
+      </c>
+      <c r="T253" t="str">
+        <v/>
+      </c>
+      <c r="U253" t="str">
+        <v/>
+      </c>
+      <c r="V253" t="str">
+        <v/>
+      </c>
+      <c r="W253" t="str">
+        <v/>
+      </c>
+      <c r="X253" t="str">
+        <v/>
+      </c>
+      <c r="Y253" t="str">
+        <v/>
+      </c>
+      <c r="Z253" t="str">
+        <v/>
+      </c>
+      <c r="AA253" t="str">
+        <v/>
+      </c>
+      <c r="AB253" t="str">
+        <v/>
+      </c>
+      <c r="AC253" t="str">
+        <v/>
+      </c>
+      <c r="AD253" t="str">
+        <v/>
+      </c>
+      <c r="AE253" t="str">
+        <v/>
+      </c>
+      <c r="AF253" t="str">
+        <v/>
+      </c>
+      <c r="AG253" t="str">
+        <v/>
+      </c>
+      <c r="AH253" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH252"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH253"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "forældede" to Nyheder.xlsx
</commit_message>
<xml_diff>
--- a/sets/Nyheder.xlsx
+++ b/sets/Nyheder.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH253"/>
+  <dimension ref="A1:AH254"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -25581,9 +25581,113 @@
         <v/>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>39b5e9bf-886f-4a1c-ac28-3f647ab019ad</v>
+      </c>
+      <c r="B254" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="C254" t="str">
+        <v>forældede</v>
+      </c>
+      <c r="D254" t="str">
+        <v>forældet</v>
+      </c>
+      <c r="E254" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F254" t="str">
+        <v/>
+      </c>
+      <c r="G254" t="str">
+        <v>-, forældede</v>
+      </c>
+      <c r="H254" t="str">
+        <v>[fʌˈεlˀəð]</v>
+      </c>
+      <c r="I254" t="str">
+        <v>https://static.ordnet.dk/mp3/11015/11015551_1.mp3</v>
+      </c>
+      <c r="J254" t="str">
+        <v>som ikke (kan) bruges længere; ikke tidssvarende</v>
+      </c>
+      <c r="K254" t="str">
+        <v>outdated</v>
+      </c>
+      <c r="L254" t="str">
+        <v>Voldtægter, kidnapning og landsforræderi forældede i hemmelighed: Her er prisen for politiets it-svigt</v>
+      </c>
+      <c r="M254" t="str">
+        <v>Voldtægter, kidnapning og landsforræderi forældede i hemmelighed: Her er prisen for politiets it-svigt | Ingeniøren</v>
+      </c>
+      <c r="N254" t="str">
+        <v>https://ing.dk/artikel/voldtaegter-kidnapning-og-landsforraederi-foraeldede-i-hemmelighed-her-er-prisen-politiets-it-svigt?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+      </c>
+      <c r="O254" t="str">
+        <v>https://ing.dk/artikel/voldtaegter-kidnapning-og-landsforraederi-foraeldede-i-hemmelighed-her-er-prisen-politiets-it-svigt?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=for%C3%A6ldede</v>
+      </c>
+      <c r="P254" t="str">
+        <v/>
+      </c>
+      <c r="Q254" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R254" t="str">
+        <v/>
+      </c>
+      <c r="S254" t="str">
+        <v/>
+      </c>
+      <c r="T254" t="str">
+        <v/>
+      </c>
+      <c r="U254" t="str">
+        <v/>
+      </c>
+      <c r="V254" t="str">
+        <v/>
+      </c>
+      <c r="W254" t="str">
+        <v/>
+      </c>
+      <c r="X254" t="str">
+        <v/>
+      </c>
+      <c r="Y254" t="str">
+        <v/>
+      </c>
+      <c r="Z254" t="str">
+        <v/>
+      </c>
+      <c r="AA254" t="str">
+        <v/>
+      </c>
+      <c r="AB254" t="str">
+        <v/>
+      </c>
+      <c r="AC254" t="str">
+        <v/>
+      </c>
+      <c r="AD254" t="str">
+        <v/>
+      </c>
+      <c r="AE254" t="str">
+        <v/>
+      </c>
+      <c r="AF254" t="str">
+        <v/>
+      </c>
+      <c r="AG254" t="str">
+        <v/>
+      </c>
+      <c r="AH254" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH253"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH254"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>